<commit_message>
Lamberts: rescrape + sample page
</commit_message>
<xml_diff>
--- a/lamberts-catalog.xlsx
+++ b/lamberts-catalog.xlsx
@@ -701,7 +701,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Για έλεγχο</t>
+          <t xml:space="preserve">Αυτόματο</t>
         </is>
       </c>
     </row>
@@ -4730,12 +4730,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Vegan Vitamin D3 1000iu</t>
+          <t xml:space="preserve">Lamberts Vitamin D3 1000iu Gummies</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 1000iu φυτικής προελεύσεως</t>
+          <t xml:space="preserve">Ζελεδάκια Βιταμίνης D3 των 1000iu</t>
         </is>
       </c>
       <c r="C97">
@@ -4746,7 +4746,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 1000iu φυτικής προελεύσεως</t>
+          <t xml:space="preserve">Ζελεδάκια Βιταμίνης D3 των 1000iu</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/product/vegan-vitamin-d3-1000iu/</t>
+          <t xml:space="preserve">https://lamberts.gr/product/vitamin-d3-1000iu-gummies/</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -4788,12 +4788,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Vegan Vitamin D3 1000iu</t>
+          <t xml:space="preserve">Lamberts Vitamin D3 1000iu Gummies</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 1000iu φυτικής προελεύσεως</t>
+          <t xml:space="preserve">Ζελεδάκια Βιταμίνης D3 των 1000iu</t>
         </is>
       </c>
       <c r="C98">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 1000iu φυτικής προελεύσεως</t>
+          <t xml:space="preserve">Ζελεδάκια Βιταμίνης D3 των 1000iu</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -4824,7 +4824,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/product/vegan-vitamin-d3-1000iu/</t>
+          <t xml:space="preserve">https://lamberts.gr/product/vitamin-d3-1000iu-gummies/</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">

</xml_diff>

<commit_message>
Lamberts: details for all pages + official images
</commit_message>
<xml_diff>
--- a/lamberts-catalog.xlsx
+++ b/lamberts-catalog.xlsx
@@ -403,7 +403,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/biome-balance-everyday-30caps-pharm24-gr-5055148411534.jpg</t>
+          <t xml:space="preserve">lamberts/biome-balance-everyday-5055148411534.png</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/vitamin-b12-1000-g-30tabs-pharm24-gr-5055148411497.jpg</t>
+          <t xml:space="preserve">lamberts/vitamin-b12-1000-g-5055148411497.png</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/chromium-complex-60tabs-pharm24-gr-5055148402020.jpg</t>
+          <t xml:space="preserve">lamberts/chromium-complex-5055148402020.png</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/wp-content/uploads/2025/01/8556-100-hr-LL823-6-1.png</t>
+          <t xml:space="preserve">lamberts/cranberry-complex-5055148403058.png</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/wp-content/uploads/2025/01/8311-60-LL734-4-hr.png</t>
+          <t xml:space="preserve">lamberts/l-glutathione-complex-5055148401566.png</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/magasorb-150mg-180tabs-pharm24-gr-5055148402136.jpg</t>
+          <t xml:space="preserve">lamberts/magasorb-300mg-effervescent-tabs-5055148402136.png</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -2513,7 +2513,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/methyl-b-complex-60tabs-pharm24-gr-5055148410698.jpg</t>
+          <t xml:space="preserve">lamberts/methyl-b-complex-5055148410698.png</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/magasorb-150mg-60tabs-pharm24-gr-5055148410605.jpg</t>
+          <t xml:space="preserve">lamberts/magasorb-300mg-effervescent-tabs-5055148410605.png</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/selenium-200-g-vitamins-a-c-e-100tabs-pharm24-gr-5055148400002.jpg</t>
+          <t xml:space="preserve">lamberts/selenium-200-g-a-c-e-5055148400002.png</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/omega-3-ultra-1300mg-60caps-pharm24-gr-5055148410674.jpg</t>
+          <t xml:space="preserve">lamberts/vegan-omega-3-oil-5055148410674.jpg</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
@@ -4173,7 +4173,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/wp-content/uploads/2025/01/8087-60_-1.png</t>
+          <t xml:space="preserve">lamberts/vitamin-b12-1000-g-5055148401900.png</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">

</xml_diff>

<commit_message>
Lamberts: regenerate overrides/catalog on top of rescrape + official images
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014FFaAMeHCcSLrUaq49VqHm
</commit_message>
<xml_diff>
--- a/lamberts-catalog.xlsx
+++ b/lamberts-catalog.xlsx
@@ -403,7 +403,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/biome-balance-everyday-30caps-pharm24-gr-5055148411534.jpg</t>
+          <t xml:space="preserve">lamberts/biome-balance-everyday-5055148411534.png</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/vitamin-b12-1000-g-30tabs-pharm24-gr-5055148411497.jpg</t>
+          <t xml:space="preserve">lamberts/vitamin-b12-1000-g-5055148411497.png</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/chromium-complex-60tabs-pharm24-gr-5055148402020.jpg</t>
+          <t xml:space="preserve">lamberts/chromium-complex-5055148402020.png</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/wp-content/uploads/2025/01/8556-100-hr-LL823-6-1.png</t>
+          <t xml:space="preserve">lamberts/cranberry-complex-5055148403058.png</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/wp-content/uploads/2025/01/8311-60-LL734-4-hr.png</t>
+          <t xml:space="preserve">lamberts/l-glutathione-complex-5055148401566.png</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/magasorb-150mg-180tabs-pharm24-gr-5055148402136.jpg</t>
+          <t xml:space="preserve">lamberts/magasorb-300mg-effervescent-tabs-5055148402136.png</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -2602,7 +2602,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/methyl-b-complex-60tabs-pharm24-gr-5055148410698.jpg</t>
+          <t xml:space="preserve">lamberts/methyl-b-complex-5055148410698.png</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/magasorb-150mg-60tabs-pharm24-gr-5055148410605.jpg</t>
+          <t xml:space="preserve">lamberts/magasorb-300mg-effervescent-tabs-5055148410605.png</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/selenium-200-g-vitamins-a-c-e-100tabs-pharm24-gr-5055148400002.jpg</t>
+          <t xml:space="preserve">lamberts/selenium-200-g-a-c-e-5055148400002.png</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/omega-3-ultra-1300mg-60caps-pharm24-gr-5055148410674.jpg</t>
+          <t xml:space="preserve">lamberts/vegan-omega-3-oil-5055148410674.jpg</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
@@ -4416,7 +4416,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/wp-content/uploads/2025/01/8087-60_-1.png</t>
+          <t xml:space="preserve">lamberts/vitamin-b12-1000-g-5055148401900.png</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">

</xml_diff>

<commit_message>
Lamberts: details for all pages
</commit_message>
<xml_diff>
--- a/lamberts-catalog.xlsx
+++ b/lamberts-catalog.xlsx
@@ -191,7 +191,50 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Φυσική πηγή 5-HTP (5-υδροξυτρυπτοφάνη)</t>
+          <t xml:space="preserve">Η 5-HTP (συντομογραφία για την 5-υδροξυτρυπτοφάνη), αποτελεί την υδροξυλιωμένη μορφή του αμινοξέως τρυπτοφάνη. Ο οργανισμός παράγει 5-ΗΤΡ από τρυπτοφάνη, η οποία εν συνεχεία μετατρέπεται σε σεροτονίνη. Η σεροτονίνη αποτελεί έναν νευροδιαβιβαστή με ευρύ φάσμα βιολογικών λειτουργιών, που αφορούν στην ρύθμιση της όρεξης, της διάθεσης, του ύπνου, στον έλεγχο των παρορμήσεων και στην μνήμη.
+Η 5-HTP που περιέχεται στο Griffonia Seed Extract της Lamberts® είναι φυσικής προελεύσεως και συγκεκριμένα προέρχεται από τους σπόρους του αφρικανικού φυτού Griffonia simplicifolia. Το εκχύλισμα των σπόρων του φυτού, αποτελεί ένα από τα πιο ευρέως διαδεδομένα συμπληρώματα 5-HTP παγκοσμίως και ιδιαίτερα δημοφιλές μεταξύ των Επαγγελματιών Υγείας των ΗΠΑ.
+Όπως συμβαίνει με όλα τα βότανα που παρασκευάζονται από τη Lamberts®, υπάρχει αυξημένη επαγρύπνηση σχετικά με την επιλογή των πρώτων υλών. Η επιλογή των πρώτων υλών γίνεται πάντοτε με βάση διεθνείς κατευθυντήριες οδηγίες που αφορούν στην καθαρότητα τους και στην απουσία περιβαλλοντικών ρύπων .
+Η συνιστώμενη ημερήσια δόση του Griffonia Seed Extract της Lamberts® παρέχει τα επίπεδα της 5-HTP που χρησιμοποιούνται στις κλινικές μελέτες .
+Όπως όλα τα σκευάσματα της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Σπόροι Griffonia
+(ως 362mg τιτλοδοτημένου εκχυλίσματος (11:1))
+3982mg
+Το οποίο παρέχει
+5-Υδρόξυτρυπτοφάνη (5-HTP)
+100mg
+Συστατικά: Διογκωτικοί Παράγοντες (Ανθρακικό Ασβέστιο), Τιτλοδοτημένο Εκχύλισμα Σπόρων Griffonia (Griffonia simplicifolia), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Στιλβωτικοί Παράγοντες (Υδροξυπροπυλο Μεθυλοκυτταρίνη, Γλυκερόλη).</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1-3 ταμπλέτες ημερησίως μισή ώρα πριν τα γεύματα ή μισή ώρα πριν την βραδινή κατάκλιση. Ξεκινήστε με μία ταμπλέτα και αυξήστε αν είναι αναγκαίο ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Το 5-HTP λαμβάνεται για περιόδους έως 3 μηνών. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες. Σε ορισμένα άτομα μπορεί να προκληθεί ήπια ζάλη. Συνίσταται η αποφυγή χειρισμού βαρέων μηχανημάτων και οδήγησης, έως όταν καθοριστεί με ποιον τρόπο δρα το 5-ΗΤΡ στον καταναλωτή. Συμβουλευτείτε τον ιατρό σας εάν λαμβάνετε αντικαταθλιπτικά.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60tabs</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 124062/17.11.2023 | Κατηγορία lamberts.gr: Ειδικά Διατροφικά Συμπληρώματα › 5-HTP</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -244,7 +287,49 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">L-Καρνιτίνη υψηλής καθαρότητας &amp; ελεύθερης μορφής</t>
+          <t xml:space="preserve">Η καρνιτίνη αποτελεί ένα σημαντικό αμινοξύ το οποίο ανευρίσκεται σε τροφές ζωικής προελεύσεως, ενώ στον οργανισμό μας συντίθεται από την λυσίνη, παρουσία της βιταμίνης C. Ο σημαντικότερος βιολογικός ρόλος της καρνιτίνης είναι η συμμετοχή της στον μεταβολισμό των λιπαρών οξέων και στην παραγωγή ενέργειας.
+Λόγω του σημαντικού ρόλου της καρνιτίνης στην οξείδωση των λιπαρών οξέων και στην παραγωγή κυτταρικής ενέργειας, τα συμπληρώματα L – Carnitine επιλέγονται συχνά από τους αθλητές στα πλαίσια σχεδιασμού προγραμμάτων αθλητικής διατροφής.
+Η ακέτυλο L-καρνιτίνη αποτελεί την ακετυλιωμένη μορφή της L-καρνιτίνης και χαρακτηρίζεται από αυξημένη απορρόφηση και βιοδιαθεσιμότητα. Με αυτή την μορφή έχει διεξαχθεί η πλειονότητα των κλινικών μελετών που αφορούν στην καρνιτίνη.
+Κάθε κάψουλα Acetyl L- Carnitine της Lamberts® παρέχει 500mg ακέτυλο L-καρνιτίνης σε ελεύθερη μορφή , έτοιμη να απορροφηθεί από τον οργανισμό, χωρίς να απαιτείται η διάσπασή της από τα πεπτικά ένζυμα.
+Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Υδροχλωρική Ακέτυλο L-Καρνιτίνη
+610mg
+Η οποία αποδίδει:
+Ακέτυλο L-Καρνιτίνη
+500mg
+Συστατικά: Υδροχλωρική Ακέτυλο L-Καρνιτίνη, Περίβλημα Κάψουλας (Υδρόξυπρόπυλο Μεθυλοκυτταρίνη), Παράγοντες Αντισυσσωμάτωσης (Στεατικό Μαγνήσιο και Διοξείδιο του Πυριτίου).</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60caps</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 13196/06.02.2019 | Κατηγορία lamberts.gr: Αμινοξέα</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -383,7 +468,50 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Καθημερινή προστασία του μικροβιώματος (10δις)</t>
+          <t xml:space="preserve">To Biome Balance Everyday της Lamberts® αποτελεί ένα σκεύασμα χωρίς προσθήκη γάλακτος, που περιέχει 10 δισεκατομμύρια βακτήρια ανά κάψουλα (κατά τη στιγμή της παρασκευής), καθιστώντας το ως ένα από τα υψηλότερης ισχύος σκευάσματα φιλικών βακτηρίων που κυκλοφορούν στο Ηνωμένο Βασίλειο.
+Τα στελέχη φιλικών βακτηρίων που περιλαμβάνονται στο Biome Balance Everyday είναι ο Lactobacillus acidophilus και το Bifidobacterium bifidum.
+Τα στελέχη αυτά έχουν χρησιμοποιηθεί στην πλειονότητα των διεξαχθέντων μελετών που αφορούν στο εντερικό μικροβίωμα.
+Τα βακτήρια που περιέχονται στο Biome Balance Everyday είναι αποξηραμένα σε υψηλές θερμοκρασίες και εσωκλείονται σε εντεροδιαλυτές κάψουλες καθυστερημένης αποδέσμευσης (Delayed Release Capsule). Οι κάψουλες αυτές παρασκευάζονται από ένα οξεάντοχο εντεροδιαλυτό κάλυμμα πολυσακχαρίτη (Polysaccharide matrix) το οποίο διασφαλίζει τη διατήρηση της βιωσιμότητας των βακτηρίων κατά την διέλευσή τους από τον στόμαχο και τον επιτυχή αποικισμό του εντέρου.
+Το Biome Balance Everyday συνιστάται σε καταστάσεις στις οποίες διαταράσσεται η ισορροπία μεταξύ των φιλικών και των παθογόνων βακτηρίων του εντερικού μικροβιώματος και είναι ιδανικό για καθημερινή και χρόνια χρήση.
+Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Bifidobacterium bifidum, Lactobacillus acidophilus
+10 x 109
+(10 δισεκατομύρια) φιλικά βακτήρια*
+*την στιγμή της παρασκευής.
+Συστατικά: Καλλιέργεια Φιλικών Βακτηρίων (αποδίδει Bifidobacterium bifidum &amp; Lactobacillus acidophilus), Περίβλημα Κάψουλας (Υπρομελλόζη &amp; Κόμμι Gellan), Παράγοντας Αντισυσσωμάτωσης (Στεατικό Οξύ).</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Να λαμβάνεται με ένα ποτήρι νερό κατά προτίμηση το πρωί μετά την αφύπνιση, όταν το pH του στομάχου είναι λιγότερο όξινο. Να μην λαμβάνεται με ζεστά ροφήματα, καθώς η ζέστη σκοτώνει τα βακτήρια. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.
+ΜΕΤΑ ΤΟ ΑΝΟΙΓΜΑ ΤΗΣ ΣΥΣΚΕΥΑΣΙΑΣ ΝΑ ΔΙΑΤΗΡΕΙΤΑΙ ΣΤΟ ΨΥΓΕΙΟ</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30 &amp; 60 caps</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 46272/17.04.2025 | Κατηγορία lamberts.gr: Φιλικά Βακτήρια και Πρεβιοτικά</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -441,7 +569,46 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Α-λιποϊκό οξύ υψηλής ισχύος</t>
+          <t xml:space="preserve">Το Alpha Lipoic Acid 300mg της Lamberts® , αποτελεί ένα υψηλής ισχύος , κλινικά ελεγμένο σκεύασμα λιποϊκού οξέος, το οποίο παρέχει 300mg ανά ταμπλέτα. Με αυτό έχει διεξαχθεί διπλή τυφλή τυχαιοποιημένη ,ελεγχόμενη με εικονικό φάρμακο, μελέτη για την αξιολόγηση της επίδρασης χορήγησης αντιοξειδωτικών σε πάσχοντες από ιδιοπαθείς εμβοές (1) .
+Όπως όλα τα σκευάσματα της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+Το α-λιποϊκό οξύ (συχνά αποκαλούμενο ως λιποϊκό οξύ ή ως θειοκτικό οξύ), αποτελεί οργανική ένωση θείου η όποια δομικά μοιάζει με βιταμίνη.
+Οι βιολογικές ιδιότητες του λιποϊκού οξέος προκύπτουν απόρροια της χαρακτηριστικής χημικής του δομής, η οποία του επιτρέπει να δρα ως αντιοξειδωτικό και στο εσωτερικό και στο εξωτερικό του κυττάρου. Το γεγονός αυτό οδήγησε πολλούς συγγραφείς να περιγράφουν το λιποϊκό οξύ, ως το «οικουμενικό αντιοξειδωτικό»
+1. A. Petridou, E. Zagora , P. Petridis , G. Korres, M .Gazouli, I. Xenelis, E. Kyrodimos, G. Kontothanasi , A. Kaliora. The Effect of Antioxidant Supplementation in Patients with Tinnitus and Normal Hearing or Hearing Loss: A randomized, Double-Blind, Placebo Controlled Trial. Nutrients. 2019 Dec 12;11(12).</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Άλφα Λιποϊκό Οξύ (Θιοκτικό οξύ)
+300mg
+Συστατικά: Ανθρακικό Ασβέστιο, Κυτταρίνη, Άλφα Λιποϊκό Οξύ, Παράγοντες Αντισυσσωμάτωσης (Στεατικό Μαγνήσιο, Διοξείδιο του Πυριτίου, Στεατικό Οξύ), Επικάλυψη Ταμπλέτας (Υδροξυπροπυλο Μεθυλοκυτταρίνη, Γλυκερόλη).</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε έως 2 ταμπλέτες ημερησίως με ή χωρίς φαγητό ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Ως αντιοξειδωτικό, λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες. Άτομα που πάσχουν από σακχαρώδη διαβήτη θα πρέπει να συμβουλευτούν τον γιατρό τους πριν τη χρήση του Alpha Lipoic Acid επειδή μπορεί να αυξήσει τη δραστικότητα της ινσουλίνης.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90tabs</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 75609/20.11.2008 | Κατηγορία lamberts.gr: Ειδικά Διατροφικά Συμπληρώματα › Α-Λιποϊκο Οξύ</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -494,7 +661,45 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">100% Ασκορβικό οξύ σε μορφή σκόνης</t>
+          <t xml:space="preserve">Η βιταμίνη C σε μορφή σκόνης της Lamberts® αποτελεί έναν εύκολο τρόπο λήψης υψηλών ποσοτήτων βιταμίνης C, αποτελώντας ταυτοχρόνως μια εναλλακτική λύση για άτομα που δεν μπορούν να καταπιούν μεγάλες ταμπλέτες.
+Το Ascorbic Acid 250 grams αποτελεί σκόνη 100% ασκορβικού οξέος, δηλαδή την κλασσική μορφή της βιταμίνης C. Η σκόνη είναι εξαιρετικά ευδιάλυτη σκόνη και διαθέτει μια αναζωογονητικά έντονη γεύση η οποία προσομοιάζει στην οξεία γεύση των εσπεριδοειδών. Μπορεί να χρησιμοποιηθεί για την ενίσχυση των φρουτοποτών και των φρουτοχυμών.
+Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά 1γρ σκόνης
+Βιταμίνη C
+1000mg
+Συστατικά: Βιταμίνη C (ως Ασκορβικό Οξύ).</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ενήλικες: Λαμβάνετε 1-2 γραμμάρια σκόνης μετά το φαγητό. 1/4 του κουταλιού του γλυκού = 1 γραμμάριο σκόνης
+Παιδιά άνω των 10 ετών: Λαμβάνετε 1/8 του κουταλιού του γλυκού = 500 mg σκόνης μετά το φαγητό. Ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη. Η σκόνη διαλύεται εύκολα σε νερό και χυμό ή μπορεί να προστεθεί αυτούσια σε φαγητό.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Πρόσληψη άνω των 1000mg Βιταμίνης C ημερησίως μπορεί να προκαλέσει ήπιες γαστρεντερικές διαταραχές.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">250gr σκόνη</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 18104/04.03.2013 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη C</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -547,7 +752,54 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής ισχύος τιτλοδοτημένο εκχύλισμα Ασβαγκάντα</t>
+          <t xml:space="preserve">Η Ασβαγκάντα (Withania somnifera), γνωστή και ως «Ινδικό τζίνσενγκ», αποτελεί βότανο που φύεται ως επί το πλείστον στην Ινδία και συνοδεύεται από μακραίωνη ιστορία χρήσης στις χώρες της Άπω Ανατολής.
+Οι σημαντικότερες φυτοχημικά δραστικές ουσίες της Ασβαγκάντα ανευρίσκονται στη ρίζα του βοτάνου και ονομάζονται βιθανολίδες (ή γουαθινολίδες / withanolides) και διαθέτουν προσαρμοσιογόνες ιδιότητες*. Η προσαρμοσιογόνος δράση του βοτάνου βρίσκει εφαρμογή σε καταστάσεις έκθεσης σε χρόνιους στρεσσογόνους παράγοντες (σωματικούς ή πνευματικούς)* και σε καταστάσεις όπου απαιτείται η βέλτιστη νοητική και γνωστική δραστηριότητα*.
+Το Ashwagandha Advance της Lamberts® αποτελεί ένα υψηλής ισχύος τιτλοδοτημένο εκχύλισμα ρίζας Ασβαγκάντας. To σύνολο του βοτάνου που χρησιμοποιείται στην παρασκευή του Ashwagandha Advance, προέρχεται από την ρίζα του βοτάνου, καθώς εκεί ανευρίσκονται αποκλειστικά οι βιθανολίδες. Έτσι κάθε ταμπλέτα παρέχει ένα εγγυημένο ποσό 15mg βιθανολιδών, μια ποσότητα που ισούται αυτής που έχει χρησιμοποιηθεί στην πλειονότητα των κλινικών μελετών.
+Επιπροσθέτως, έχουν προστεθεί βιταμίνη C και ψευδάργυρος, συστατικά τα οποία είναι γνωστό ότι συμβάλλουν στη φυσιολογική λειτουργία του ανοσοποιητικού*.
+Το Ashwagandha Advance, όπως όλα τα σκευάσματα της Lamberts®, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη C
+40mg
+Ψευδάργυρος
+5mg
+Ασβαγκάντα
+ως 300mg (18,9:1) τιτλοδοτημένου εκχυλίσματος
+5671mg
+το οποίο αποδίδει
+Βιθανολίδες
+15mg
+Συστατικά: Τιτλοδοτημένο Εκχύλισμα Ασβαγκάντα (Withania somnifera), Περίβλημα Κάψουλας (Υδρόξυπροπυλο Μεθυλοκυτταρίνη), Βιταμίνη C (Ασκορβικό Οξύ), Παράγοντες Αντισυσσωμάτωσης (Στεατικό Μαγνήσιο &amp; Διοξείδιο του Πυριτίου), Κιτρικός Ψευδάργυρος.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ενήλικες λαμβάνετε 1 κάψουλα ημερησίως ή σύμφωνα με τις οδηγίες του γιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60caps</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 99365/26.08.2025 | Κατηγορία lamberts.gr: Βότανα › Προσαρμοσιογόνα βότανα</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -562,7 +814,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/wp-content/uploads/2025/01/8576-60_NEW-1.png</t>
+          <t xml:space="preserve">lamberts/ashwagandha-advance-5055148412982.png</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -600,7 +852,89 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Αναβράζουσα πολυβιταμίνη για πλήρη κάλυψη</t>
+          <t xml:space="preserve">H Α-Ζ αναβράζον της Lamberts®, αποτελεί μια φόρμουλα της μίας ταμπλέτας ημερησίως η οποία παρέχει το σύνολο των απαραίτητων μικροθρεπτικών συστατικών, πολλά εκ των οποίων στο 100% της Διατροφικής Τιμής Αναφοράς.
+Η Α-Ζ της Lamberts® μπορεί να χρησιμοποιηθεί με 2 τρόπους:
+1. είτε κατά την διάρκεια της εφηβείας (14-18 ετών) ως πολυβιταμίνη μακροχρόνιας χορήγησης,
+2. είτε σε μεγαλύτερες ηλικίες ως φόρμουλα συντήρησης των μικροθρεπτικών συστατικών.
+Παρά το γεγονός ότι η Α-Ζ παρέχει επίπεδα μικροθρεπτικών συστατικών παρόμοια με αντίστοιχες πολυβιταμινούχες φόρμουλες που κυκλοφορούν στην αγορά, έχει σημαντικά μικρότερο κόστος αγοράς. Τα αναβράζοντα δισκία αποτελούν εναλλακτική επιλογή για άτομα που δεν μπορούν να καταπιούν μεγάλες ταμπλέτες και διαθέτουν ευχάριστη γεύση μάνγκο και ανανά.
+Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζονται σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές Πληροφορίες
+Aνά δισκίο
+Βιταμίνη Α
+800µg RE
+Βιταμίνη D (D3)
+5μg
+Βιταμίνη E
+12mg α-TE
+Βιταμίνη Κ
+75μg
+Βιταμίνη C
+80mg
+Θειαμίνη (B1)
+1,1mg
+Ριβοφλαβίνη (B2)
+1,4mg
+Νιασίνη (B3)
+16mg NE
+Βιταμίνη B6
+1,4mg
+Φολικό οξύ
+200μg
+Βιταμίνη B12
+2,5μg
+Βιοτίνη
+50μg
+Παντοθενικό οξύ (B5)
+6mg
+Ασβέστιο
+160mg
+Μαγνήσιο
+75mg
+Σίδηρος
+5mg
+Ψευδάργυρος
+5mg
+Μαγγάνιο
+2mg
+Σελήνιο
+55μg
+Χρώμιο
+40μg
+Μολυβδαίνιο
+50μg
+Ιώδιο
+150μg
+Συστατικά: Κιτρικό Οξύ, Ρυθμιστές Οξύτητας (Διττανθρακικό Νάτριο &amp; Ανθρακικό Νάτριο), Ανθρακικό Ασβέστιο, Ανθρακικό Μαγνήσιο, Υγραντικό (Σορβιτόλη), Ινουλίνη, Βιταμίνη C (Ασκορβικό Οξύ), Ενισχυτικό Γεύσης, Άμυλο, Φωσφορικό Τριασβέστιο, Γλυκαντικός Παράγοντας (Σουκραλόζη), Νιασίνη (Νικοτιναμίδιο), Κιτρικός Ψευδάργυρος, Θειϊκός Σίδηρος, Βιταμίνη Ε (Οξεϊκή dl-alpha Τοκοφερόλη), Παντοθενικό Οξύ (Παντοθενικό Ασβέστιο), Θειϊκό Μαγγάνιο, Βιταμίνη Β6 (Υδροχλωρική Πυριδοξίνη), Ριβοφλαβίνη, Μονονιτρική Θειαμίνη, Οξεϊκή Βιταμίνη Α, Φολικό Οξύ, Ιωδικό Κάλιο, Τριχλωριούχο Χρώμιο, Νατριούχο Σελήνιο, Μολυβδαίνιο, Βιταμίνη Κ1, Βιοτίνη, Βιταμίνη D3, Βιταμίνη Β12 (Κυανοκοβαλαμίνη).</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 δισκίο ημερησίως (διαλυμένο σε ένα ποτήρι νερό) με το γεύμα ή σύμφωνα με τη σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Μπορεί να προκληθεί κίτρινος χρωματισμός των ούρων. Αυτό είναι αβλαβές και υποδεικνύει ότι το σώμα αποβάλλει την περίσσια ποσότητα της βιταμίνης Β2 (riboflavin). Το προϊόν αυτό περιέχει Βιταμίνη Α, να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες ή γυναίκες με πιθανότητα μελλοντικής εγκυμοσύνης. Περιεχει Βιταμίνη Κ, να μην λαμβάνεται από άτομα που βρίσκονται υπό αγωγή με κουμαρινικά αντιπηκτικά, εκτός εάν υπάρχει αντίθετη ιατρική σύσταση. Περιέχει Σίδηρο και η υπέρβαση της δοσολογίας μπορεί να είναι επιζήμια, ιδιαίτερα σε μικρά παιδιά. Να φυλάσσεται σε μέρος και θέση την οποία δεν βλέπουν και δεν προσεγγίζουν παιδιά.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20δισκία</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 93184/2013 | Κατηγορία lamberts.gr: Πολυβιταμίνες › Για εφήβους 14-18 ετών</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -745,7 +1079,46 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής καθαρότητας Βιταμίνη Β12 για την κάλυψη αυξημένων αναγκών</t>
+          <t xml:space="preserve">Η βιταμίνη B12 κατέχει εξέχουσα θέση μεταξύ των βιταμινών, καθώς διαδραματίζει κεντρικό ρόλο σε θεμελιώδεις οργανικές λειτουργίες. Συγκεκριμένα εμπλέκεται στη σύνθεση του DNA και της μυελίνης, παίζοντας ρόλο στη διαδικασία της κυτταρικής διαίρεσης, συμβάλλοντας στο φυσιολογικό σχηματισμό των ερυθρών αιμοσφαιρίων και στη φυσιολογική λειτουργία του νευρικού συστήματος*. Επιπροσθέτως, όπως όλες οι βιταμίνες του συμπλέγματος Β διαθέτει σημαντικές μεταβολικές ιδιότητες, συμβάλλοντας στο φυσιολογικό μεταβολισμό της ομοκυστεΐνης* και στη φυσιολογική λειτουργία των μεταβολικών διεργασιών που αποσκοπούν στην παραγωγή ενέργειας και στη μείωση της κούρασης και της κόπωσης *.
+Η βιταμίνη Β12 ανευρίσκεται σε τροφές ζωικής προελεύσεως, όπως είναι το κόκκινο κρέας. Για το λόγο αυτό, η συμπληρωματική λήψη βιταμίνης Β12 είναι συχνή πρακτική από χορτοφάγους και αυστηρώς χορτοφάγους (vegans). Συχνά συνιστάται και σε ηλικιωμένους, στους οποίους η ανεπάρκεια Β12 είναι συχνό εύρημα λόγω πολυφαρμακίας, πτωχής διατροφής και αχλωρυδρίας.
+Το σκεύασμα Vitamin B12 100μg της Lamberts® παρέχει 100μg βιταμίνης Β12 (ως μεθυλοκοβαλαμίνη) ανά ταμπλέτα, μια ποσότητα που απευθύνεται σε άτομα με αυξημένες ανάγκες σε Β12 (όπως οι χορτοφάγοι, οι αποκλειστικοί χορτοφάγοι και άτομα στο στάδιο της ανάρρωσης).
+Όπως όλα τα σκευάσματα της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+* (ΕΕ) αριθ. 432/2012</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Βιταμίνη B12
+100μg
+Συστατικά: Φωσφορικό Διασβέστιο, Κυτταρίνη, Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Βιταμίνη Β12 (Μέθυλοκοβαλαμίνη).</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100tabs</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 18104/04.03.2013 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνες B</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -894,7 +1267,54 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Μασώμενο Ασβέστιο με D3 και Φρουκτοολιγοσακχαρίτες</t>
+          <t xml:space="preserve">Το Chewable Calcium των 400mg της Lamberts® αποτελεί ένα σκεύασμα μασώμενου ασβεστίου το οποίο παρέχει 400mg στοιχειακού ασβεστίου και 2,5mg βιταμίνης D3 ανά ταμπλέτα.
+Εν αντιθέσει με την συντριπτική πλειοψηφία των εταιρειών, που προσθέτουν σε όλες τις μασώμενες φόρμουλες ζάχαρη ως βελτιωτικό της γεύσης, εμείς χρησιμοποιούμε έναν ειδικό τύπο γλυκαντικών ευδιάλυτων ινών που ονομάζονται φρουκτοολιγοσακχαρίτες (FOS).
+Οι φρουκτοολιγοσακχαρίτες:
+1.Είναι 100% φυσικής προελεύσεως (εκχειλίζονται από τη ρίζα αντιδιού
+2.Δεν προκαλούν τερηδόνα
+3.Δεν αυξάνουν τον γλυκαιμικό δείκτη (Είναι κατάλληλοι για χρήση από διαβητικούς ασθενείς)
+4.Σε προκλινικές μελέτες φαίνεται ότι προάγουν την απορρόφηση του ασβεστίου.
+Οι ταμπλέτες διαθέτουν ευχάριστη γεύση λεμονιού ώστε να διευκολύνεται η λήψη τους, ιδιαιτέρως από παιδιά και όπως όλα τα σκευάσματα της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Βιταμίνη D (D3)
+2,5μg
+Ασβέστιο (ως Ανθρακικό Ασβέστιο)
+400mg
+Φρουκτο-ολιγοσακχαρίτες (FOS)
+1000mg
+Συστατικά: Φρουκτοολιγοσακχαρίτες, Ανθρακικό Ασβέστιο, Παράγοντες Αντισυσσωμάτωσης (Στεατικό Οξύ, Διοξείδιο του Πυριτίου &amp; Στεατικό Μαγνήσιο), Γεύση (Λεμόνι), Γλυκαντική Ουσία (Σουκραλόζη), Βιταμίνη D3 (Χοληκαλσιφερόλη).</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Για παιδιά 4 ετών και άνω: Μασήστε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.
+Για ενήλικες: Μασήστε 1-2 ταμπλέτες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60tabs</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 89129/16.12.2015 | Κατηγορία lamberts.gr: Μέταλλα › Σκευάσματα &amp; Συνδυασμοί Ασβεστίου</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -947,7 +1367,59 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Σύμπλεγμα Χρωμίου ,Βιταμινών και Μετάλλων</t>
+          <t xml:space="preserve">Το Chromium Complex της Lamberts® αποτελεί μια ειδικά σχεδιασμένη φόρμουλα κλινικής διατροφής για την ενίσχυση του μεταβολισμού. Η βάση του συγκεκριμένου σκευάσματος είναι το χρώμιο, το οποίο αποτελεί ένα εκ των σημαντικότερων μεταβολικά ενεργών μικροθρεπτικών συστατικών καθώς συμμετέχοντας στο μονοπάτι σηματοδότησης της ινσουλίνης συμβάλλει στο φυσιολογικό μεταβολισμό των μακροθρεπτικών συστατικών και στη διατήρηση των φυσιολογικών επιπέδων γλυκόζης στο αίμα*.
+To Chromium Complex παρέχει 200µg στοιχειακού χρωμίου ανά ταμπλέτα (ως πικολινικό χρώμιο). Το πικολινικό χρώμιο αποτελεί τη μορφή χρωμίου που έχει χρησιμοποιηθεί στην πλειοψηφία των διεξαχθέντων κλινικών μελετών και η οποία χαρακτηρίζεται από εξαιρετικά υψηλή απορρόφηση και βιοδιαθεσιμότητα.
+Εκτός του χρωμίου, το Chromium Complex της Lamberts® παρέχει ψευδάργυρο, που συμβάλλει στο φυσιολογικό μεταβολισμό των μακροθρεπτικών συστατικών και των λιπαρών οξέων* και βιταμίνες C,B1,B3,B6, μαγνήσιο και χαλκό τα οποία συμβάλλουν στη φυσιολογική λειτουργία των μεταβολικών διεργασιών που αποσκοπούν στην παραγωγή ενέργειας*.
+Όπως όλα τα σκευάσματα της Lamberts® , τo Chromium Complex παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Βιταμίνη C
+100mg
+Θειαμίνη (Β1)
+5mg
+Νιασίνη (Β3)
+5mg NE
+Βιταμίνη Β6
+5mg
+Μαγνήσιο
+300mg
+Ψευδάργυρος
+15mg
+Χαλκός
+0,5mg
+Χρώμιο
+200μg
+Συστατικά: Μαγνήσιο (Υδροξείδιο &amp; Οξείδιο), Βιταμίνη C (Ασκορβικό Οξύ), Διογκωτικοί Παράγοντες (Κυτταρίνη &amp; Υδρόξυπροπυλο Κυτταρίνη), Κιτρικός Ψευδάργυρος, Επικάλυψη Ταμπλέτας (Ανθρακικό Ασβέστιο &amp; Ισομάλτη, Υδρόξυπροπυλο Μεθυλοκυτταρίνη), Παράγοντες Αντισυσσωμάτωσης (Στεατικό Οξύ, Διοξείδιο του Πυριτίου &amp; Στεατικό Μαγνήσιο), Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη), Μονονιτρική Θειαμίνη, Βιταμίνη Β6 (Υδροχλωρική Πυριδοξίνη), Νιασίνη (Νικοτιναμίδιο), Γλυκονικός Χαλκός, Πικολινικό Χρώμιο.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Οι διαβητικοί πρέπει να συμβουλεύονται τον γιατρό τους πριν της χρήσεως του συγκεκριμένου σκευάσματος.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100tabs</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 8571/16.01.2014 | Κατηγορία lamberts.gr: Μέταλλα › Χρώμιο</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1000,7 +1472,58 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Μουρουνέλαιο 5πλης μοριακής απόσταξης</t>
+          <t xml:space="preserve">Το Cod Liver Oil 1000mg της Lamberts® αποτελεί ένα υψηλής ισχύος και καθαρότητας σκεύασμα μουρουνέλαιου με προσθήκη συμπυκνωμένου ιχθυελαίου, για την επίτευξη υψηλότερης συγκέντρωσης σε Ω-3 λιπαρά. Κάθε κάψουλα παρέχει 1000mg μουρουνέλαιου και συμπυκνωμένου ιχθυελαίου, τα οποία παρέχουν 280mg Ω-3 λιπαρών οξέων.
+Επιπροσθέτως παρέχονται ικανοποιητικές ποσότητες βιταμινών A,D και E, οι οποίες συμβάλλουν στη διατήρηση της φυσιολογικής όρασης , στη φυσιολογική λειτουργία του ανοσοποιητικού και στην προστασία των κυττάρων από το οξειδωτικό στρες, αντίστοιχα*.
+Τόσο το μουρουνέλαιο, όσο και το ιχθυέλαιο του Cod Liver Oil της Lamberts® είναι 5πλής μοριακής απόσταξης για την διασφάλιση της μέγιστης καθαρότητας και παρασκευάζονται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+Η προστασία των ελαίων από την οξείδωση εντός της κάψουλας, επιτυγχάνεται χάρη στην προσθήκη φυσικής βιταμίνης Ε.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Μίγμα Μουρουνέλαιου και Συμπυκνωμένου Ιχθυέλαιου σώματος ψαριού
+1000mg
+Ολικά Ω3
+280mg
+Eicosapentaenoic Acid (EPA)
+144mg
+Docosahexaenoic Acid (DHA)
+107mg
+Βιταμίνη Α
+800μg RE
+Βιταμίνη D (D3) (400iu)
+10µg
+Βιταμίνη E
+10mg α-TE
+Συστατικά: Μουρουνέλαιο και Συμπυκνωμένο Ιχθυέλαιο* σώματος ψαριού 5πλής απόσταξης, Περίβλημα Κάψουλας (Βόειος Ζελατίνη &amp; Γλυκερόλη), Βιταμίνη Ε (Οξεϊκή dl-α-Τοκοφερόλη), Παλμιτική Βιταμίνη Α, Βιταμίνη D3 (Χοληκαλσιφερόλη)*.
+*με αντιοξειδωτικό: dl-α-τοκοφερόλη</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Άτομα που λαμβάνουν ασπιρίνη ή από του στόματος αντιπηκτικά πρέπει να συμβουλεύονται τον ιατρό τους, προ της λήψης του Cod Liver Oil 1000mg. Το προϊόν αυτό περιέχει Βιταμίνη Α. Να μην λαμβάνεται από έγκυες ή θηλάζουσες ή γυναίκες που πρόκειται να κυοφορήσουν, εκτός αν συσταθεί από τον Ιατρό τους .
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">180caps</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 24280/11.03.2021 | Κατηγορία lamberts.gr: Ω - Λιπαρά Οξέα › Ω-3 Λιπαρά οξέα από ψάρι</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1053,7 +1576,47 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εξαιρετικά υψηλής ισχύος Συνένζυμο Q10 αυξημένης απορρόφησης</t>
+          <t xml:space="preserve">Το συνένζυμο Q10 αποτελεί ουσία που μοιάζει με βιταμίνη και βρίσκεται στα μιτοχόνδρια του συνόλου των κυττάρων του ανθρώπινου οργανισμού. Εκεί αποτελεί απαραίτητο συστατικό της μιτοχονδριακής αλυσίδας μεταφοράς ηλεκτρονίων (αναπνευστική άλυσος), συμβάλλοντας στην παραγωγή κυτταρικής ενέργειας.
+Καθώς διαδραματίζει σημαντικό ρόλο στην παραγωγή ενέργειας, οι συγκεντρώσεις του συνενζύμου Q10 είναι υψηλότερες σε όργανα με υψηλές ενεργειακές απαιτήσεις (όπως η καρδιά, οι μύες, ο εγκέφαλος, το ήπαρ και οι πνεύμονες). Η αύξηση της ηλικίας και η χρήση φαρμάκων, όπως οι στατίνες μειώνουν την παραγωγή συνενζύμου Q10 από τον οργανισμό.
+Το Co-Enzyme Q10 200mg της Lamberts® παρέχει εγγυημένα 200mg συνενζύμου Q10 ανά κάψουλα.
+Το συνένζυμο ανευρίσκεται σε ελαιώδες εναιώρημα και εσωκλείεται σε εντεροδιαλυτή κάψουλα, καθώς αυτή αποτελεί την φαρμακοτεχνική μορφή με την βέλτιστη απορρόφηση και βιοδιαθεσιμότητα*.
+Όπως όλα τα σκευάσματα της Lamberts® παρασκευάζονται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+* Pepping J. Co Enzyme Q10 Am. Health Syst. Pharm 1999; 56:519-521</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Συνένζυμο Q10 (Ουμπικινόνη)
+200mg
+Συστατικά: Έλαιο ηλιόσπορου, Περίβλημα Κάψουλας (Ζελατίνη, Γλυκερόλη, Χρωστικές : Οξείδιο του Σιδήρου, Συνένζυμο Q10,Λεκιθίνη Ηλίανθου, Μονοστεαρική Γλυκερόλη.</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60caps</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 31869/18.04.2013 | Κατηγορία lamberts.gr: Συνένζυμο Q10 και Ουμπικινόλη</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1111,7 +1674,46 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Συνένζυμο Q10 αυξημένης απορρόφησης</t>
+          <t xml:space="preserve">Το συνένζυμο Q10 αποτελεί ουσία που μοιάζει με βιταμίνη και βρίσκεται στα μιτοχόνδρια του συνόλου των κυττάρων του ανθρώπινου οργανισμού. Εκεί αποτελεί απαραίτητο συστατικό της μιτοχονδριακής αλυσίδας μεταφοράς ηλεκτρονίων (αναπνευστική άλυσος), συμβάλλοντας στην παραγωγή κυτταρικής ενέργειας.
+Καθώς διαδραματίζει σημαντικό ρόλο στην παραγωγή ενέργειας, οι συγκεντρώσεις του συνενζύμου Q10 είναι υψηλότερες σε όργανα με υψηλές ενεργειακές απαιτήσεις (όπως η καρδιά, οι μύες, ο εγκέφαλος, το ήπαρ και οι πνεύμονες). Η αύξηση της ηλικίας και η χρήση φαρμάκων, όπως οι στατίνες μειώνουν την παραγωγή συνενζύμου Q10 από τον οργανισμό.
+Το Co-Enzyme Q10 30mg της Lamberts® παρέχει εγγυημένα 30mg συνενζύμου Q10 ανά κάψουλα, μια συγκέντρωση που καλύπτει τις ανάγκες του μέσου ανθρώπου. Το συνένζυμο ανευρίσκεται σε ελαιώδες εναιώρημα και εσωκλείεται σε εντεροδιαλυτή κάψουλα, καθώς αυτή αποτελεί την φαρμακοτεχνική μορφή με την βέλτιστη απορρόφηση και βιοδιαθεσιμότητα*.
+Όπως όλα τα σκευάσματα της Lamberts® παρασκευάζονται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+* Pepping J. Co Enzyme Q10 Am. Health Syst. Pharm 1999; 56:519-521</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Συνένζυμο Q10 (Ουμπικινόνη)
+30mg
+Συστατικά: Έλαιο Hλιόσπορου, Περίβλημα Κάψουλας (Πηκτωματοποιητές: Τροποποιημένο Άμυλο, Γλυκερόλη &amp; Καραγεννάνη, Χρωστικές: Οξείδιο του Σιδήρου), Συνένζυμο Q10, Μονοστεαρική Γλυκερόλη.</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1-3 κάψουλες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30&amp;60caps</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 25404/11.3.2014 | Κατηγορία lamberts.gr: Συνένζυμο Q10 και Ουμπικινόλη</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1164,7 +1766,50 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής ισχύος εκχύλισμα Κράνμπερι με Βιταμίνη C</t>
+          <t xml:space="preserve">Το Cranberry capsules 18.750mg της Lamberts® αποτελεί ένα από τα υψηλότερης ισχύος σκευάσματα κράνμπερι σε κάψουλες παγκοσμίως. Κάθε κάψουλα αποδίδει 375mg τιτλοδοτημένου εκχυλίσματος καρπών κράνμπερι, ισοδύναμο με 18.750mg φρέσκων καρπών κράνμπερι!
+Επιπροσθέτως , παρέχεται μια σημαντική ποσότητα βιταμίνης C, η οποία συμβάλλει στη φυσιολογική λειτουργία του ανοσοποιητικού *.
+Στην παρασκευή του σκευάσματος ακολουθείται μια εξειδικευμένη διαδικασία που διασφαλίζει την υψηλή ισχύ και την ασφάλεια χρήσης του τελικού προϊόντος: Η πρώτη ύλη περιλαμβάνει φρέσκους ώριμους καρπούς κράνμπερι οι οποίοι, αρχικά καθαρίζονται και απολυμαίνονται για την απομάκρυνση ανεπιθύμητων συστατικών. Εν συνεχεία ο χυμός που παράγεται από την επεξεργασία των καρπών, αποξηραίνεται σε συνθήκες χαμηλής πίεσης και θερμοκρασίας για τη διατήρηση των βιοδραστικών συστατικών και τρέπεται σε σκόνη. Το τελικό στάδιο παραγωγής περιλαμβάνει τον ψεκασμό της σκόνης με ξηρό αέρα οδηγώντας στην παρασκευή του τελικού προϊόντος που δεν περιέχει ζάχαρη.
+Η όλη διαδικασία παρασκευής του σκευάσματος διασφαλίζει την δραστικότητα του τελικού προϊόντος και την δυνατότητα χορήγησης σε άτομα που ακολουθούν δίαιτες με συγκεκριμένους θερμιδικούς περιορισμούς.
+Το Cranberry capsules 18.750mg όπως όλα τα σκευάσματα της Lamberts®, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+Αρ. Πρ. Γνωστ. ΕΟΦ: 112728/27.09.2024</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Bιταμίνη C
+40mg
+Καρποί Cranberry
+ως 375 mg τιτλοδοτημένου εκχυλίσματος (50:1)
+18.750mg
+Συστατικά: Εκχύλισμα Cranberry (Vaccinium Macrocarpon), Περίβλημα Κάψουλας (Υδρόξυπροπυλο Μεθυλοκυτταρίνη), Βιταμίνη C (Ασκορβικό Οξύ), Παράγοντες Αντισυσσωμάτωσης (Στεατικό Μαγνήσιο και Διοξείδιο του Πυριτίου).</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καµία γνωστή για την προτεινόµενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60caps</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατηγορία lamberts.gr: Βότανα › Σκευάσματα Cranberry</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1217,7 +1862,50 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής ισχύος εκχύλισμα Κράνμπερι με Βιταμίνη C</t>
+          <t xml:space="preserve">Το Cranberry capsules 18.750mg της Lamberts® αποτελεί ένα από τα υψηλότερης ισχύος σκευάσματα κράνμπερι σε κάψουλες παγκοσμίως. Κάθε κάψουλα αποδίδει 375mg τιτλοδοτημένου εκχυλίσματος καρπών κράνμπερι, ισοδύναμο με 18.750mg φρέσκων καρπών κράνμπερι!
+Επιπροσθέτως , παρέχεται μια σημαντική ποσότητα βιταμίνης C, η οποία συμβάλλει στη φυσιολογική λειτουργία του ανοσοποιητικού *.
+Στην παρασκευή του σκευάσματος ακολουθείται μια εξειδικευμένη διαδικασία που διασφαλίζει την υψηλή ισχύ και την ασφάλεια χρήσης του τελικού προϊόντος: Η πρώτη ύλη περιλαμβάνει φρέσκους ώριμους καρπούς κράνμπερι οι οποίοι, αρχικά καθαρίζονται και απολυμαίνονται για την απομάκρυνση ανεπιθύμητων συστατικών. Εν συνεχεία ο χυμός που παράγεται από την επεξεργασία των καρπών, αποξηραίνεται σε συνθήκες χαμηλής πίεσης και θερμοκρασίας για τη διατήρηση των βιοδραστικών συστατικών και τρέπεται σε σκόνη. Το τελικό στάδιο παραγωγής περιλαμβάνει τον ψεκασμό της σκόνης με ξηρό αέρα οδηγώντας στην παρασκευή του τελικού προϊόντος που δεν περιέχει ζάχαρη.
+Η όλη διαδικασία παρασκευής του σκευάσματος διασφαλίζει την δραστικότητα του τελικού προϊόντος και την δυνατότητα χορήγησης σε άτομα που ακολουθούν δίαιτες με συγκεκριμένους θερμιδικούς περιορισμούς.
+Το Cranberry capsules 18.750mg όπως όλα τα σκευάσματα της Lamberts®, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+Αρ. Πρ. Γνωστ. ΕΟΦ: 112728/27.09.2024</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Bιταμίνη C
+40mg
+Καρποί Cranberry
+ως 375 mg τιτλοδοτημένου εκχυλίσματος (50:1)
+18.750mg
+Συστατικά: Εκχύλισμα Cranberry (Vaccinium Macrocarpon), Περίβλημα Κάψουλας (Υδρόξυπροπυλο Μεθυλοκυτταρίνη), Βιταμίνη C (Ασκορβικό Οξύ), Παράγοντες Αντισυσσωμάτωσης (Στεατικό Μαγνήσιο και Διοξείδιο του Πυριτίου).</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καµία γνωστή για την προτεινόµενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60caps</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατηγορία lamberts.gr: Βότανα › Σκευάσματα Cranberry</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1270,7 +1958,55 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εκχύλισμα Σκόνης Κράνμπερι με Βιταμίνη C και FOS</t>
+          <t xml:space="preserve">To Cranberry Complex από την Lamberts® είναι μία από τις πιο ισχυρές μορφές κράνμπερι παγκοσμίως. Για την παραγωγή 1 γραμμαρίου συμπυκνωμένης σκόνης, απαιτούνται περίπου 25,101 γραμμάρια φρέσκων κράνμπερι. Επομένως, για κάθε δόση 5 γραμμαρίων σκόνης (που περιέχει 2,47 γραμμάρια κράνμπερι), χρησιμοποιούνται περίπου 2,47 × 25,101 = 62 γραμμάρια φρέσκων κράνμπερι (62.000 mg)!
+Επιπλέον, κάθε 5 γραμμάρια σκόνης παρέχουν σημαντική ποσότητα διαλυτών πρεβιοτικών φρουκτοολιγοσακχαριτών και βιταμίνης C, που συμβάλλουν στη φυσιολογική λειτουργία του ανοσοποιητικού συστήματος*.
+Η διαδικασία παραγωγής αυτής της σύνθεσης ακολουθεί μια εξειδικευμένη μέθοδο που διασφαλίζει την υψηλή ισχύ και την ασφάλεια του τελικού προϊόντος: Το πρώτης ύλης αποτελείται από φρέσκα, ώριμα κράνμπερι που πρώτα καθαρίζονται και απολυμαίνονται για την αφαίρεση ανεπιθύμητων συστατικών. Στη συνέχεια, ο χυμός που λαμβάνεται από την επεξεργασία των μούρων ξηραίνεται υπό χαμηλή πίεση και θερμοκρασία, ώστε να διατηρηθούν οι βιοδραστικές ενώσεις, και μετατρέπεται σε σκόνη.
+Το τελικό στάδιο παραγωγής περιλαμβάνει την ξήρανση της σκόνης με ξηρό αέρα, με αποτέλεσμα ένα τελικό προϊόν χωρίς ζάχαρη.
+Ολόκληρη η διαδικασία παραγωγής διασφαλίζει την ισχύ του τελικού προϊόντος καθώς και την καταλληλότητά του για άτομα που ακολουθούν δίαιτες με συγκεκριμένους περιορισμούς σε θερμίδες.
+Το Cranberry Complex, όπως και όλες οι συνθέσεις της Lamberts®, παράγεται στο Ηνωμένο Βασίλειο σύμφωνα με τα αυστηρά πρότυπα Φαρμακευτικής Ορθής Παρασκευαστικής Πρακτικής (Pharmaceutical GMP).
+*Βάσει του Κανονισμού (ΕΕ) 432/2012 (συμπεριλαμβανομένων ισχυρισμών για βοτανικά / «υπό εξέταση» ισχυρισμός για βοτανική ουσία)
+Αρ. Γνωστοποίησης ΕΟΦ: 22936/12.04.2005
+ΜΕ ΠΡΟΣΘΗΚΗ ΑΠΟΞΗΡΑΝΤΙΚΟΥ ΔΙΣΚΟΥ ΓΕΛΗΣ ΠΥΡΙΤΙΟΥ ΓΙΑ ΤΗΝ ΔΙΑΤΗΡΗΣΗ ΙΔΑΝΙΚΩΝ ΕΠΙΠΕΔΩΝ ΥΓΡΑΣΙΑΣ.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά 5γρ
+Βιταμίνη C
+60mg
+Cranberry
+ως 2470mg τιτλοδοτημένου εκχυλίσματος (19:1)
+47.000mg
+Φρουκτο-ολιγοσακχαρίτες (FOS)
+2186mg
+Συστατικά: Φρουκτο-ολιγοσακχαρίτες (FOS), Σκόνη Συμπυκνωμένου Χυμού Cranberry (Vaccinium macrocarpon L.), Βιταμίνη C (Ασκορβικό Οξύ).</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 5-10 γραμμάρια ημερησίως ή σύμφωνα με τις οδηγίες του γιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε τη συνιστώμενη ημερήσια δόση.5 γραμμάρια σκόνης αντιστοιχούν σε 1 κουταλάκι του γλυκού.Αδειάστε τη σκόνη σε ένα ποτήρι με κρύο νερό ή χυμό και ανακατέψτε μέχρι να διαλυθεί.Το Cranberry Complex μπορεί να λαμβάνεται συνεχώς για παρατεταμένο χρονικό διάστημα.</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Δεν είναι γνωστές προφυλάξεις για τη συνιστώμενη δοσολογία.
+Αλλεργίες:ΑΥΤΟ ΤΟ ΠΡΟΪΟΝ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρια, οστρακοειδή ή θειώδη άλατα.</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100gr σκόνης</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατηγορία lamberts.gr: Βότανα › Σκευάσματα Cranberry</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -1361,7 +2097,44 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής καθαρότητας και ισχύος έλαιο Μέντας</t>
+          <t xml:space="preserve">Η μέντα έχει μακρά παράδοση χρήσης ως βοηθητικό πέψης* και για τον λόγο αυτόν, η κατανάλωση τσαγιού μέντας μετά το γεύμα αποτελεί μια κοινή και αρκετά διαδεδομένη πρακτική σε αρκετές χώρες του κόσμου. Οι ευεργετικές ιδιότητες της μέντας αποδίδονται τα πτητικά έλαια των φύλλων της, και ιδιαίτερα στην μενθόλη.
+Κάθε κάψουλα Peppermint Oil της Lamberts® παρέχει 100mg καθαρού φυσικού ελαίου, αποσταγμένου από φύλλα μέντας. Η διαδικασία εκχύλισης και η καψουλοποίηση του ελαίου που χρησιμοποιείται στο παρόν σκεύασμα, διασφαλίζει την διατήρηση των πτητικών ελαίων σε αρίστη κατάσταση, έως την στιγμή κατανάλωση τους.
+Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Έλαιο Μέντας
+100mg
+Συστατικά: Έλαιο Ηλιόσπορου, Περίβλημα Κάψουλας (Τροποποιημένο Άμυλο, Γλυκερόλη, Πηκτωματοποιητής: Καραγεννάνη, Ρυθμιστής Οξύτητας: Ανθρακικό Νάτριο), Έλαιο Μέντας (Mentha piperita).</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1-2 κάψουλες ημερησίως, από μια μετά από κάθε γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καµία γνωστή για την προτεινόµενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90caps</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 24279/11.03.2021 | Κατηγορία lamberts.gr: Συμπληρώματα πέψης</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -1467,7 +2240,51 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Έλαιο Νυχτολούλουδου των 1000mg με Βιταμίνη Ε</t>
+          <t xml:space="preserve">Το έλαιο νυχτολούλουδου (Evening Primrose Oil ) αποτελεί μία από τις ελάχιστες φυσικές πηγές γ-λινολεϊκού οξέος (GLA). Το GLA αποτελεί πολυακόρεστο Ω-6 λιπαρό οξύ, με ευρείες βιολογικές δράσεις που προκύπτουν από το ότι αποτελεί πρόδρομο μόριο της προσταγλανδίνης PGE1. Αν και ο οργανισμός μπορεί να συνθέσει GLA, πολλές φορές αυτό δεν αρκεί και απαιτείται διατροφική πρόσληψη.
+Το GLA συνιστάται συχνά σε γυναίκες κατά τη διάρκεια της εμμήνου ρήσεως και κατά τη διάρκεια της εμμηνόπαυσης.
+To Pure Evening Primrose Oil 1000mg αποτελεί ένα υψηλής ισχύος και καθαρότητας σκεύασμα ελαίου νυχτολούλουδου το οποίο παρέχει 90mg GLA ανά κάψουλα.
+Το έλαιο που χρησιμοποιείται είναι προσεκτικά επιλεγμένο με βάση την καθαρότητα του και την περιεκτικότητα σε GLA. Επιπροσθέτως, παρέχει μια εξαιρετική ποσότητα βιταμίνης Ε, η οποία συμβάλλει στην προστασία των κυττάρων από το οξειδωτικό στρες*.
+Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη Ε
+10mg
+Έλαιο Νυχτολούλουδου
+1000mg
+το οποίο αποδίσει
+Γ-Λινολενικό Οξύ (GLA)
+90mg
+Συστατικά: Έλαιο Νυχτολούλουδου (Oenothera biennis), Περίβλημα Κάψουλας (Βόειος Ζελατίνη, Γλυκερόλη), Αντιοξειδωτικό: Βιταμίνη Ε (Οξεϊκή dl-α-Τοκοφερόλη).</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1- 3 κάψουλες ημερησίως με το γεύμα ή σύμφωνα με τις οδηγίες του γιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Άτομα που πάσχουν από επιληψία πρέπει να συμβουλεύονται τον Ιατρό τους πρίν την λήψη του συγκεκριμένου συμπληρώματος.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90caps</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 69789/08.11.2006 | Κατηγορία lamberts.gr: Ω - Λιπαρά Οξέα › Ω-6 Λιπαρά οξέα</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -1624,7 +2441,53 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής καθαρότητας έλαιο Λιναρόσπορου ψυχρής έκθλιψης</t>
+          <t xml:space="preserve">Ο λιναρόσπορος αποτελεί μια εξαιρετική εναλλακτική πηγή Ω-3 λιπαρών οξέων, καθώς το έλαιο του αποτελείται σε ποσοστό άνω του 50% από α-λινολενικό οξύ. Το α-λινολενικό οξύ τρέπεται στον οργανισμό σε EPA και DHA, με το ποσοστό της μετατροπής να καθορίζεται από τις ανάγκες του οργανισμού. Επιπροσθέτως , το α-λινολενικό οξύ επεμβαίνει άμεσα στον μεταβολισμό και στην ομοιοστασία των λιπιδίων. Μάλιστα, η ημερήσια πρόσληψη 2g α-λινολενικού οξέος, συμβάλλει στη διατήρηση των φυσιολογικών επιπέδων χοληστερόλης στο αίμα*.
+Εκτός, της υψηλής ποσότητας α-λινολενικού οξέος, το έλαιο λιναρόσπορου , παρέχει και μια σημαντική ποσότητα λινολεϊκού οξέος. Το λινολεϊκό οξύ αποτελεί απαραίτητο Ω-6 λιπαρό οξύ, από το οποίο συντίθενται ενδογενώς τα υπόλοιπα Ω-6 λιπαρά.
+Το Flax Seed Oil 1000mg της Lamberts® αποτελεί ένα υψηλής ισχύος σκεύασμα λιναρόσπορου ψυχρής έκθλιψης , με περιεκτικότητα σε α-λινολενικό οξύ που υπερβαίνει το 60% . Η ψυχρή έκθλιψη αποτελεί μέθοδο εκχύλισης φυτικών ελαίων χωρίς προσθήκη οποιουδήποτε τύπου θέρμανσης, διασφαλίζοντας την δομική ακεραιότητα των μικροθρεπτικών συστατικών και την παραγωγή ενός τελικού προϊόντος ανωτάτης ποιότητας.
+Το έλαιο προστατεύεται από την οξείδωση με την προσθήκη Βιταμίνης Ε.
+Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Έλαιο Λιναρόσπορου
+1000mg
+Το οποίο αποδίδει:
+Α-Λινολενικό Οξύ
+680mg
+Λινολεϊκό Οξύ
+122mg
+Βιταμίνη Ε
+2mg
+Συστατικά: Έλαιο Λιναρόσπορου (Linum usitatissimum), Περίβλημα Κάψουλας (Πηκτωματοποιητές: Γλυκερόλη, Τροποποιημένο Άμυλο &amp; Καραγεννάνη, Χρωστικές: Οξείδιο του Σιδήρου), Αντιοξειδωτικό: Βιταμίνη Ε (dl-α-τοκοφερόλη).</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Μασήστε 1- 3 κάψουλες ημερησίως με το γεύμα ή σύμφωνα με τις οδηγίες του γιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινομένη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90caps</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 69790/08.11.2006 | Κατηγορία lamberts.gr: Ω - Λιπαρά Οξέα › Ω-3 Λιπαρά οξέα φυτικής προελεύσεως</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -1796,7 +2659,67 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Η ολοκληρωμένη φόρμουλα Γλυκοζαμίνης &amp; Χονδροϊτίνης</t>
+          <t xml:space="preserve">Το Glucosamine Complete της Lamberts® αποτελεί ένα ολοκληρωμένο σύμπλεγμα θειικής γλυκοζαμίνης και χονδροϊτίνης φυτικής προελεύσεως (GlucosaGreen® και φυτοδροϊτίνης , αντίστοιχα), σε συνδυασμό με το σύνολο των βιοδραστικών συστατικών για τα οποία υπάρχουν επαρκείς και αξιόπιστες βιβλιογραφικές αναφορές για την δράση τους στον αρθρικό χόνδρο (ΜSM, κερσετίνη , τιτλοδοτημένο εκχύλισμα πιπερόριζας (Ginger) και τιτλοδοτημένο εκχύλισμα καρπών αγριοτριανταφυλλιάς (Rose Hip).
+Κάθε δραστικό συστατικό έχει επιλεγεί με βάση τόσο τον μηχανισμό δράσης του, όσο την συνέργεια των συστατικών μεταξύ τους.
+Η GlucosaGreen® αποτελεί θειική γλυκοζαμίνη 100% φυτικής προελεύσεως που παρασκευάζεται από μη γενετικά τροποποιημένο καλαμπόκι μέσω μιας εξειδικευμένης και πρωτοποριακής διαδικασίας ζύμωσης. Η διαδικασία αυτή διασφαλίζει την παραγωγή θειικής γλυκοζαμίνης που είναι πανομοιότυπη και βιοισοδύναμη με τη θειική γλυκοζαμίνη των οστρακοειδών.
+Επιπροσθέτως:
+Δεν περιέχει κανένα διατροφικό αλλεργιογόνο και ως εκ τούτου είναι κατάλληλη για χρήση από άτομα με ιστορικό υπερευαισθησίας στα οστρακοειδή.
+Ο έλεγχος των πρώτων υλών και η ιχνηλασιμότητα στην όλη διαδικασία διασφαλίζει την απουσία περιβαλλοντικών ρύπων στο τελικό προϊόν και την δυνατότητα ασφαλούς μακροχρόνιας χορήγησης.
+Η όλη διαδικασία παραγωγής είναι φιλική ως προς το περιβάλλον καθώς απαιτεί μικρότερή κατανάλωση νερού και άλλων πρώτων υλών και συνοδεύεται από συντριπτικά μικρότερη παραγωγή υγρών και στερεών αποβλήτων.
+Η φυτοδροϊτίνη αποτελεί χονδροϊτίνη 100% φυτικής προελεύσεως με ταυτόσημη χημική δομή και βιοισοδυναμία με τη θειική χονδροϊτίνη που παρασκευάζεται από ζωικές πηγές. Η πηγή προελεύσεως της φυτοδροϊτίνης είναι τα βρώσιμα θαλάσσια φύκια, κυστοειδές φύκι (Fucus Vesicullosus) και μαρούλι της θάλασσας (Ulva lactuca).
+Η συνιστώμενη ημερήσια δόση των 3 ταμπλετών του Glucosamine Complete της Lamberts® παρέχει 1400mg θειικής γλυκοζαμίνης , μια συγκέντρωση που έχει χρησιμοποιηθεί στην πλειονότητα των κλινικών μελετών.
+Όπως όλα τα σκευάσματα της Lamberts® , το Glucosamine Complete παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά 3 ταμπλέτες
+GlucosaGreen®
+Θειϊκή Γλυκοζαμίνη 2KCl
+1857mg
+Η οποία περιέχει Θειϊκή Γλυκοζαμίνη
+1400mg
+Η οποία αποδίδει Βάση Γλυκοζαμίνης
+1100mg
+Φυτοδροϊτίνη™
+(Ισοδύναμο Χονδροϊτίνης 300mg)
+330mg
+MSM (Μεθυλοσουλφονυλμεθάνη)
+150mg
+Κερσετίνη
+50mg
+Τζίντζερ (παρέχεται από 60mg εκχυλίσματος 20:1)
+1200mg
+Καρποί Αγριοτριανταφυλλιάς (παρέχεται από 100mg εκχυλίσματος 4:1)
+400mg
+Συστατικά: GlucosaGreen® (Θειϊκή Γλυκοζαμίνη 2KCl), Τροποποιημένο Άμυλο, Κυτταρίνη, Φυτοδροϊτίνη™ (Fucus Vesiculosus, Ulva Lactuca, Υαλουρονικό Νάτριο), Μεθυλοσουλφονυλμεθάνη, Εκχύλισμα Καρπών Αγριοτριανταφυλλιάς (Rosa canina L.), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Μαγνήσιο &amp; Στεατικό Οξύ), Κερσετίνη, Εκχύλισμα Τζίντζερ (Zingiber officianale), Στιλβωτικοί Παράγοντες (Υδροξυπροπυλο Mεθυλοκυτταρίνη &amp; Γλυκερόλη).</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 3 ταμπλέτες ημερησίως, κατά προτίμηση μια με το πρωινό και μια με το μεσημεριανό ή το βραδινό σας ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60&amp;120tabs</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 39051/13.04.2022 | Κατηγορία lamberts.gr: Συμπληρώματα για Αρθρώσεις</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -1854,7 +2777,67 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Η ολοκληρωμένη φόρμουλα Γλυκοζαμίνης &amp; Χονδροϊτίνης</t>
+          <t xml:space="preserve">Το Glucosamine Complete της Lamberts® αποτελεί ένα ολοκληρωμένο σύμπλεγμα θειικής γλυκοζαμίνης και χονδροϊτίνης φυτικής προελεύσεως (GlucosaGreen® και φυτοδροϊτίνης , αντίστοιχα), σε συνδυασμό με το σύνολο των βιοδραστικών συστατικών για τα οποία υπάρχουν επαρκείς και αξιόπιστες βιβλιογραφικές αναφορές για την δράση τους στον αρθρικό χόνδρο (ΜSM, κερσετίνη , τιτλοδοτημένο εκχύλισμα πιπερόριζας (Ginger) και τιτλοδοτημένο εκχύλισμα καρπών αγριοτριανταφυλλιάς (Rose Hip).
+Κάθε δραστικό συστατικό έχει επιλεγεί με βάση τόσο τον μηχανισμό δράσης του, όσο την συνέργεια των συστατικών μεταξύ τους.
+Η GlucosaGreen® αποτελεί θειική γλυκοζαμίνη 100% φυτικής προελεύσεως που παρασκευάζεται από μη γενετικά τροποποιημένο καλαμπόκι μέσω μιας εξειδικευμένης και πρωτοποριακής διαδικασίας ζύμωσης. Η διαδικασία αυτή διασφαλίζει την παραγωγή θειικής γλυκοζαμίνης που είναι πανομοιότυπη και βιοισοδύναμη με τη θειική γλυκοζαμίνη των οστρακοειδών.
+Επιπροσθέτως:
+Δεν περιέχει κανένα διατροφικό αλλεργιογόνο και ως εκ τούτου είναι κατάλληλη για χρήση από άτομα με ιστορικό υπερευαισθησίας στα οστρακοειδή.
+Ο έλεγχος των πρώτων υλών και η ιχνηλασιμότητα στην όλη διαδικασία διασφαλίζει την απουσία περιβαλλοντικών ρύπων στο τελικό προϊόν και την δυνατότητα ασφαλούς μακροχρόνιας χορήγησης.
+Η όλη διαδικασία παραγωγής είναι φιλική ως προς το περιβάλλον καθώς απαιτεί μικρότερή κατανάλωση νερού και άλλων πρώτων υλών και συνοδεύεται από συντριπτικά μικρότερη παραγωγή υγρών και στερεών αποβλήτων.
+Η φυτοδροϊτίνη αποτελεί χονδροϊτίνη 100% φυτικής προελεύσεως με ταυτόσημη χημική δομή και βιοισοδυναμία με τη θειική χονδροϊτίνη που παρασκευάζεται από ζωικές πηγές. Η πηγή προελεύσεως της φυτοδροϊτίνης είναι τα βρώσιμα θαλάσσια φύκια, κυστοειδές φύκι (Fucus Vesicullosus) και μαρούλι της θάλασσας (Ulva lactuca).
+Η συνιστώμενη ημερήσια δόση των 3 ταμπλετών του Glucosamine Complete της Lamberts® παρέχει 1400mg θειικής γλυκοζαμίνης , μια συγκέντρωση που έχει χρησιμοποιηθεί στην πλειονότητα των κλινικών μελετών.
+Όπως όλα τα σκευάσματα της Lamberts® , το Glucosamine Complete παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά 3 ταμπλέτες
+GlucosaGreen®
+Θειϊκή Γλυκοζαμίνη 2KCl
+1857mg
+Η οποία περιέχει Θειϊκή Γλυκοζαμίνη
+1400mg
+Η οποία αποδίδει Βάση Γλυκοζαμίνης
+1100mg
+Φυτοδροϊτίνη™
+(Ισοδύναμο Χονδροϊτίνης 300mg)
+330mg
+MSM (Μεθυλοσουλφονυλμεθάνη)
+150mg
+Κερσετίνη
+50mg
+Τζίντζερ (παρέχεται από 60mg εκχυλίσματος 20:1)
+1200mg
+Καρποί Αγριοτριανταφυλλιάς (παρέχεται από 100mg εκχυλίσματος 4:1)
+400mg
+Συστατικά: GlucosaGreen® (Θειϊκή Γλυκοζαμίνη 2KCl), Τροποποιημένο Άμυλο, Κυτταρίνη, Φυτοδροϊτίνη™ (Fucus Vesiculosus, Ulva Lactuca, Υαλουρονικό Νάτριο), Μεθυλοσουλφονυλμεθάνη, Εκχύλισμα Καρπών Αγριοτριανταφυλλιάς (Rosa canina L.), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Μαγνήσιο &amp; Στεατικό Οξύ), Κερσετίνη, Εκχύλισμα Τζίντζερ (Zingiber officianale), Στιλβωτικοί Παράγοντες (Υδροξυπροπυλο Mεθυλοκυτταρίνη &amp; Γλυκερόλη).</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 3 ταμπλέτες ημερησίως, κατά προτίμηση μια με το πρωινό και μια με το μεσημεριανό ή το βραδινό σας ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60&amp;120tabs</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 39051/13.04.2022 | Κατηγορία lamberts.gr: Συμπληρώματα για Αρθρώσεις</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -1912,7 +2895,52 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής ισχύος σύμπλεγμα Γλουταθειόνης</t>
+          <t xml:space="preserve">Η γλουταθειόνη αποτελεί τριπεπτίδιο, το οποίο συντίθεται σε όλα τα κύτταρα του οργανισμού από γλουταμινικό οξύ, κυστεΐνη και γλυκίνη . Η γλουταθειόνη αποτελεί ένα από τα σημαντικότερα μόρια του οργανισμού καθώς αποτελεί βασικό ρυθμιστή στην εξουδετέρωση των ελευθέρων ριζών.
+Εκτός της αντιοξειδωτικής της δράσης, η γλουταθειόνη συμμετέχει και στην ενδοκυττάρια εξουδετέρωση τοξινών. Μάλιστα, η ενδοκυττάρια εξουδετέρωση των τοξινών από την γλουταθειόνη, αποτελεί ένα από τους βασικούς μηχανισμούς με τους οποίους το ήπαρ δρα ως όργανο αποτοξίνωσης.
+Το Glutathione Complex της Lamberts® περιέχει επαρκή επίπεδα των 3 πεπτιδίων που συνθέτουν την γλουταθειόνη όπως επίσης και το τριπεπτίδιο της γλουταθειόνης για την μεγιστοποίηση της απορρόφησης και της βιοδιαθεσιμότητας.
+Όπως όλα τα σκευάσματα της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+Σημαντική Σημείωση: Η Γλουταθειόνη αποτελεί θειούχο αμινοξύ και χαρακτηρίζεται από έντονη οσμή. Η οσμή είναι καθόλα φυσιολογική και δεν στοιχειοθετεί αλλοίωση του σκευάσματος.</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+L-Γλουταμικό Οξύ
+194mg
+L-Κυστεΐνη
+158mg
+Γλυκίνη
+98mg
+L-Γλουταθειόνη
+50mg
+Συστατικά: L-Κυστεΐνη, L-Γλουταμικό Οξύ, Περίβλημα Κάψουλας (Υδρόξυπροπυλο Μεθυλοκυτταρίνη), Γλυκίνη, L-Γλουταθειόνη (μειωμένη μορφή), Διογκωτικός Παράγοντας (Κυτταρίνη), Παράγοντες Αντισυσσωμάτωσης (Στεατικό Μαγνήσιο &amp; Διοξείδιο του Πυριτίου).</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1-3 κάψουλες ημερησίως με νερό ή χυμό φρούτων ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη. Τα αμινοξέα έχουν καλύτερη απορρόφηση όταν λαμβάνονται μισή ώρα πριν το φαγητό ή τον ύπνο.</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60caps</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 67439/08.10.2015 | Κατηγορία lamberts.gr: Αμινοξέα</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -1965,7 +2993,50 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Φυσική πηγή 5-HTP (5-υδροξυτρυπτοφάνη)</t>
+          <t xml:space="preserve">Η 5-HTP (συντομογραφία για την 5-υδροξυτρυπτοφάνη), αποτελεί την υδροξυλιωμένη μορφή του αμινοξέως τρυπτοφάνη. Ο οργανισμός παράγει 5-ΗΤΡ από τρυπτοφάνη, η οποία εν συνεχεία μετατρέπεται σε σεροτονίνη. Η σεροτονίνη αποτελεί έναν νευροδιαβιβαστή με ευρύ φάσμα βιολογικών λειτουργιών, που αφορούν στην ρύθμιση της όρεξης, της διάθεσης, του ύπνου, στον έλεγχο των παρορμήσεων και στην μνήμη.
+Η 5-HTP που περιέχεται στο Griffonia Seed Extract της Lamberts® είναι φυσικής προελεύσεως και συγκεκριμένα προέρχεται από τους σπόρους του αφρικανικού φυτού Griffonia simplicifolia. Το εκχύλισμα των σπόρων του φυτού, αποτελεί ένα από τα πιο ευρέως διαδεδομένα συμπληρώματα 5-HTP παγκοσμίως και ιδιαίτερα δημοφιλές μεταξύ των Επαγγελματιών Υγείας των ΗΠΑ.
+Όπως συμβαίνει με όλα τα βότανα που παρασκευάζονται από τη Lamberts®, υπάρχει αυξημένη επαγρύπνηση σχετικά με την επιλογή των πρώτων υλών. Η επιλογή των πρώτων υλών γίνεται πάντοτε με βάση διεθνείς κατευθυντήριες οδηγίες που αφορούν στην καθαρότητα τους και στην απουσία περιβαλλοντικών ρύπων .
+Η συνιστώμενη ημερήσια δόση του Griffonia Seed Extract της Lamberts® παρέχει τα επίπεδα της 5-HTP που χρησιμοποιούνται στις κλινικές μελέτες .
+Όπως όλα τα σκευάσματα της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Σπόροι Griffonia
+(ως 362mg τιτλοδοτημένου εκχυλίσματος (11:1))
+3982mg
+Το οποίο παρέχει
+5-Υδρόξυτρυπτοφάνη (5-HTP)
+100mg
+Συστατικά: Διογκωτικοί Παράγοντες (Ανθρακικό Ασβέστιο), Τιτλοδοτημένο Εκχύλισμα Σπόρων Griffonia (Griffonia simplicifolia), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Στιλβωτικοί Παράγοντες (Υδροξυπροπυλο Μεθυλοκυτταρίνη, Γλυκερόλη).</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1-3 ταμπλέτες ημερησίως μισή ώρα πριν τα γεύματα ή μισή ώρα πριν την βραδινή κατάκλιση. Ξεκινήστε με μία ταμπλέτα και αυξήστε αν είναι αναγκαίο ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Το 5-HTP λαμβάνεται για περιόδους έως 3 μηνών. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες. Σε ορισμένα άτομα μπορεί να προκληθεί ήπια ζάλη. Συνίσταται η αποφυγή χειρισμού βαρέων μηχανημάτων και οδήγησης, έως όταν καθοριστεί με ποιον τρόπο δρα το 5-ΗΤΡ στον καταναλωτή. Συμβουλευτείτε τον ιατρό σας εάν λαμβάνετε αντικαταθλιπτικά.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60tabs</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 124062/17.11.2023 | Κατηγορία lamberts.gr: Ειδικά Διατροφικά Συμπληρώματα › 5-HTP</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -2385,7 +3456,54 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Αναβράζον Μαγνήσιο υψηλής απορρόφησης και βιοδιαθεσιμότητας</t>
+          <t xml:space="preserve">Το αναβράζον MagAsorb της Lamberts παρέχει εγγυημένα 300mg υψηλής βιοδιαθεσιμότητας μαγνήσιο με προσθήκη Βιταμίνης Β6 (4,2mg ανά ταμπλέτα)
+Το μαγνήσιο αποτελεί ένα από τα σημαντικότερα μέταλλα για τον οργανισμό καθώς παίζει ρόλο στη διαδικασία της κυτταρικής διαίρεσης και συμβάλλει:
+στη μείωση της κούρασης και της κόπωσης
+στην ισορροπία των ηλεκτρολυτών
+στη φυσιολογική λειτουργία των μεταβολικών διεργασιών που αποσκοπούν στην παραγωγή ενέργειας
+στη φυσιολογική λειτουργία του νευρικού συστήματος και των μυών
+στη φυσιολογική σύνθεση των πρωτεϊνών
+στη φυσιολογική ψυχολογική λειτουργία
+στη διατήρηση της φυσιολογικής κατάστασης των οστών και των δοντιώ
+Όπως όλα τα σκευάσματα της Lamberts, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Μαγνήσιο
+(ως Ανθρακικό, Κιτρικό και Οξείδιο του Μαγνησίου)
+300mg
+Βιταμίνη B6
+4.2mg
+Συστατικά: Κιτρικό Οξύ, Ανθρακικό Μαγνήσιο, Ρυθμιστές Οξύτητας: Ανθρακικό Νάτριο, Κιτρικό Μαγνήσιο, Υγραντικό: Σορβιτόλη, Οξείδιο του Μαγνησίου, Ινουλίνη, Ενισχυτικό Γεύσης, Παράγοντας Αντισυσσωμάτωσης (Φωσφορικό Ασβέστιο), Γλυκαντικός Παράγοντας (Σουκραλόζη), Βιταμίνη Β6 (Υδροχλωρική Πυριδοξίνη), Χρωστικές: Ριβοφλαβίνη.</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 δισκίο ημερησίως (διαλυμένο σε ένα ποτήρι νερό) μετά το γεύμα ή σύμφωνα με τη σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Κατανάλωση μαγνησίου που υπερβαίνει τα 400mg δύναται να προκαλέσει ήπιες γαστρεντερικές διαταραχές σε ευαίσθητα άτομα.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20δισκία</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 63116/09.06.2023 | Κατηγορία lamberts.gr: Μέταλλα › Μαγνήσιο</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -2438,7 +3556,54 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Αναβράζον Μαγνήσιο υψηλής απορρόφησης και βιοδιαθεσιμότητας</t>
+          <t xml:space="preserve">Το αναβράζον MagAsorb της Lamberts παρέχει εγγυημένα 300mg υψηλής βιοδιαθεσιμότητας μαγνήσιο με προσθήκη Βιταμίνης Β6 (4,2mg ανά ταμπλέτα)
+Το μαγνήσιο αποτελεί ένα από τα σημαντικότερα μέταλλα για τον οργανισμό καθώς παίζει ρόλο στη διαδικασία της κυτταρικής διαίρεσης και συμβάλλει:
+στη μείωση της κούρασης και της κόπωσης
+στην ισορροπία των ηλεκτρολυτών
+στη φυσιολογική λειτουργία των μεταβολικών διεργασιών που αποσκοπούν στην παραγωγή ενέργειας
+στη φυσιολογική λειτουργία του νευρικού συστήματος και των μυών
+στη φυσιολογική σύνθεση των πρωτεϊνών
+στη φυσιολογική ψυχολογική λειτουργία
+στη διατήρηση της φυσιολογικής κατάστασης των οστών και των δοντιώ
+Όπως όλα τα σκευάσματα της Lamberts, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Μαγνήσιο
+(ως Ανθρακικό, Κιτρικό και Οξείδιο του Μαγνησίου)
+300mg
+Βιταμίνη B6
+4.2mg
+Συστατικά: Κιτρικό Οξύ, Ανθρακικό Μαγνήσιο, Ρυθμιστές Οξύτητας: Ανθρακικό Νάτριο, Κιτρικό Μαγνήσιο, Υγραντικό: Σορβιτόλη, Οξείδιο του Μαγνησίου, Ινουλίνη, Ενισχυτικό Γεύσης, Παράγοντας Αντισυσσωμάτωσης (Φωσφορικό Ασβέστιο), Γλυκαντικός Παράγοντας (Σουκραλόζη), Βιταμίνη Β6 (Υδροχλωρική Πυριδοξίνη), Χρωστικές: Ριβοφλαβίνη.</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 δισκίο ημερησίως (διαλυμένο σε ένα ποτήρι νερό) μετά το γεύμα ή σύμφωνα με τη σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Κατανάλωση μαγνησίου που υπερβαίνει τα 400mg δύναται να προκαλέσει ήπιες γαστρεντερικές διαταραχές σε ευαίσθητα άτομα.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20δισκία</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 63116/09.06.2023 | Κατηγορία lamberts.gr: Μέταλλα › Μαγνήσιο</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -2587,7 +3752,68 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εξειδικευμένο Σύμπλεγμα Βιταμινών Β</t>
+          <t xml:space="preserve">Το Methyl B Complex της Lamberts αποτελεί ένα ειδικά σχεδιασμένο υψηλής ισχύος σύμπλεγμα βιταμινών Β το οποίο παρέχει το σύνολο των βιταμινών Β σε υψηλές ποσότητες σε συνδυασμό με χολίνη και ινοσιτόλη.
+Το ιδιαίτερο χαρακτηριστικό του Methyl B Complex, το οποίο το διαφοροποιεί από άλλα συμπλέγματα Β της εταιρείας μας, είναι ότι παρέχει τις μεταβολικά ενεργείς μορφές του φολικού οξέος, της βιταμίνης Β6 και της βιταμίνης Β12.
+Συγκεκριμένα παρέχει :
+1. Φολικό οξύ σε μορφή L-μεθυλοφολικού ασβεστίου: Το L-μεθυλοφολικό ασβέστιο ου αποτελεί τη μεταβολικά ενεργό (μεθυλιωμένη) μορφή φολικού οξέος.
+2. Βιταμίνη Β6 σε μορφή 5 φωσφορικής πυριδοξάλης (Pyridoxal 5-Phosphate ,P5P): Η 5 φωσφορική πυριδοξάλη αποτελεί την μεταβολικά ενεργό μορφή της βιταμίνης Β6 και ως εκ τούτου χρησιμοποιείται άμεσα από τον οργανισμό, καθώς ενσωματώνεται άμεσα στις μεταβολικές αντιδράσεις.
+3. Βιταμίνη Β12 σε μορφή μεθυλοκοβαλαμίνης: Η μεθυλοκοβαλαμίνη οποία αποτελεί την μεταβολικά ενεργό μορφή της βιταμίνης Β12 και τη βιταμίνη Β12 με την μέγιστη απορρόφηση και βιοδιαθεσιμότητα.
+Τα συγκεκριμένα μικροθρεπτικά συστατικά συμμετέχουν στον μεταβολισμό της ομοκυστεΐνης, συμβάλλοντας στην μείωση των επίπεδων της*, ενώ η χρήση των μεταβολικά ενεργών (μεθυλιωμένων) μορφών τους διασφαλίζει την κάλυψη και των ατόμων που αδυνατούν να τα μεθυλιώσουν (πολυμορφισμοί στο γονίδιο MTHFR).
+Όπως όλα τα σκευάσματα της Lamberts® , το Methyl B Complex της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Θειαμίνη (B1)
+25mg
+Ριβοφλαβίνη (Β2)
+28mg
+Νιασίνη (B3)
+32mg NE
+Βιταμίνη Β6 (ως P5P)
+12mg
+Φολικό οξύ
+ως L-Μεθυλοφολικό Ασβέστιο
+200µg
+Βιταμίνη B12
+300µg
+Βιοτίνη
+250µg
+Παντοθενικό Οξύ (Β5)
+50mg
+Ινοσιτόλη
+30mg
+Χολίνη
+30mg
+Συστατικά: Τροποποιημένο Άμυλο, Διογκωτικός Παράγοντας (Κυτταρίνη), Διτρυγική Χολίνη, Παντοθενικό Οξύ (Παντοθενικό Ασβέστιο), Μονονιτρική Θειαμίνη, Νιασίνη (Νικοτιναμίδιο), Ινοσιτόλη, Ριβοφλαβίνη, Βιταμίνη Β6 (ως 5-Φωσφορική Μονοϋδρική Πυριδοξάλη), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Επικάλυψη Ταμπλέτας (Υδροξυπρόπυλο Μεθυλοκυτταρίνη, Γλυκερόλη), Βιταμίνη Β12 (Μεθυλοκοβαλαμίνη), Φολικό Οξύ (L-Μεθυλοφολικό Ασβέστιο), Βιοτίνη.</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες. Μακροχρόνια λήψη αυτής της ποσότητας της Β6 μπορεί να οδηγήσει σε εμφάνιση ήπιων αιμωδιών και μυρμηκιάσεων στα άκρα.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60tabs</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 94173/7.12.2016 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνες B</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -2736,7 +3962,54 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Αναβράζον Μαγνήσιο υψηλής απορρόφησης και βιοδιαθεσιμότητας</t>
+          <t xml:space="preserve">Το αναβράζον MagAsorb της Lamberts παρέχει εγγυημένα 300mg υψηλής βιοδιαθεσιμότητας μαγνήσιο με προσθήκη Βιταμίνης Β6 (4,2mg ανά ταμπλέτα)
+Το μαγνήσιο αποτελεί ένα από τα σημαντικότερα μέταλλα για τον οργανισμό καθώς παίζει ρόλο στη διαδικασία της κυτταρικής διαίρεσης και συμβάλλει:
+στη μείωση της κούρασης και της κόπωσης
+στην ισορροπία των ηλεκτρολυτών
+στη φυσιολογική λειτουργία των μεταβολικών διεργασιών που αποσκοπούν στην παραγωγή ενέργειας
+στη φυσιολογική λειτουργία του νευρικού συστήματος και των μυών
+στη φυσιολογική σύνθεση των πρωτεϊνών
+στη φυσιολογική ψυχολογική λειτουργία
+στη διατήρηση της φυσιολογικής κατάστασης των οστών και των δοντιώ
+Όπως όλα τα σκευάσματα της Lamberts, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Μαγνήσιο
+(ως Ανθρακικό, Κιτρικό και Οξείδιο του Μαγνησίου)
+300mg
+Βιταμίνη B6
+4.2mg
+Συστατικά: Κιτρικό Οξύ, Ανθρακικό Μαγνήσιο, Ρυθμιστές Οξύτητας: Ανθρακικό Νάτριο, Κιτρικό Μαγνήσιο, Υγραντικό: Σορβιτόλη, Οξείδιο του Μαγνησίου, Ινουλίνη, Ενισχυτικό Γεύσης, Παράγοντας Αντισυσσωμάτωσης (Φωσφορικό Ασβέστιο), Γλυκαντικός Παράγοντας (Σουκραλόζη), Βιταμίνη Β6 (Υδροχλωρική Πυριδοξίνη), Χρωστικές: Ριβοφλαβίνη.</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 δισκίο ημερησίως (διαλυμένο σε ένα ποτήρι νερό) μετά το γεύμα ή σύμφωνα με τη σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Κατανάλωση μαγνησίου που υπερβαίνει τα 400mg δύναται να προκαλέσει ήπιες γαστρεντερικές διαταραχές σε ευαίσθητα άτομα.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20δισκία</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 63116/09.06.2023 | Κατηγορία lamberts.gr: Μέταλλα › Μαγνήσιο</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -2794,7 +4067,53 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Η “advance” φόρμουλα για την υγεία των οστών</t>
+          <t xml:space="preserve">Το Osteoguard ® Advance αποτελεί μια ειδικά σχεδιασμένη φόρμουλα για την οστική υγεία με ασβέστιο, μαγνήσιο, βιταμίνη D3 και βιταμίνη K2. Τα ιδιαίτερα χαρακτηριστικά στο σχεδιασμό του Osteoguard® Advance περιλαμβάνουν:
+Την επιλογή των συγκεκριμένων μικροθρεπτικών συστατικών και της συγκέντρωσης αυτών: Η επιλογή των μικροθρεπτικών συστατικών και της ποσότητας τους έγινε βάσει των ιδιοτήτων τους επί του οστικού μεταβολισμού καθώς, το ασβέστιο, το μαγνήσιο και οι βιταμίνες D &amp; K, συμβάλλουν* στην διατήρηση της φυσιολογικής κατάστασης των οστών.
+Την επιλογή των μορφών των μεταλλικών αλάτων με τις οποίες διασφαλίζεται η μέγιστη δυνατή απορρόφηση και βιοδιαθεσιμότητα: Οι μορφές αλάτων των μετάλλων του Osteoguard® Advance είναι αυτές με τις οποίες διασφαλίζεται η μέγιστη δυνατή απορρόφηση και βιοδιαθεσιμότητα . Συγκεκριμένα το άλας ασβεστίου στο παρόν σκεύασμα αποτελεί μίγμα ανθρακικού και κιτρικού ασβεστίου , ενώ το άλας μαγνησίου αποτελεί μίγμα ανθρακικού ,κιτρικού και υδροξειδίου του μαγνησίου.
+Την επιλογή της ιδανικής αναλογία ασβεστίου / μαγνησίου: Η αναλογία ασβεστίου/μαγνησίου του Osteoguard® Advance είναι 2:1, καθώς η αναλογία αυτή ενισχύει περαιτέρω την απορρόφηση του ασβεστίου από τον εντερικό βλεννογόνο.
+Όπως σε όλα τα σκευάσματα της Lamberts® που περιέχουν Κ2, η βιταμίνη Κ2 στο Osteoguard ® Advance , βρίσκεται στη φυσική της μορφή (ως μενακινόνη/ΜΚ-7) . Εν αντιθέσει με αντίστοιχα σκευάσματα του ανταγωνισμού που χρησιμοποιούν Κ2 από προερχόμενη από το νάττο (παραδοσιακό ιαπωνικό τρόφιμο που παρασκευάζεται από φασόλια σόγιας ), η Κ2 της Lamberts® παρασκευάζεται από ρεβίθια μέσω μιας ειδικής διαδικασίας ζύμωσης. Το γεγονός αυτό διασφαλίζει ότι το σκεύασμά μας δεν περιέχει ως διατροφικά αλλεργιογόνα σόγια και υποπροϊόντα γάλακτος.
+Όπως όλα τα σκευάσματα της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά 2 ταμπλέτες
+Βιταμίνη D3
+10μg
+Βιταμίνη K2
+90μg
+Ασβέστιο
+500mg
+Μαγνήσιο
+250mg
+Συστατικά: Ασβέστιο (Ανθρακικό &amp; Κιτρικό), Μαγνήσιο (Κιτρικό, Υδροξείδιο του Μαγνησίου και Ανθρακικό Μαγνήσιο), Διογκωτικοί Παράγοντες (Κυτταρίνη), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη), Βιταμίνη Κ2 ως Μενακινόνη-7 (ΜΚ-7), Επικάλυψη Ταμπλέτας (Υδροξυπροπυλο Μεθυλοκυτταρίνη &amp; Γλυκερόλη), Βιταμίνη D3 (Χοληκαλσιφερόλη).</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 2 ταμπλέτες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90tabs</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 7723/24.01.2019 | Κατηγορία lamberts.gr: Μέταλλα › Σκευάσματα &amp; Συνδυασμοί Ασβεστίου</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -2814,7 +4133,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/wp-content/uploads/2025/01/8227-90-hr.png</t>
+          <t xml:space="preserve">lamberts/osteoguard-advance-5055148412050.png</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -2852,7 +4171,52 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Σελήνιο των 200μg &amp; αντιοξειδωτικές Βιταμίνες A, C &amp; E</t>
+          <t xml:space="preserve">Το σελήνιο αποτελεί ένα από τα σημαντικότερα μικροθρεπτικά συστατικά με ευρύ φάσμα βιολογικών δράσεων που περιλαμβάνουν τη συμβολή του στη φυσιολογική σπερματογένεση, στη φυσιολογική θυρεοειδική λειτουργία ,στη διατήρηση της φυσιολογικής κατάστασης των μαλλιών και των νυχιών, στη φυσιολογική λειτουργία του ανοσοποιητικού συστήματος, και στην προστασία των κυττάρων από το οξειδωτικό στρες*.
+Παρά το σημαντικό του ρόλο ωστόσο, η σύγχρονη διατροφική πρόσληψη σεληνίου είναι ανεπαρκής.
+Το Selenium 200μg A+C+E, αποτελεί ένα υψηλής ισχύος σκεύασμα σεληνίου, το οποίο ανά ταμπλέτα παρέχει 200μg στοιχειακού σεληνίου σε συνδυασμό με υψηλές ποσότητες βιταμινών Α ,C και Ε.
+Όπως το σελήνιο, έτσι και οι βιταμίνες Α, C και Ε, είναι γνωστές για τις αντιοξειδωτικές τους ιδιότητες, καθώς συμβάλλουν στην προστασία των κυττάρων από το οξειδωτικό στρες*.
+Όπως όλα τα σκευάσματα της Lamberts® ,το Selenium 200μg A+C+E παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Βιταμίνη A
+400μg RE
+Βιταμίνη E
+24mg
+Βιταμίνη C
+80mg
+Σελήνιο
+200μg
+Συστατικά: Διογκωτικοί Παράγοντες (Φωσφορικό Διασβέστιο &amp; Κυτταρίνη), Βιταμίνη C (Ασκορβικό Οξύ), Βιταμίνη Ε (Οξεική dl-a Ττοκοφερόλη), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη), Οξεική Βιταμίνη Α, Σελήνιο (L-Σεληνομεθειονίνη &amp; Νατριούχο Σελήνιο).</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Το προϊόν περιέχει βιταμίνη Α. Να μην λαμβάνεται από έγκυους ή θηλάζουσες ή γυναίκες με πιθανότητα εγκυμοσύνης.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100tabs</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 93182/05.12.2013 | Κατηγορία lamberts.gr: Μέταλλα › Σελήνιο</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -2991,7 +4355,104 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Πλήρης κάλυψη γυναικών γυναικών &gt; 50 ετών</t>
+          <t xml:space="preserve">Η Multi-Guard® Osteo Advance 50+ αποτελεί την πιο ολοκληρωμένη και υψηλής περιεκτικότητας πολυβιταμινούχο φόρμουλα που κυκλοφορεί στο Ηνωμένο Βασίλειο για γυναίκες άνω των 50 ετών.
+Ο σχεδιασμός της συγκεκριμένης φόρμουλας έχει ως κεντρικό άξονα την ομοιοστασία του οστικού μεταβολισμού. Για τον λόγο αυτό έχουν προστεθεί επαρκή επίπεδα βιταμίνης D που συμβάλλει στη φυσιολογική απορρόφηση / χρησιμοποίηση του ασβεστίου και υψηλά επίπεδα βιταμίνης Κ2 (ως μενακινόνη /ΜΚ7), ασβεστίου (500mg) και μαγνησίου (250mg) καθώς αυτά τα μικροθρεπτικά συστατικά συμβάλλουν στη διατήρηση της φυσιολογικής κατάστασης των οστών*.
+Οι υψηλές δόσεις ασβεστίου και μαγνησίου, οδήγησαν στην συνιστώμενη ημερήσια δόση των 3 ταμπλετών, ωστόσο καθιστούν περιττή την λήψη ξεχωριστών σκευασμάτων ασβεστίου και μαγνησίου και ως εκ τούτου διασφαλίζουν την ευκολότερη συμμόρφωση στις οδηγίες του Επαγγελματία της Υγείας. Επιπροσθέτως, η αναλογία ασβεστίου/μαγνησίου του Osteoguard® Advance είναι 2:1, γεγονός που ενισχύει περαιτέρω την απορρόφηση του ασβεστίου από τον εντερικό βλεννογόνο.
+Εκτός της βιταμίνης D και των υψηλών δόσεων ασβεστίου και μαγνησίου, η Multi-Guard® Osteo Advance 50+ παρέχει άλλα 23 μικροθρεπτικά συστατικά αποτελώντας μια ολοκληρωμένη επιλογή για γυναίκες άνω των 50 ετών. Μεταξύ αυτών παρέχει τις αντιοξειδωτικές βιταμίνες A,C,E, το σύνολο των βιταμινών Β και άριστα επίπεδα όλων των ιχνοστοιχείων.
+Τέλος, το Multi-Guard® Osteo Advance 50+ περιέχει λουτεΐνη και υψηλές ποσότητες φυσικών αντιοξειδωτικών. Η λουτεΐνη αποτελεί καροτενοειδές που βρίσκεται στα πράσινα λαχανικά και διαδραματίζει σημαντικό ρόλο στην υγεία του οφθαλμού. Σε κάθε ταμπλέτα Multi-Guard® Osteo Advance 50+ περιέχονται 2mg λουτεΐνης φυσικής προσελεύσεως.
+Τα φυσικά αντιοξειδωτικά που περιλαμβάνονται στο Multi-Guard® Osteo Advance 50+ προέρχονται από τιτλοδοτημένα εκχυλίσματα κουρκουμά (Curcuma longa) , δενδρολίβανου (Rosmarinus officinalis L.) και σπόρων κόκκινου σταφυλιού (Vitis vinifera). Και τα τρία βότανα συνοδεύονται από σημαντικό όγκο αναφορών στη σύγχρονη βιβλιογραφία σχετικά με τις βιολογικές τους δράσεις.
+To Multi-Guard® Osteo Advance 50+, όπως όλα τα σκευάσματα της Lamberts®, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές Πληροφορίες
+Ανά 3 ταμπλέτες
+Βιταμίνη A
+800µg
+Βιταμίνη D (D3)
+10μg
+Βιταμίνη Ε
+24mg α-TE
+Βιταμίνη Κ (Κ2)
+75μg
+Βιταμίνη C
+120mg
+Θειαμίνη (Β1)
+5mg
+Ριβοφλαβίνη (Β2)
+4mg
+Νιασίνη (Β3)
+16mg
+Βιταμίνη Β6
+10mg
+Φολικό Οξύ
+200μg
+Βιταμίνη Β12
+100µg
+Βιοτίνη
+150μg
+Παντοθενικό Οξύ (Β5)
+12mg
+Ασβέστιο
+500mg
+Μαγνήσιο
+250mg
+Σίδηρος
+7mg
+Ψευδάργυρος
+15mg
+Χαλκός
+1mg
+Μαγγάνιο
+0,45mg
+Σελήνιο
+110µg
+Χρώμιο
+200μg
+Ιώδιο
+150μg
+Διτρυγική Χολίνη
+5mg
+Ινοσιτόλη
+5mg
+PABA
+5mg
+Λουτεΐνη
+2mg
+Τιτλοδοτημένο εκχύλισμα κουρκουμά
+50mg
+Τιτλοδοτημένο εκχύλισμα δενδρολίβανου
+13mg
+Τιτλοδοτημένο εκχύλισμα σπόρων κόκκινου σταφυλιού
+50mg
+Συστατικά: Ανθρακικό Ασβέστιο, Ανθρακικό και Κιτρικό Μαγνήσιο, Κυτταρίνη, Ασκορβικό Οξύ, Επικάλυψη Ταμπλέτας (Υδρόξυπροπυλο Μεθυλοκυτταρίνη, Πολυδεξτρόζη, Ανθρακικό Ασβέστιο, Χρωστικές: Οξείδιο του Σιδήρου), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ και Στεατικό Μαγνήσιο), Dl-α Τοκοφερόλη, Εκχύλισμα Κουρκουμά (Curcuma longa), Εκχύλισμα Σπόρου Κόκκινου Σταφυλιού (Vitis vinifera), Κιτρικός Ψευδάργυρος, Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη), Μενακινόνη-7 (MΚ-7), Φουμαρικός Σίδηρος, Νικοτιναμίδιο, Παντοθενικό Ασβέστιο, Εκχύλισμα Δενδρολίβανου (Rosmarinus officinalis), Υδροχλωρική Πυριδοξίνη, Κυανοκοβαλαμίνη, Σύμπλεγμα Λουτεΐνης (Λουτεΐνη (Tagetes erecta) &amp; Αντιοξειδωτικά: Εκχύλισμα Δενδρολίβανου (Rosmarinus officinalis)), Οξεική Βιταμίνη Α, Γλυκονικός Χαλκός, Μονονιτρική Θειαμίνη, Χοληκαλσιφερόλη, Παρα Αμινο Βενζοϊκό Οξύ, Διτρυγική Χολίνη, Ινοσιτόλη, Ριβοφλαβίνη, Γλυκονικό Μαγγάνιο, Πικολινικό Χρώμιο, L-Σεληνομεθειονίνη &amp; Νατριούχος Σελενίτης, Φολικό οξύ, Ιωδιούχο Κάλιο, Βιοτίνη.</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 3 ταμπλέτες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Μπορεί να προκληθεί κίτρινος χρωματισμός των ούρων. Αυτό είναι αβλαβές και υποδεικνύει ότι το σώμα αποβάλλει την περίσσια ποσότητα της βιταμίνης Β2 (riboflavin). Το προϊόν αυτό περιέχει σίδηρο, και η υπέρβαση της δοσολογίας μπορεί να είναι επιζήμια, ιδιαίτερα σε μικρά παιδιά. Φυλάξτε το σε σημείο ασφαλές από τα παιδιά. Δεν συνιστάται για εγκύους ή θηλάζουσες γυναίκες ή γυναίκες με πιθανότητα μελλοντικής εγκυμοσύνης, εκτός εάν υπάρχει σαφής σύσταση από θεράποντα γυναικολόγο. Να μην λαμβάνεται από άτομα που βρίσκονται υπό αγωγή με κουμαρινικά αντιπηκτικά, εκτός εάν υπάρχει αντίθετη ιατρική σύσταση. Δεν συνίσταται για άτομα κάτω των 18 ετών.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">120tabs</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 89115/16.12.2015 | Κατηγορία lamberts.gr: Πολυβιταμίνες › Για τη γυναίκα</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -3049,7 +4510,104 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Πλήρης κάλυψη γυναικών γυναικών &gt; 50 ετών</t>
+          <t xml:space="preserve">Η Multi-Guard® Osteo Advance 50+ αποτελεί την πιο ολοκληρωμένη και υψηλής περιεκτικότητας πολυβιταμινούχο φόρμουλα που κυκλοφορεί στο Ηνωμένο Βασίλειο για γυναίκες άνω των 50 ετών.
+Ο σχεδιασμός της συγκεκριμένης φόρμουλας έχει ως κεντρικό άξονα την ομοιοστασία του οστικού μεταβολισμού. Για τον λόγο αυτό έχουν προστεθεί επαρκή επίπεδα βιταμίνης D που συμβάλλει στη φυσιολογική απορρόφηση / χρησιμοποίηση του ασβεστίου και υψηλά επίπεδα βιταμίνης Κ2 (ως μενακινόνη /ΜΚ7), ασβεστίου (500mg) και μαγνησίου (250mg) καθώς αυτά τα μικροθρεπτικά συστατικά συμβάλλουν στη διατήρηση της φυσιολογικής κατάστασης των οστών*.
+Οι υψηλές δόσεις ασβεστίου και μαγνησίου, οδήγησαν στην συνιστώμενη ημερήσια δόση των 3 ταμπλετών, ωστόσο καθιστούν περιττή την λήψη ξεχωριστών σκευασμάτων ασβεστίου και μαγνησίου και ως εκ τούτου διασφαλίζουν την ευκολότερη συμμόρφωση στις οδηγίες του Επαγγελματία της Υγείας. Επιπροσθέτως, η αναλογία ασβεστίου/μαγνησίου του Osteoguard® Advance είναι 2:1, γεγονός που ενισχύει περαιτέρω την απορρόφηση του ασβεστίου από τον εντερικό βλεννογόνο.
+Εκτός της βιταμίνης D και των υψηλών δόσεων ασβεστίου και μαγνησίου, η Multi-Guard® Osteo Advance 50+ παρέχει άλλα 23 μικροθρεπτικά συστατικά αποτελώντας μια ολοκληρωμένη επιλογή για γυναίκες άνω των 50 ετών. Μεταξύ αυτών παρέχει τις αντιοξειδωτικές βιταμίνες A,C,E, το σύνολο των βιταμινών Β και άριστα επίπεδα όλων των ιχνοστοιχείων.
+Τέλος, το Multi-Guard® Osteo Advance 50+ περιέχει λουτεΐνη και υψηλές ποσότητες φυσικών αντιοξειδωτικών. Η λουτεΐνη αποτελεί καροτενοειδές που βρίσκεται στα πράσινα λαχανικά και διαδραματίζει σημαντικό ρόλο στην υγεία του οφθαλμού. Σε κάθε ταμπλέτα Multi-Guard® Osteo Advance 50+ περιέχονται 2mg λουτεΐνης φυσικής προσελεύσεως.
+Τα φυσικά αντιοξειδωτικά που περιλαμβάνονται στο Multi-Guard® Osteo Advance 50+ προέρχονται από τιτλοδοτημένα εκχυλίσματα κουρκουμά (Curcuma longa) , δενδρολίβανου (Rosmarinus officinalis L.) και σπόρων κόκκινου σταφυλιού (Vitis vinifera). Και τα τρία βότανα συνοδεύονται από σημαντικό όγκο αναφορών στη σύγχρονη βιβλιογραφία σχετικά με τις βιολογικές τους δράσεις.
+To Multi-Guard® Osteo Advance 50+, όπως όλα τα σκευάσματα της Lamberts®, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές Πληροφορίες
+Ανά 3 ταμπλέτες
+Βιταμίνη A
+800µg
+Βιταμίνη D (D3)
+10μg
+Βιταμίνη Ε
+24mg α-TE
+Βιταμίνη Κ (Κ2)
+75μg
+Βιταμίνη C
+120mg
+Θειαμίνη (Β1)
+5mg
+Ριβοφλαβίνη (Β2)
+4mg
+Νιασίνη (Β3)
+16mg
+Βιταμίνη Β6
+10mg
+Φολικό Οξύ
+200μg
+Βιταμίνη Β12
+100µg
+Βιοτίνη
+150μg
+Παντοθενικό Οξύ (Β5)
+12mg
+Ασβέστιο
+500mg
+Μαγνήσιο
+250mg
+Σίδηρος
+7mg
+Ψευδάργυρος
+15mg
+Χαλκός
+1mg
+Μαγγάνιο
+0,45mg
+Σελήνιο
+110µg
+Χρώμιο
+200μg
+Ιώδιο
+150μg
+Διτρυγική Χολίνη
+5mg
+Ινοσιτόλη
+5mg
+PABA
+5mg
+Λουτεΐνη
+2mg
+Τιτλοδοτημένο εκχύλισμα κουρκουμά
+50mg
+Τιτλοδοτημένο εκχύλισμα δενδρολίβανου
+13mg
+Τιτλοδοτημένο εκχύλισμα σπόρων κόκκινου σταφυλιού
+50mg
+Συστατικά: Ανθρακικό Ασβέστιο, Ανθρακικό και Κιτρικό Μαγνήσιο, Κυτταρίνη, Ασκορβικό Οξύ, Επικάλυψη Ταμπλέτας (Υδρόξυπροπυλο Μεθυλοκυτταρίνη, Πολυδεξτρόζη, Ανθρακικό Ασβέστιο, Χρωστικές: Οξείδιο του Σιδήρου), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ και Στεατικό Μαγνήσιο), Dl-α Τοκοφερόλη, Εκχύλισμα Κουρκουμά (Curcuma longa), Εκχύλισμα Σπόρου Κόκκινου Σταφυλιού (Vitis vinifera), Κιτρικός Ψευδάργυρος, Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη), Μενακινόνη-7 (MΚ-7), Φουμαρικός Σίδηρος, Νικοτιναμίδιο, Παντοθενικό Ασβέστιο, Εκχύλισμα Δενδρολίβανου (Rosmarinus officinalis), Υδροχλωρική Πυριδοξίνη, Κυανοκοβαλαμίνη, Σύμπλεγμα Λουτεΐνης (Λουτεΐνη (Tagetes erecta) &amp; Αντιοξειδωτικά: Εκχύλισμα Δενδρολίβανου (Rosmarinus officinalis)), Οξεική Βιταμίνη Α, Γλυκονικός Χαλκός, Μονονιτρική Θειαμίνη, Χοληκαλσιφερόλη, Παρα Αμινο Βενζοϊκό Οξύ, Διτρυγική Χολίνη, Ινοσιτόλη, Ριβοφλαβίνη, Γλυκονικό Μαγγάνιο, Πικολινικό Χρώμιο, L-Σεληνομεθειονίνη &amp; Νατριούχος Σελενίτης, Φολικό οξύ, Ιωδιούχο Κάλιο, Βιοτίνη.</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 3 ταμπλέτες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Μπορεί να προκληθεί κίτρινος χρωματισμός των ούρων. Αυτό είναι αβλαβές και υποδεικνύει ότι το σώμα αποβάλλει την περίσσια ποσότητα της βιταμίνης Β2 (riboflavin). Το προϊόν αυτό περιέχει σίδηρο, και η υπέρβαση της δοσολογίας μπορεί να είναι επιζήμια, ιδιαίτερα σε μικρά παιδιά. Φυλάξτε το σε σημείο ασφαλές από τα παιδιά. Δεν συνιστάται για εγκύους ή θηλάζουσες γυναίκες ή γυναίκες με πιθανότητα μελλοντικής εγκυμοσύνης, εκτός εάν υπάρχει σαφής σύσταση από θεράποντα γυναικολόγο. Να μην λαμβάνεται από άτομα που βρίσκονται υπό αγωγή με κουμαρινικά αντιπηκτικά, εκτός εάν υπάρχει αντίθετη ιατρική σύσταση. Δεν συνίσταται για άτομα κάτω των 18 ετών.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">120tabs</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 89115/16.12.2015 | Κατηγορία lamberts.gr: Πολυβιταμίνες › Για τη γυναίκα</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -3102,7 +4660,99 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ρύθμιση μεταβολισμού και ενεργειακού ισοζυγίου</t>
+          <t xml:space="preserve">Το Multi-Guard® Sugar Control αποτελεί μια υψηλής ισχύος πολυβιταμινούχο φόρμουλα, η οποία στοχεύει στη ρύθμιση του μεταβολισμού και στη διατήρηση του ενεργειακού ισοζυγίου του οργανισμού μεταξύ των γευμάτων.
+Περιέχει 25 μικροθρεπτικά συστατικά για την πλήρη κάλυψη του οργανισμού, εκ των οποίων ιδιαίτερη έμφαση δόθηκε σε εκείνα, που εμπλέκονται με σημαντικό τρόπο στον μεταβολισμό των υδατανθράκων.
+Συγκεκριμένα στην συνιστώμενη δόση των 2 ταμπλετών ημερησίως, παρέχει σε επαρκείς / υψηλές ποσότητες:
+1. Χρώμιο: Το χρώμιο εμπλέκεται στο σηματοδοτικό μονοπάτι της ινσουλίνης, συμβάλλοντας στο φυσιολογικό μεταβολισμό των μακροθρεπτικών συστατικών και στη διατήρηση των φυσιολογικών επιπέδων γλυκόζης στο αίμα*.
+2. Ψευδάργυρος: Ο ψευδάργυρος ανευρίσκεται στο σύνολο των κυττάρων του οργανισμού, όντας απαραίτητος σε μια πληθώρα φυσιολογικών βιολογικών λειτουργιών. Μεταξύ αυτών εμπλέκεται σε πληθώρα μεταβολικών αντιδράσεων, συμβάλλοντας στο φυσιολογικό μεταβολισμό των υδατανθράκων *.
+3. Βιταμίνες συμπλέγματος Β: To Multi-Guard® Sugar Control περιέχει το σύνολο των βιταμινών Β, μια ομάδα υδατοδιαλυτών βιταμινών, με εξέχουσα σημασία για τον ανθρώπινο οργανισμό, καθώς σχεδόν κάθε μεταβολική αντίδραση του οργανισμού απαιτεί την παρουσία τους. Εξ αυτών, οι βιταμίνες Β1,Β2,Β3,Β5,Β6 ,Β12 και η βιοτίνη συμβάλουν στη φυσιολογική λειτουργία των μεταβολικών διεργασιών που αποσκοπούν στην παραγωγή ενέργειας, ενώ η Β6 συμβάλλει επιπροσθέτως στον φυσιολογικό μεταβολισμό του γλυκογόνου*. Στο Multi-Guard® Sugar Control η Β6 περιέχεται ως η 5-φωσφορική πυριδοξάλη (P5P), η οποία αποτελεί την μεταβολικά ενεργό μορφή της Β6.
+4. Μαγνήσιο: Η επαρκής διατροφική πρόσληψη μαγνησίου είναι πολύ σημαντική για τον ανθρώπινο μεταβολισμό, καθώς το μαγνήσιο εμπλέκεται σε πάνω από 300 μεταβολικές αντιδράσεις συμβάλλοντας στη φυσιολογική λειτουργία των μεταβολικών διεργασιών που αποσκοπούν στην παραγωγή ενέργειας* . Εντούτοις, οι σύγχρονες δίαιτες και ιδιαίτερα αυτές που χαρακτηρίζονται από αυξημένη κατανάλωση επεξεργασμένων τροφίμων , χαρακτηρίζονται από ανεπαρκή παροχή μαγνησίου, καθιστώντας την ανεπάρκεια μαγνησίου ως μια από τις πιο διαδεδομένες σύγχρονες διατροφικές ανεπάρκειες. To Multi-Guard® Sugar Control παρέχει υψηλή ποσότητα στοιχειακού μαγνησίου στην συνιστώμενη ημερήσια δόση των 2 ταμπλετών, διασφαλίζοντας την κάλυψη του οργανισμού σε αυτό το πολύτιμο, μεταβολικά, μέταλλο.
+5. Κανέλλα: Την τελευταία εικοσαετία, μια πληθώρα επιστημονικών δεδομένων συνδέουν τις δραστικές ουσίες της κανέλλας με τον μεταβολισμό της γλυκόζης. Στο Multi-Guard® Sugar Control παρέχεται μια πολύ υψηλή ποσότητα τιτλοδοτημένου εκχυλίσματος φλοιού κανέλλας Κασσία (Cinnamonum cassia) καθώς με αυτό έχει διεξαχθεί η πλειονότητα των δημοσιευμένων μελετών. Η χρήση του φλοιού της κανέλλας για την παρασκευή του εκχυλίσματος έγινε ,γιατί εκεί ανευρίσκονται οι μεταβολικά δραστικές ουσίες. Το εκχύλισμα δεν περιέχει κουμαρίνη και ως εκ τούτου είναι κατάλληλη για μακροχρόνια χρήση και δεν ενέχει κίνδυνο αλληλεπίδρασης με κουμαρινικά αντιπηκτικά.
+Το Multi-Guard® Sugar Control όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές Πληροφορίες
+Ανά 2 ταμπλέτες
+Βιταμίνη D (D3)
+5µg
+Βιταμίνη Ε
+50mg α-ΤΕ
+Βιταμίνη Κ (K1)
+20µg
+Βιταμίνη C
+100mg
+Θειαμίνη (B1)
+25mg
+Ριβοφλαβίνη (B2)
+12mg
+Νιασίνη (B3)
+50mg NE
+Βιταμίνη Β6 (ως P5P)
+10mg
+Φολικό Οξύ
+400µg
+Βιταμίνη Β12
+50μg
+Βιοτίνη
+150μg
+Παντοθενικό Οξύ
+25mg
+Ασβέστιο
+120mg
+Μαγνήσιο
+300mg
+Σίδηρος
+14mg
+Ψευδάργυρος
+15mg
+Χαλκός
+0,5mg
+Μαγγάνιο
+0,5mg
+Σελήνιο
+200μg
+Χρώμιο
+200μg
+Ιώδιο
+150μg
+Διτρυγική Χολίνη
+25mg
+Ινοσιτόλη
+25mg
+PABA
+25mg
+Κανέλα ως 80 mg τιτλοδοτημένου
+εκχυλίσματος (25:1)
+2000mg
+Συστατικά: Μαγνήσιο (Οξείδιο του Μαγνησίου &amp; Κιτρικό Μαγνήσιο), Διογκωτικός Παράγοντας (Κυτταρίνη), Ανθρακικό Ασβέστιο, Βιταμίνη C (Ασκορβικό Οξύ), Επικάλυψη Ταμπλέτας (Πολυδεξτρόζη, Υδρόξυπροπυλο Μεθυλοκυτταρίνη &amp; Ανθρακικό Ασβέστιο, Χρωστικές: Οξείδιο του Σιδήρου), Εκχύλισμα Φλοιού Κανέλλας (Cinnamomum cassia), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Βιταμίνη Ε (Όξινη ηλεκτρική dl-α-Τοκοφερόλη), Νιασίνη (Νικοτιναμίδιο), Κιτρικός Ψευδάργυρος, Σίδηρος (Φουμαρικός Σίδηρος), Μονονιτρική Θειαμίνη, Ενυδατικός Παράγοντας (Διασταυρούμενη Νατριούχος Σελλουλόζη), Παντοθενικό Οξύ (Παντοθενικό Ασβέστιο), Παρα Αμινο Βενζοϊκό Οξύ, Διτρυγική Χολίνη, Ινοσιτόλη, Ριβοφλαβίνη, Βιταμίνη Β6 (Ως 5-Φωσφορική Πυριδοξάλη), Βιταμίνη Β12 (Κυανοκοβαλαμίνη), Βιταμίνη D3 (Xοληκαλσιφερόλη), Σελήνιο (L-Σεληνομεθειονίνη &amp; Νατριούχος Σελενίτης), Πικολινικό Χρώμιο, Θειϊκό Μαγγάνιο, Θειϊκός Χαλκός, Φολικό οξύ, Βιταμίνη Κ1 (Φυλλοκινόνη), Ιωδικό Κάλιο, Βιοτίνη.</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 2 ταμπλέτες ημερησίως, κατά προτίμηση μια με το πρωινό και μια με το μεσημεριανό ή το βραδινό σας ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Μπορεί να προκληθεί κίτρινος χρωματισμός των ούρων. Αυτό είναι αβλαβές και υποδεικνύει ότι το σώμα αποβάλλει την περίσσια ποσότητα της βιταμίνης Β2 (riboflavin). Το προϊόν αυτό περιέχει σίδηρο, και η υπέρβαση της δοσολογίας μπορεί να είναι επιζήμια, ιδιαίτερα σε μικρά παιδιά. Φυλάξτε το σε σημείο ασφαλές από τα παιδιά. Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες. Να μην λαμβάνεται από άτομα που βρίσκονται υπό αγωγή με κουμαρινικά αντιπηκτικά, εκτός εάν υπάρχει αντίθετη ιατρική σύσταση.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30&amp;120tabs</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 153615/19.12.2024 | Κατηγορία lamberts.gr: Πολυβιταμίνες › Μεταβολισμός</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -3203,7 +4853,46 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής ισχύος Βιταμίνη Ε φυσικής μορφής</t>
+          <t xml:space="preserve">Με τον όρο Βιταμίνη Ε, εννοούμε μια οικογένεια λιποδιαλυτών χημικών ενώσεων με ισχυρές αντιοξειδωτικές ιδιότητες που ονομάζονται τοκοφερόλες. Οι τοκοφερόλες διακρίνονται με τα γράμματα του ελληνικού αλφαβήτου σε: α, β, γ, δ, ε, ζ και η. Η σημαντικότερη εξ αυτών είναι η α τοκοφερόλη (d-alpha-tocopherol), καθώς χαρακτηρίζεται από καλύτερη απορρόφηση και βιοδιαθεσιμότητα και με αυτή την μορφή έχει διεξαχθεί η πλειονότητα των κλινικών μελετών.
+Η βιταμίνη Ε θεωρείται ως ένα από τα σημαντικότερα διατροφικά αντιοξειδωτικά για τον άνθρωπο, συμβάλλοντας στην προστασία των κυττάρων από το οξειδωτικό στρες* . Συγκεκριμένα θεωρείται ως το κατεξοχήν μη- πολικό αντιοξειδωτικό προστατεύοντας τις κυτταρικές μεμβράνες και τις λιποπρωτεΐνες από την οξειδωτική βλάβη.
+Το σκεύασμα Vitamin E-400iu της Lamberts® παρέχει 400iu βιταμίνης Ε ανά κάψουλα. Η βιταμίνη Ε που χρησιμοποιείται είναι 100% φυσική, καθώς παράγεται από τους σπόρους του ηλιοτρόπιου υπό την μορφή ‘d’-alpha tocopherol. Η μορφή αυτή είναι πανομοιότυπη της βιταμίνης Ε που ανευρίσκεται σε διατροφικές πηγές όπως οι σπόροι και τα φυτικά έλαια.
+Επιπροσθέτως η βιταμίνη Ε περικλείεται σε εντεροδιαλυτή κάψουλα για να επιτυγχάνεται η μέγιστη δυνατή απορρόφηση από το έντερο με την έκκριση της χολής.
+Το Vitamin E-400IU όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη E (φυσική μορφή d-alpha tocopherol)
+268mg (400iu) α-ΤΕ
+Συστατικά: Φυσική μορφή Βιταμίνης Ε (d-alpha Τοκοφερόλη), Περίβλημα Κάψουλας (Γλυκερόλη, Τροποποιημένο Άμυλο, Γαλακτωματοποιητής: Καραγενάννη, Ρυθμιστής Οξύτητας: Ανθρακικό Νάτριο.</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1-2 κάψουλες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες και θυλάζουσες γυναίκες. Η Βιταμίνη Ε της Lamberts είναι φυσική βιταμίνη Ε (υπό την μορφή d-α-Τοκοφερόλης) που είναι η μορφή Βιταμίνης Ε που ανευρίσκεται σ τις τροφές. Η φυσική βιταμίνη Ε διακρίνεται από καλύτερη απορρόφηση και ισχυρότερη βιολογική δράση, εν συγκρίσει με την συνθετική Βιταμίνη Ε.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60&amp;180caps</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 47122/12.06.2013 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη E</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -3337,7 +5026,56 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Έλαιο EPA &amp; DHA από άλγη ελεγχόμενης καλλιέργειας</t>
+          <t xml:space="preserve">Το Vegan Omega 3 Oil αποτελεί συμπλήρωμα διατροφής σε μορφή ελαίου από την άλγη Schizochytrium sp. .Το Vegan Omega 3 Oil παρέχει 100mg EPA και 500mg DHA ανά 5ml ελαίου, μια ποσότητα που συμβάλλει στην φυσιολογική λειτουργία της καρδιάς και στη διατήρηση της φυσιολογικής λειτουργίας του εγκεφάλου και της φυσιολογικής όρασης*.
+Η καλλιέργεια της άλγης που χρησιμοποιούμε για την παρασκευή της συγκεκριμένης σειράς, γίνεται σε ελεγχόμενο περιβάλλον, διασφαλίζοντας την απουσία περιβαλλοντικών επιμολύνσεων στο παραγόμενο έλαιο.
+Το έλαιο του Vegan Omega 3 Oil:
+περιέχει τα Ω3 λιπαρά οξέα στην τριγλυκεριδική μορφή τους
+προστατεύεται από την οξείδωση με την προσθήκη φυσικών αντιοξειδωτικών (τοκοφερόλες και εκχύλισμα δενδρολίβανου)
+περιέχει μηδενικούς περιβαλλοντικούς ρύπους, καθώς η καλλιέργεια της άλγης για την παραγωγή του ελαίου γίνεται σε ελεγχόμενο περιβάλλον.
+Το παρόν συμπλήρωμα στοχεύει στην κάλυψη συγκεκριμένων πληθυσμιακών ομάδων όπως οι χορτοφάγοι (Vegetarians) και οι αποκλειστικά χορτοφάγοι (Vegans), οι οποίες διατρέχουν αυξημένο κίνδυνο διατροφικής έλλειψης Ω3 λιπαρών οξέων, λόγω διατροφικών περιορισμών.
+Εκτός των χορτοφάγων και των αποκλειστικά χορτοφάγων , το παρόν συμπλήρωμα μπορεί να χρησιμοποιηθεί και από άτομα με αλλεργία στο ψάρι, τα οποία διατρέχουν αυξημένο κίνδυνο διατροφικής ανεπάρκειας του EPA και του DHA.
+Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+Αρ. Πρ. Γνωστ. ΕΟΦ: 133292/12.11.2024</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά 5ml
+Έλαιο Θαλάσσιας Άλγης
+4885mg
+το οποίο παρέχει:
+EPA
+100mg
+DHA
+500mg
+Συστατικά: Έλαιο Θαλάσσιας Άλγης (έλαιο πλούσιο σε DHA &amp; EPA από την μικροάλγη Schizochytrium sp.), Γεύση Λεμονιού, Αντιοξειδωτικά (Μίγμα Φυσικών Τοκοφερολών &amp; Εκχύλισμα Δενδρολίβανου).</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Το προϊόν συνιστάται μόνο για ενήλικες. Λαμβάνετε 5ml (1 κουταλάκι του γλυκού) ημερησίως ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Έγκυες ή θηλάζουσες γυναίκες συνιστάται να λαμβάνουν 1 κάψουλα ημερησίως. Να μην λαμβάνεται από άτομα κάτω των 18 ετών.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">150ml υγρό</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατηγορία lamberts.gr: Ω - Λιπαρά Οξέα › Ω-3 Λιπαρά οξέα φυτικής προελεύσεως</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -3390,7 +5128,56 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Έλαιο EPA &amp; DHA από άλγη ελεγχόμενης καλλιέργειας</t>
+          <t xml:space="preserve">Το Vegan Omega 3 Oil αποτελεί συμπλήρωμα διατροφής σε μορφή ελαίου από την άλγη Schizochytrium sp. .Το Vegan Omega 3 Oil παρέχει 100mg EPA και 500mg DHA ανά 5ml ελαίου, μια ποσότητα που συμβάλλει στην φυσιολογική λειτουργία της καρδιάς και στη διατήρηση της φυσιολογικής λειτουργίας του εγκεφάλου και της φυσιολογικής όρασης*.
+Η καλλιέργεια της άλγης που χρησιμοποιούμε για την παρασκευή της συγκεκριμένης σειράς, γίνεται σε ελεγχόμενο περιβάλλον, διασφαλίζοντας την απουσία περιβαλλοντικών επιμολύνσεων στο παραγόμενο έλαιο.
+Το έλαιο του Vegan Omega 3 Oil:
+περιέχει τα Ω3 λιπαρά οξέα στην τριγλυκεριδική μορφή τους
+προστατεύεται από την οξείδωση με την προσθήκη φυσικών αντιοξειδωτικών (τοκοφερόλες και εκχύλισμα δενδρολίβανου)
+περιέχει μηδενικούς περιβαλλοντικούς ρύπους, καθώς η καλλιέργεια της άλγης για την παραγωγή του ελαίου γίνεται σε ελεγχόμενο περιβάλλον.
+Το παρόν συμπλήρωμα στοχεύει στην κάλυψη συγκεκριμένων πληθυσμιακών ομάδων όπως οι χορτοφάγοι (Vegetarians) και οι αποκλειστικά χορτοφάγοι (Vegans), οι οποίες διατρέχουν αυξημένο κίνδυνο διατροφικής έλλειψης Ω3 λιπαρών οξέων, λόγω διατροφικών περιορισμών.
+Εκτός των χορτοφάγων και των αποκλειστικά χορτοφάγων , το παρόν συμπλήρωμα μπορεί να χρησιμοποιηθεί και από άτομα με αλλεργία στο ψάρι, τα οποία διατρέχουν αυξημένο κίνδυνο διατροφικής ανεπάρκειας του EPA και του DHA.
+Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+Αρ. Πρ. Γνωστ. ΕΟΦ: 133292/12.11.2024</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά 5ml
+Έλαιο Θαλάσσιας Άλγης
+4885mg
+το οποίο παρέχει:
+EPA
+100mg
+DHA
+500mg
+Συστατικά: Έλαιο Θαλάσσιας Άλγης (έλαιο πλούσιο σε DHA &amp; EPA από την μικροάλγη Schizochytrium sp.), Γεύση Λεμονιού, Αντιοξειδωτικά (Μίγμα Φυσικών Τοκοφερολών &amp; Εκχύλισμα Δενδρολίβανου).</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Το προϊόν συνιστάται μόνο για ενήλικες. Λαμβάνετε 5ml (1 κουταλάκι του γλυκού) ημερησίως ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Έγκυες ή θηλάζουσες γυναίκες συνιστάται να λαμβάνουν 1 κάψουλα ημερησίως. Να μην λαμβάνεται από άτομα κάτω των 18 ετών.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">150ml υγρό</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατηγορία lamberts.gr: Ω - Λιπαρά Οξέα › Ω-3 Λιπαρά οξέα φυτικής προελεύσεως</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -3448,7 +5235,69 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ολοκληρωμένος συνδυασμός Ω3, Ω6 &amp; Ω9 Λιπαρών Οξέων</t>
+          <t xml:space="preserve">Το Omega 3-6-9 της Lamberts® αποτελεί ένα μοναδικό συμπλήρωμα διατροφής, καθώς περιέχει το σύνολο της οικογένειας των Ω λιπαρών, σε συνδυασμό με βιταμίνη D. Τόσο η πηγή προέλευσης , όσο και η συγκέντρωση των Ω λιπαρών, προσδίδουν στο Omega 3-6-9 σημαντικά συγκριτικά πλεονεκτήματα.
+Συγκεκριμένα:
+• Τα Ω-3 λιπαρά οξέα (EPA &amp; DHA), προέρχονται από ιχθυέλαιο λιπαρών ψαριών, 5πλής μοριακής απόσταξης για τη διασφάλιση της μέγιστης καθαρότητας και της δυνατότητας συνεχόμενης χορήγησης.
+• Τα Ω-6 λιπαρά (λινολεϊκό και γ-λινολενικό οξύ), προέρχονται από υψηλής καθαρότητας έλαιο σπόρων Starflower, καθώς οι σπόροι του Starflower αποτελούν την πλουσιότερη φυτική πηγή Ω-6 λιπαρών.
+• Το Ω-9 λιπαρό οξύ (ελαϊκό οξύ) προέρχεται από έξτρα παρθένο ελαιόλαδο. Σε κάθε κάψουλα περιέχεται το εντυπωσιακό ποσό των 200mg ελαϊκού οξέος, καθιστώντας το Omega 3-6-9 , ως ένα από τα ισχυρότερα σκευάσματα ,σε συγκέντρωση ελαϊκού οξέος, παγκοσμίως.
+Η διατροφική πρόσληψη των Ω λιπαρών οξέων, συνοδεύεται από πολλαπλά – βιβλιογραφικά επιβεβαιωμένα – οφέλη για την ανθρώπινη υγεία. Συγκεκριμένα, η ημερήσια πρόσληψη 250 mg DHA συμβάλλει στη διατήρηση της φυσιολογικής λειτουργίας του εγκεφάλου και της φυσιολογικής όρασης, ενώ η αθροιστική ημερήσια πρόσληψη 250 mg EPA &amp; DHA συμβάλλει στη φυσιολογική λειτουργία της καρδιάς*.
+Επιπροσθέτως, η αντικατάσταση κορεσμένων λιπαρών από ακόρεστα λιπαρά (όπως είναι το ελαϊκό) στη διατροφή συμβάλλει στη διατήρηση των φυσιολογικών επιπέδων χοληστερόλης στο αίμα *.
+Το Omega 3-6-9 ,όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Μίγμα Συμπυκνωμένου Ιχθυελαίου, Έλαιου Starflower και Ελαιόλαδου
+1200mg
+Το οποίο αποδίδει:
+Ολικά Ω-3 Λιπαρά Οξέα
+379mg
+Εκ των οποίων
+Eicosapentaenoic Acid (EPA)
+Docosahexaenoic Acid (DHA)
+196mg
+127mg
+Ολικά Ω-6 Λιπαρά Οξέα
+Εκ των οποίων
+Λινολεϊκό Οξύ
+Γ-Λινολενικό Οξύ (GLA)
+125mg
+66mg
+Ολικά Ω-9 Λιπαρά Οξέα
+Εκ των οποίων
+Ελαϊκό Οξύ
+200mg
+Βιταμίνη D
+5μg
+Συστατικά: Ιχθυέλαιο (Συμπυκνωμένο Ιχθυέλαιο* Σώματος Ψαριού 5πλής Απόσταξης, Αντιοξειδωτικά: Μικτές Τοκοφερόλες), Περίβλημα Κάψουλας (Πηκτωματοποιητές: Βόειος Ζελατίνη &amp; Γλυκερόλη), Ελαιόλαδο, Έλαιο Starflower, Βιταμίνη D3 (Χοληκαλσιφερόλη &amp; Αντιοξειδωτικά: dl-α Τοκοφερόλη).</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Μασήστε 1- 2 κάψουλες ημερησίως με το γεύμα ή σύμφωνα με τις οδηγίες του γιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Άτομα που λαμβάνουν ασπιρίνη ή από του στόματος αντιπηκτικά πρέπει να συμβουλεύονται τον ιατρό τους, προ της λήψης του Ωμέγα 3, 6 και 9.
+Αλλεργίες: Περιέχει ψάρι. ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">120caps</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 16012/10.03.2005 | Κατηγορία lamberts.gr: Ω - Λιπαρά Οξέα › Ω-3, Ω-6 &amp; Ω-9 Λιπαρά οξέα</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -3501,7 +5350,53 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Η “advance” φόρμουλα για την υγεία των οστών</t>
+          <t xml:space="preserve">Το Osteoguard ® Advance αποτελεί μια ειδικά σχεδιασμένη φόρμουλα για την οστική υγεία με ασβέστιο, μαγνήσιο, βιταμίνη D3 και βιταμίνη K2. Τα ιδιαίτερα χαρακτηριστικά στο σχεδιασμό του Osteoguard® Advance περιλαμβάνουν:
+Την επιλογή των συγκεκριμένων μικροθρεπτικών συστατικών και της συγκέντρωσης αυτών: Η επιλογή των μικροθρεπτικών συστατικών και της ποσότητας τους έγινε βάσει των ιδιοτήτων τους επί του οστικού μεταβολισμού καθώς, το ασβέστιο, το μαγνήσιο και οι βιταμίνες D &amp; K, συμβάλλουν* στην διατήρηση της φυσιολογικής κατάστασης των οστών.
+Την επιλογή των μορφών των μεταλλικών αλάτων με τις οποίες διασφαλίζεται η μέγιστη δυνατή απορρόφηση και βιοδιαθεσιμότητα: Οι μορφές αλάτων των μετάλλων του Osteoguard® Advance είναι αυτές με τις οποίες διασφαλίζεται η μέγιστη δυνατή απορρόφηση και βιοδιαθεσιμότητα . Συγκεκριμένα το άλας ασβεστίου στο παρόν σκεύασμα αποτελεί μίγμα ανθρακικού και κιτρικού ασβεστίου , ενώ το άλας μαγνησίου αποτελεί μίγμα ανθρακικού ,κιτρικού και υδροξειδίου του μαγνησίου.
+Την επιλογή της ιδανικής αναλογία ασβεστίου / μαγνησίου: Η αναλογία ασβεστίου/μαγνησίου του Osteoguard® Advance είναι 2:1, καθώς η αναλογία αυτή ενισχύει περαιτέρω την απορρόφηση του ασβεστίου από τον εντερικό βλεννογόνο.
+Όπως σε όλα τα σκευάσματα της Lamberts® που περιέχουν Κ2, η βιταμίνη Κ2 στο Osteoguard ® Advance , βρίσκεται στη φυσική της μορφή (ως μενακινόνη/ΜΚ-7) . Εν αντιθέσει με αντίστοιχα σκευάσματα του ανταγωνισμού που χρησιμοποιούν Κ2 από προερχόμενη από το νάττο (παραδοσιακό ιαπωνικό τρόφιμο που παρασκευάζεται από φασόλια σόγιας ), η Κ2 της Lamberts® παρασκευάζεται από ρεβίθια μέσω μιας ειδικής διαδικασίας ζύμωσης. Το γεγονός αυτό διασφαλίζει ότι το σκεύασμά μας δεν περιέχει ως διατροφικά αλλεργιογόνα σόγια και υποπροϊόντα γάλακτος.
+Όπως όλα τα σκευάσματα της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά 2 ταμπλέτες
+Βιταμίνη D3
+10μg
+Βιταμίνη K2
+90μg
+Ασβέστιο
+500mg
+Μαγνήσιο
+250mg
+Συστατικά: Ασβέστιο (Ανθρακικό &amp; Κιτρικό), Μαγνήσιο (Κιτρικό, Υδροξείδιο του Μαγνησίου και Ανθρακικό Μαγνήσιο), Διογκωτικοί Παράγοντες (Κυτταρίνη), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη), Βιταμίνη Κ2 ως Μενακινόνη-7 (ΜΚ-7), Επικάλυψη Ταμπλέτας (Υδροξυπροπυλο Μεθυλοκυτταρίνη &amp; Γλυκερόλη), Βιταμίνη D3 (Χοληκαλσιφερόλη).</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 2 ταμπλέτες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90tabs</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 7723/24.01.2019 | Κατηγορία lamberts.gr: Μέταλλα › Σκευάσματα &amp; Συνδυασμοί Ασβεστίου</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -3521,7 +5416,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/wp-content/uploads/2025/01/8227-90-hr.png</t>
+          <t xml:space="preserve">lamberts/osteoguard-advance-5055148412067.png</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -3559,7 +5454,69 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ηλεκτρολύτες και Υδατάνθρακες για την διάρκεια της εκγύμνασης</t>
+          <t xml:space="preserve">Το Energy Drink της Lamberts ® αποτελεί ένα μοναδικό προϊόν αθλητικής διατροφής καθώς περιέχει:
+Ηλεκτρολύτες (ανόργανα μέταλλα), όπως νάτριο, κάλιο, ασβέστιο, χλώριο, φώσφορο και μαγνήσιο για την αναπλήρωση των ηλεκτρολυτών που χάνονται μέσω της εφίδρωσης.
+Σύμπλοκους υδατάνθρακες σε μορφή πολυσακχαριτών μακράς και μέσης αλύσου, διασφαλίζοντας την παροχή ενέργειας στον οργανισμό, σταθεροποιώντας τα επίπεδα γλυκόζης του αίματος και αποτρέποντας την εξάντληση του μυϊκού γλυκογόνου κατά την διάρκεια της εκγύμνασης. Το γλυκογόνο του μυϊκού ιστού αποτελεί μια από τις πρώτες πηγές ενέργειας κατά την διάρκεια της εκγύμνασης. Ουσιαστικά πρόκειται για πολυσακχαρίτη (μόρια σακχάρου που συνδέονται μεταξύ τους) και η διάσπασή του κατά την διάρκεια της εκγύμνασης παρέχει τα ,αναγκαία για την κάλυψη των ενεργειακών αναγκών του οργανισμού, μόρια σακχάρου. Η εξάντληση των αποθεμάτων του μυϊκού γλυκογόνου συνοδεύεται από έναρξη διάσπασης των πρωτεϊνών του μυϊκού ιστού στα επιμέρους αμινοξέα, ώστε να διασφαλιστεί η κάλυψη των ενεργειακών αναγκών που συνοδεύουν την εκγύμναση, κάτι που οδηγεί στην εμφάνιση μυαλγίας και κόπωσης.
+Βιταμίνη C. Η βιταμίνη C συμβάλλει στην ενεργοποίηση του μεταβολισμού και την φυσιολογική λειτουργία του ανοσοποιητικού* κατά την διάρκεια της έντονης εκγύμνασης. Επίσης συμβάλλει την μείωση της κόπωσης που συνοδεύει έντονα προγράμματα εκγύμνασης.
+Το Energy Drink της Lamberts® μπορεί να ληφθεί:
+1.πριν και κατά την διάρκεια του προγράμματος εκγύμνασης διασφαλίζοντας την παροχή ενέργειας στον οργανισμό, αποτρέποντας την εξάντληση του μυϊκού γλυκογόνου και αναπληρώνοντας τους ηλεκτρολύτες.
+2.μετά το πέρας του προγράμματος εκγύμνασης για την αντιμετώπιση της κόπωσης (αποκατάσταση των επιπέδων του μυϊκού γλυκογόνου και των ηλεκτρολυτών).
+Όπως όλα τα σκευάσματα της Lamberts® , το Energy Drink παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+Αριθ. Πρωτ. Γνωστοποίησης ΕΟΦ: 41705/23.06.2008</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές Πληροφορίες
+Ανά 50γρ
+Ενέργεια
+732kJ/175kcal
+Υδατάνθρακες
+43,7g
+εκ των οποίων σάκχαρα
+5,5g
+Άλας
+0,246g
+Bιταμίνη C
+206mg
+Kάλιο
+294.3mg
+Χλώριο
+151.7mg
+Ασβέστιο
+87.1mg
+Φώσφορο
+160.3mg
+Μαγνήσιο
+82.6mg
+Συστατικά: Μαλτοδεξτρίνη, Αποξηραμένο Σιρόπι Γλυκόζης, Ρυθμιστής Οξύτητας (Κιτρικό Οξύ), Διφωσφορικό Κάλιο, Αρωματισμός, Χλωριούχο Νάτριο, Ανθρακικό Ασβέστιο, Βιταμίνη C (Ασκορβικό Οξύ), Φυσική Χρωστική (Βήτα Καροτένη), Κιτρικό Μαγνήσιο, Φωσφορικό Μαγνήσιο, Τεχνητό Γλυκαντικό.</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προσθέστε 50gr σκόνης σε 500ml κρύου νερού και αναδεύστε. Μπορεί να ληφθεί πριν, κατά τη διάρκεια και μετά το πέρας του προγράμματος εκγύμνασης. Μπορούν να ληφθούν έως 4 τέτοιες δόσεις ημερησίως.
+Διατηρείστε το μίγμα στο ψυγείο και καταναλώστε το μέσα σε 3 ώρες από την παρασκευή. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Αυτό το προϊόν δεν συνίσταται για παιδιά ή για εγκύους ή θηλάζουσες γυναίκες.
+Αλλεργίες: Περιέχει γάλα, σόγια και δημητριακά. Παρασκευάζεται σε εργοστάσιο που χρησιμοποιεί δημητριακά.</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1000g σκόνη</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατηγορία lamberts.gr: Αθλητική διατροφή › Ηλεκτρολύτες</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -3698,7 +5655,50 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Έλαιο Νυχτολούλουδου των 500mg με προσθήκη Βιταμίνης Ε</t>
+          <t xml:space="preserve">Το έλαιο νυχτολούλουδου (Evening Primrose Oil ) αποτελεί μία από τις ελάχιστες φυσικές πηγές γ-λινολεϊκού οξέος (GLA). Το GLA αποτελεί πολυακόρεστο Ω-6 λιπαρό οξύ, με ευρείες βιολογικές δράσεις που προκύπτουν από το ότι αποτελεί πρόδρομο μόριο της προσταγλανδίνης PGE1. Αν και ο οργανισμός μπορεί να συνθέσει GLA, πολλές φορές αυτό δεν αρκεί και απαιτείται διατροφική πρόσληψη.
+Το GLA συνιστάται συχνά σε γυναίκες κατά τη διάρκεια της εμμήνου ρήσεως και κατά τη διάρκεια της εμμηνόπαυσης.
+To Pure Evening Primrose Oil 500mg αποτελεί ένα υψηλής ισχύος και καθαρότητας σκεύασμα ελαίου νυχτολούλουδου το οποίο παρέχει 50mg GLA ανά κάψουλα.
+Το έλαιο που χρησιμοποιείται είναι προσεκτικά επιλεγμένο με βάση την καθαρότητα του και την περιεκτικότητα σε GLA. Επιπροσθέτως, παρέχει μια εξαιρετική ποσότητα βιταμίνης Ε, η οποία συμβάλλει στην προστασία των κυττάρων από το οξειδωτικό στρες*.
+Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη Ε
+10mg
+Έλαιο Νυχτολούλουδου
+500mg
+Γ-Λινολενικό Οξύ (GLA)
+50mg
+Συστατικά: Έλαιο Νυχτολούλουδου, Περίβλημα Κάψουλας (Τροποποιημένο Άμυλο, Γλυκερόλη Πηκτωματοποιητής: Καραγεννάνη), Βιταμίνη Ε (Οξεϊκή dl-α-τοκοφερόλη).</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Μασήστε 1- 4 κάψουλες ημερησίως με το γεύμα ή σύμφωνα με τις οδηγίες του γιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Άτομα που πάσχουν από επιληψία πρέπει να συμβουλεύονται τον Ιατρό τους πρίν την λήψη του συγκεκριμένου συμπληρώματος.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">180caps</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 4629/20.01.2017 | Κατηγορία lamberts.gr: Ω - Λιπαρά Οξέα › Ω-6 Λιπαρά οξέα</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -3756,7 +5756,52 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ιχθυέλαιο 5πλής μοριακής απόσταξης των 1100mg</t>
+          <t xml:space="preserve">Το Pure Fish Oil 1100mg της Lamberts® αποτελεί ένα υψηλής ισχύος και καθαρότητας σκεύασμα ιχθυελαίου, το οποίο παρέχει 700mg Ω-3 λιπαρών οξέων ανά κάψουλα. Το γεγονός αυτό καθιστά το Pure Fish Oil 1100mg ως ένα από τα υψηλότερης ισχύος σκευάσματα ιχθυελαίων, κάτι που αντικατοπτρίζεται στις προτιμήσεις των Επαγγελματιών Υγείας.
+Επιπροσθέτως, η συνιστώμενη ημερήσια δόση κυμαίνεται από 1-3 κάψουλες, επιτρέποντας στον Επαγγελματία της Υγείας την εξατομίκευση της αγωγής αναλόγως του επιθυμητού επιπέδου EPA &amp; DHA.
+Όπως όλα τα ιχθυέλαια της Lamberts® , το ιχθυέλαιο που χρησιμοποιείται στο Pure Fish Oil 1100mg είναι 5πλής μοριακής απόσταξης για την διασφάλιση της μέγιστης καθαρότητας και τη δυνατότητα μακροχρόνιας χορήγησης και παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+Η προστασία του ελαίου εντός της κάψουλας από την οξείδωση, επιτυγχάνεται χάρη στην προσθήκη φυσικής βιταμίνης Ε.</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Συμπυκνωμένο Ιχθυέλαιο σώματος ψαριού
+1100mg
+Το οποίο αποδίδει Ολικά Ω3
+700mg
+Εκ των οποίων:
+Eicosapentaenoic Acid (EPA)
+355mg
+Docosahexaenoic Acid (DHA)
+237mg
+Συστατικά: Ιχθυέλαιο (Συμπυκνωμένο Ιχθυέλαιο σώματος ψαριού 5πλής απόσταξης, Αντιοξειδωτικό: Μικτές Τοκοφερόλες), Περίβλημα Κάψουλας (Ζελατίνη (Βοδινή), Γλυκερόλη).</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1-3 κάψουλες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Άτομα που λαμβάνουν ασπιρίνη ή από του στόματος αντιπηκτικά πρέπει να συμβουλεύονται τον ιατρό τους, προ της λήψης του Pure Fish Oil.
+Αλλεργίες: Περιέχει ψάρι. ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60, 120&amp;180caps</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 16012/10.03.2005 | Κατηγορία lamberts.gr: Ω - Λιπαρά Οξέα › Ω-3 Λιπαρά οξέα από ψάρι</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -3814,7 +5859,52 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ιχθυέλαιο 5πλής μοριακής απόσταξης των 1100mg</t>
+          <t xml:space="preserve">Το Pure Fish Oil 1100mg της Lamberts® αποτελεί ένα υψηλής ισχύος και καθαρότητας σκεύασμα ιχθυελαίου, το οποίο παρέχει 700mg Ω-3 λιπαρών οξέων ανά κάψουλα. Το γεγονός αυτό καθιστά το Pure Fish Oil 1100mg ως ένα από τα υψηλότερης ισχύος σκευάσματα ιχθυελαίων, κάτι που αντικατοπτρίζεται στις προτιμήσεις των Επαγγελματιών Υγείας.
+Επιπροσθέτως, η συνιστώμενη ημερήσια δόση κυμαίνεται από 1-3 κάψουλες, επιτρέποντας στον Επαγγελματία της Υγείας την εξατομίκευση της αγωγής αναλόγως του επιθυμητού επιπέδου EPA &amp; DHA.
+Όπως όλα τα ιχθυέλαια της Lamberts® , το ιχθυέλαιο που χρησιμοποιείται στο Pure Fish Oil 1100mg είναι 5πλής μοριακής απόσταξης για την διασφάλιση της μέγιστης καθαρότητας και τη δυνατότητα μακροχρόνιας χορήγησης και παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+Η προστασία του ελαίου εντός της κάψουλας από την οξείδωση, επιτυγχάνεται χάρη στην προσθήκη φυσικής βιταμίνης Ε.</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Συμπυκνωμένο Ιχθυέλαιο σώματος ψαριού
+1100mg
+Το οποίο αποδίδει Ολικά Ω3
+700mg
+Εκ των οποίων:
+Eicosapentaenoic Acid (EPA)
+355mg
+Docosahexaenoic Acid (DHA)
+237mg
+Συστατικά: Ιχθυέλαιο (Συμπυκνωμένο Ιχθυέλαιο σώματος ψαριού 5πλής απόσταξης, Αντιοξειδωτικό: Μικτές Τοκοφερόλες), Περίβλημα Κάψουλας (Ζελατίνη (Βοδινή), Γλυκερόλη).</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1-3 κάψουλες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Άτομα που λαμβάνουν ασπιρίνη ή από του στόματος αντιπηκτικά πρέπει να συμβουλεύονται τον ιατρό τους, προ της λήψης του Pure Fish Oil.
+Αλλεργίες: Περιέχει ψάρι. ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60, 120&amp;180caps</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 16012/10.03.2005 | Κατηγορία lamberts.gr: Ω - Λιπαρά Οξέα › Ω-3 Λιπαρά οξέα από ψάρι</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -3953,7 +6043,48 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής ισχύος τιτλοδοτημένο εκχύλισμα καρπών Αγριοτριανταφυλλιάς</t>
+          <t xml:space="preserve">Οι καρποί αγριοτριανταφυλλιάς (Rosa canina,Rose hips) αποτελούν μια από τις πλουσιότερες φυσικές πηγές βιταμίνης C. Ως εκ τούτου αποτελούν μια από τις πιο ισχυρές αντιοξειδωτικές φυτικές πηγές, καθότι η βιταμίνη C συμβάλλει στην προστασία των κυττάρων από το οξειδωτικό στρες και στην αναγέννηση της ανηγμένης μορφής της βιταμίνης Ε*. Για τον λόγο αυτό ως δείκτης τιτλοδότησης των εκχυλισμάτων αγριοτριανταφυλλιάς χρησιμοποιείται η συγκέντρωση της βιταμίνης C.
+Το Rosehip 10.000mg της Lamberts® αποτελεί ένα από τα υψηλότερης ισχύος τιτλοδοτημένα εκχυλίσματα καρπών αγριοτριανταφυλλιάς παγκοσμίως. Κάθε ταμπλέτα παρέχει 500mg τιτλοδοτημένου εκχυλίσματος, ισοδύναμου με 10.000 mg αποξηραμένων καρπών αγριοτριανταφυλλιάς, το οποίο αποδίδει 250mg φυσικής βιταμίνης C. Το επίπεδο αυτό συμβαδίζει απόλυτα με το επίπεδο που χρησιμοποιήθηκε σε δημοσιευμένες μελέτες.
+Όπως όλα τα σκευάσματα της Lamberts®, το Rosehip 10.000mg παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Καρποί Αγριοτριανταφυλλιάς
+(ως 500 mg τιτλοδοτημένου εκχυλίσματος (20:1))
+10.000mg
+Το οποίο αποδίδει:
+Βιταμίνη C
+250mg
+Συστατικά: Διογκωτικοί Παράγοντες (Ανθρακικό Ασβέστιο &amp; Κυτταρίνη), Τιτλοδοτημένο Εκχύλισμα Καρπών Αγριοτριανταφυλλιάς (Rosa canina) (Ασκορβικό Οξύ, Φυσικό Εκχύλισμα Καρπών Αγριοτριανταφυλλιάς), Επικάλυψη Ταμπλέτας (Στιλβωτικοί Παράγοντες: Ανθρακικό Ασβέστιο &amp; Ισομάλτη, Χρωστικές: Οξείδιο του Σιδήρου, Υδρόξυπροπυλο Μεθυλοκυτταρίνη), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη).</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60tabs</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 26977/23.03.2016 | Κατηγορία lamberts.gr: Βότανα › Αντιοξειδωτικά Βότανα</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -4006,7 +6137,52 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Σελήνιο των 200μg &amp; αντιοξειδωτικές Βιταμίνες A, C &amp; E</t>
+          <t xml:space="preserve">Το σελήνιο αποτελεί ένα από τα σημαντικότερα μικροθρεπτικά συστατικά με ευρύ φάσμα βιολογικών δράσεων που περιλαμβάνουν τη συμβολή του στη φυσιολογική σπερματογένεση, στη φυσιολογική θυρεοειδική λειτουργία ,στη διατήρηση της φυσιολογικής κατάστασης των μαλλιών και των νυχιών, στη φυσιολογική λειτουργία του ανοσοποιητικού συστήματος, και στην προστασία των κυττάρων από το οξειδωτικό στρες*.
+Παρά το σημαντικό του ρόλο ωστόσο, η σύγχρονη διατροφική πρόσληψη σεληνίου είναι ανεπαρκής.
+Το Selenium 200μg A+C+E, αποτελεί ένα υψηλής ισχύος σκεύασμα σεληνίου, το οποίο ανά ταμπλέτα παρέχει 200μg στοιχειακού σεληνίου σε συνδυασμό με υψηλές ποσότητες βιταμινών Α ,C και Ε.
+Όπως το σελήνιο, έτσι και οι βιταμίνες Α, C και Ε, είναι γνωστές για τις αντιοξειδωτικές τους ιδιότητες, καθώς συμβάλλουν στην προστασία των κυττάρων από το οξειδωτικό στρες*.
+Όπως όλα τα σκευάσματα της Lamberts® ,το Selenium 200μg A+C+E παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Βιταμίνη A
+400μg RE
+Βιταμίνη E
+24mg
+Βιταμίνη C
+80mg
+Σελήνιο
+200μg
+Συστατικά: Διογκωτικοί Παράγοντες (Φωσφορικό Διασβέστιο &amp; Κυτταρίνη), Βιταμίνη C (Ασκορβικό Οξύ), Βιταμίνη Ε (Οξεική dl-a Ττοκοφερόλη), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη), Οξεική Βιταμίνη Α, Σελήνιο (L-Σεληνομεθειονίνη &amp; Νατριούχο Σελήνιο).</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Το προϊόν περιέχει βιταμίνη Α. Να μην λαμβάνεται από έγκυους ή θηλάζουσες ή γυναίκες με πιθανότητα εγκυμοσύνης.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100tabs</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 93182/05.12.2013 | Κατηγορία lamberts.gr: Μέταλλα › Σελήνιο</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -4112,7 +6288,47 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής ισχύος Συνένζυμο Q10 αυξημένης απορρόφησης</t>
+          <t xml:space="preserve">Το συνένζυμο Q10 αποτελεί ουσία που μοιάζει με βιταμίνη και βρίσκεται στα μιτοχόνδρια του συνόλου των κυττάρων του ανθρώπινου οργανισμού. Εκεί αποτελεί απαραίτητο συστατικό της μιτοχονδριακής αλυσίδας μεταφοράς ηλεκτρονίων (αναπνευστική άλυσος), συμβάλλοντας στην παραγωγή κυτταρικής ενέργειας.
+Καθώς διαδραματίζει σημαντικό ρόλο στην παραγωγή ενέργειας, οι συγκεντρώσεις του συνενζύμου Q10 είναι υψηλότερες σε όργανα με υψηλές ενεργειακές απαιτήσεις (όπως η καρδιά, οι μύες, ο εγκέφαλος, το ήπαρ και οι πνεύμονες). Η αύξηση της ηλικίας και η χρήση φαρμάκων, όπως οι στατίνες μειώνουν την παραγωγή συνενζύμου Q10 από τον οργανισμό.
+Το Co-Enzyme Q10 100mg της Lamberts® παρέχει εγγυημένα 100mg συνενζύμου Q10 ανά κάψουλα.
+Το συνένζυμο ανευρίσκεται σε ελαιώδες εναιώρημα και εσωκλείεται σε εντεροδιαλυτή κάψουλα, καθώς αυτή αποτελεί την φαρμακοτεχνική μορφή με την βέλτιστη απορρόφηση και βιοδιαθεσιμότητα*.
+Όπως όλα τα σκευάσματα της Lamberts® παρασκευάζονται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+* Pepping J. Co Enzyme Q10 Am. Health Syst. Pharm 1999; 56:519-521</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Συνένζυμο Q10 (Ουμπικινόνη)
+100mg
+Συστατικά: Έλαιο ηλιόσπορου, Περίβλημα Κάψουλας (Ζελατίνη, Γλυκερόλη, Χρωστικές : Οξείδιο του Σιδήρου, Συνένζυμο Q10,Λεκιθίνη Ηλίανθου, Μονοστεαρική Γλυκερόλη.</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30&amp;60caps</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 22932/12.04.2005 | Κατηγορία lamberts.gr: Συνένζυμο Q10 και Ουμπικινόλη</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -4218,7 +6434,47 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Κουρκουμίνη ταχείας αποδέσμευσης για άμεση απορρόφηση</t>
+          <t xml:space="preserve">Το Turmeric Fast Release αποτελεί ένα υψηλής ισχύος τιτλοδοτημένο εκχύλισμα ρίζας κουρκουμά, που παρέχει 95% κουρκουμίνη, ένα ποσοστό που αντιστοιχεί σε αυτό που έχει χρησιμοποιηθεί στην πλειονότητα των δημοσιευμένων κλινικών ερευνών.
+Κάθε ταμπλέτα περιέχει 200mg τιτλοδοτημένου εκχυλίσματος ρίζας κουρκουμά (αποδίδει εγγυημένα 95% κουρκουμινοειδών) που ισοδυναμεί με 10.000mg σκόνης του μπαχαρικού.
+Οι ταμπλέτες είναι ταχείας αποδέσμευσης διασφαλίζοντας άμεση απελευθέρωση και απορρόφηση της κουρκουμίνης (εντός 15-30 λεπτών από την κατάποση).
+Η επιλογή της πρώτης ύλης του κουρκουμά, γίνεται με βάση διεθνείς κατευθυντήριες οδηγίες που αφορούν στην καθαρότητα του και στην απουσία περιβαλλοντικών ρύπων. Συγκεκριμένα , εφαρμόζεται μια εξειδικευμένη διαδικασία 10 διαφορετικών σταδίων ποιοτικού ελέγχου, διασφαλίζοντας την απουσία τόσο περιβαλλοντικών επιμολύνσεων όσο και την απουσία μικροβιολογικής επιμόλυνσης από βακτήρια και μύκητες.
+Το Turmeric Fast Release όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Τιτλοδοτημένο εκχύλισμα Ριζώματος Κουρκουμά
+(Ισοδύναμο με 10.000mg Ρίζας Κουρκουμά – Αποδίδοντας 95% κουρκουμινοειδή)
+200mg
+Συστατικά: Διογκωτικοί Παράγοντες (Κυτταρίνη &amp; Ανθρακικό Ασβέστιο), Τιτλοδοτημένο Εκχύλισμα Ριζώματος Κουρκουμά (Curcuma longa), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ και Στεατικό Μαγνήσιο), Επικάλυψη Tαμπλέτας (Υδροξυπρόπυλο-μεθυλοκυτταρίνη και Γλυκερόλη), Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη).</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες. Δεν συνίσταται για άτομα κάτω των 18 ετών.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60&amp;120tabs</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 7722/24.01.2019 | Κατηγορία lamberts.gr: Βότανα › Σκευάσματα Κουρκουμά</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -4304,7 +6560,68 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής ισχύος σύμπλεγμα Βιταμινών Β</t>
+          <t xml:space="preserve">Το B-100 Complex της Lamberts® αποτελεί ένα ολοκληρωμένο, εξαιρετικά υψηλής ισχύος σύμπλεγμα βιταμινών Β. Περιέχει το σύνολο των βιταμινών Β σε υψηλές ποσότητες σε συνδυασμό με χολίνη, ινοσιτόλη και PABA (π-αμινοβουτυρικό οξύ).
+Το B-100 Complex της Lamberts® συνιστάται:
+σε περιπτώσεις που απαιτείται ταχεία βελτίωση στην πρόσληψη των βιταμινών Β
+σε άτομα με υψηλές ανάγκες σε βιταμίνες Β
+και σε άτομα που ακολουθούν μακροχρονίως διατροφή ανεπαρκή σε βιταμίνες Β.
+Όπως όλα τα σκευάσματα της Lamberts® , το Neuro-Guard της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές Πληροφορίες
+Aνά ταμπλέτα
+Θειαμίνη (B1)
+100mg
+Ριβοφλαβίνη (B2)
+100mg
+Νιασίνη (B3)
+100mg NE
+Βιταμίνη B6
+10mg
+Φολικό Οξύ
+400μg
+Βιταμίνη B12
+100μg
+Βιοτίνη
+100μg
+Παντοθενικό Οξύ (Β5)
+100mg
+Διτρυγική Χολίνη
+100mg
+Μυο-Ινοσιτόλη
+100mg
+PABA
+30mg
+Συστατικά: Διογκωτικός Παράγοντας (Κυτταρίνη &amp; Φωσφορικό Διασβέστιο), Μονονιτρική Θειαμίνη, Παντοθενικό Οξύ (Παντοθενικό Ασβέστιο), Ινοσιτόλη, Ριβοφλαβίνη, Νιασίνη (Νικοτιναμίδιο), Διτρυγική Χολίνη, Υδρόξυπροπυλο Κυτταρίνη, Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Παρα Αμινοβενζοϊκό Οξύ, Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη), Επικάλυψη Ταμπλέτας (Υδρόξυπροπυλο Μεθυλοκυτταρίνη, Γλυκερόλη), Βιταμίνη Β6 (Υδροχλωρική Πυριδοξίνη), Φολικό οξύ, Βιταμίνη Β12 (Μεθυλοκοβαλαμίνη), Βιοτίνη.</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς,
+ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60&amp;200tabs</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 47121/12.06.2013 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνες B</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
@@ -4454,7 +6771,48 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Μη όξινη μορφή Βιταμίνης C</t>
+          <t xml:space="preserve">Η λήψη μεγάλων δόσεων βιταμίνης C μπορεί να προκαλέσει ήπιες γαστρεντερικές διαταραχές, λόγω της όξινης φύσης του ασκορβικού οξέος . Η πιθανότητα αυτή αυξάνεται σε άτομα με ιστορικό γαστρεντερικών διαταραχών.
+Σε περιπτώσεις όπου κρίνεται αναγκαία η χορήγηση υψηλών δόσεων βιταμίνης C, ή /και η χορήγηση βιταμίνης C σε άτομα με ατομικό αναμνηστικό γαστρεντερικών διαταραχών συνιστούμε τη Gentle Vitamin C των 500mg. Το προϊόν αυτό παρέχει βιταμίνη C σε μορφή ασκορβικού ασβεστίου (calcium ascorbate), μία μη όξινη και πλήρως απορροφήσιμη μορφή βιταμίνης C.
+Με τη χρήση του συγκεκριμένου σκευάσματος μπορούν να ληφθούν μέχρι 2gr βιταμίνης C ημερησίως (4 ταμπλέτες). Σε αυτές τις περιπτώσεις συνιστούμε τη λήψη των απαιτούμενων ταμπλετών σε διαφορετικές ώρες κατά τη διάρκεια της ημέρας.
+Κάθε ταμπλέτα παρέχει επίσης 77mg ασβεστίου γεγονός που μπορεί να συνεισφέρει σημαντικά στη πρόσληψη ασβεστίου, ειδικότερα σε περιπτώσεις ημερήσιας λήψης μεγάλου αριθμού ταμπλετών.
+Όπως όλα τα σκευάσματα της Lamberts® ,η Gentle Vitamin C 500mg παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Βιταμίνη C
+500mg
+Ασβέστιο
+77mg
+Συστατικά: Ασκορβικό Ασβέστιο (αποδίδει Βιταμίνη C και Ασβέστιο), Διογκωτικός Παράγοντας (Κυτταρίνη &amp; Ανθρακικό Ασβέστιο), Παράγοντες Aντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Μαγνήσιο &amp; Στεατικό Οξύ), Τροποποιημένο Άμυλο, Σταθεροποιητής (Υδρόξυπρόπυλο Κυτταρίνη), Επικάλυψη Ταμπλέτας (Υδρόξυπρόπυλο Μέθυλοκυτταρίνη, Γλυκερόλη).</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1-4 ταμπλέτες, ημερησίως με το γεύμα, ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Πρόσληψη άνω των 1000mg Βιταμίνης C ημερησίως μπορεί να προκαλέσει ήπιες γαστρεντερικές διαταραχές.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100tabs</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 27750/28.03.2016 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη C</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -4507,7 +6865,47 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Φολικό οξύ σε one-a-day φόρμουλα</t>
+          <t xml:space="preserve">Το φολικό οξύ (ή βιταμίνη Β9) αποτελεί την ένατη βιταμίνη του συμπλέγματος Β. Αποτελώντας υδατοδιαλυτή βιταμίνη δεν αποθηκεύεται για μεγάλο χρονικό διάστημα στον οργανισμό, γεγονός που καθιστά αναγκαία την καθημερινή διατροφική του πρόσληψη.
+Ο σημαντικότερος βιολογικός ρόλος του φολικού οξέος είναι η συμμετοχή του στην σύνθεση του DNA και του RNA , διαδραματίζοντας με τον τρόπο αυτό καθοριστικό ρόλο στην κυτταρική διαίρεση*. Για τον λόγο αυτό είναι ιδιαίτερα σημαντικό για την φυσιολογική αιμοποίηση και την ανάπτυξη του μητρικού ιστού κατά την διάρκεια της κύησης*.
+Η συμβολή του φολικού οξέος στην ανάπτυξη του μητρικού ιστού φαίνεται από το ότι η λήψη 400μg φολικού οξέος κατά την διάρκεια του πρώτου τριμήνου της κύησης, είναι αναγκαία για την πρόληψη εμφάνισης δυσπλασιών του νευρικού σωλήνα.
+Το παρόν συμπλήρωμα διατροφής παρέχει 400μg φολικού οξέος ανά ταμπλέτα, μια ποσότητα που είναι 3 φορές υψηλότερη αυτής που παρέχει μια μέση δίαιτα και αποτελεί την ποσότητα που συνιστάται συχνότερα από τους Επαγγελματίας της Υγείας.
+Όπως όλα τα σκευάσματα της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+*(ΕΕ) αριθ. 432/2012</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Φολικό Οξύ
+400μg
+Συστατικά: Φωσφορικό Διασβέστιο, Κυτταρίνη, Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Φολικό Οξύ.</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100tabs</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 30053/15.09.1998 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνες B</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -4608,7 +7006,65 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Πλήρες σύμπλεγμα Βιταμινών Β</t>
+          <t xml:space="preserve">Το B-50 Complex της Lamberts® αποτελεί ένα ολοκληρωμένο, υψηλής ισχύος σύμπλεγμα βιταμινών Β. Περιέχει το σύνολο των βιταμινών Β σε υψηλές ποσότητες σε συνδυασμό με χολίνη, ινοσιτόλη και PABA (π-αμινοβουτυρικό οξύ).
+Mπορεί να χρησιμοποιηθεί για μεγάλο χρονικό διάστημα, διασφαλίζοντας την πλήρη κάλυψη του οργανισμού σε βιταμίνες του συμπλέγματος Β.
+Σε ανεξάρτητη συγκριτική μελέτη που διεξήχθη στο Ηνωμένο Βασίλειο ,η οποία αξιολόγησε την ποιότητα σκευασμάτων του συμπλέγματος Β , το B-50 Complex της Lamberts® απέσπασε την υψηλότερη βαθμολογία (5 αστέρια/ Proof, March 2003).
+Όπως όλα τα σκευάσματα της Lamberts® , το Vitamin B-50 Complex παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Θειαμίνη (Β1)
+50mg
+Ριβοφλαβίνη (B2)
+50mg
+Νιασίνη (B3)
+50mg NE
+Βιταμίνη B6
+5mg
+Φολικό Οξύ
+400μg
+Βιταμίνη B12
+50μg
+Βιοτίνη
+50μg
+Παντοθενικό Οξύ (Β5)
+50mg
+Ινοσιτόλη
+50mg
+Διτρυγική Χολίνη
+50mg
+PABA
+15mg
+Συστατικά: Διογκωτικός Παράγοντας (Κυτταρίνη), Ανθρακικό Ασβέστιο, Μονονιτρική Θειαμίνη, Παντοθενικό Οξύ (Παντοθενικό Ασβέστιο), Ινοσιτόλη, Ριβοφλαβίνη, Νιασίνη (Νικοτιναμίδιο), Διτρυγική Χολίνη, Παράγοντες Αντισυσσωμάτωσης (Στεατικό Οξύ, Διοξείδιο του Πυριτίου &amp; Στεατικό Μαγνήσιο), Παρά Αμινό Βενζοϊκό Οξύ, Στιλβωτικοί Παράγοντες (Υδροξυπροπυλο Μεθυλοκυτταρίνη, Γλυκερόλη), Βιταμίνη Β6 (Υδροχλωρική Πυριδοξίνη), Φολικό Οξύ, Βιταμίνη Β12 (Μεθυλοκοβαλαμίνη), Βιοτίνη.</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60 &amp; 120tabs</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 54111/4.10.2004 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνες B</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -4666,7 +7122,51 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη C των 1000mg, ελεγχόμενης αποδέσμευσης</t>
+          <t xml:space="preserve">Ο ιδανικός τρόπος πρόσληψης της βιταμίνης C είναι σε μικρές ποσότητες συνεχόμενα κατά τη διάρκεια όλου του εικοσιτετραώρου. Ωστόσο, όπως είναι προφανές, κάτι τέτοιο είναι φύσει αδύνατον. Για την επίλυση του προβλήματος αυτού η Lamberts® δημιούργησε τις ταμπλέτες Βιταμίνης C Time Release (βαθμιαίας αποδέσμευσης).
+Οι ταμπλέτες παράγονται με μία εξειδικευμένη διαδικασία, η οποία ενσωματώνει τα θρεπτικά στοιχεία σε μικροσφαιρίδια, επιτρέποντάς την σταδιακή απελευθέρωση τους κατόπιν της κατάποσης. Με τον τρόπο αυτό επιτυγχάνεται η σταδιακή και συνεχόμενη απορρόφηση της βιταμίνης C η οποία διαρκεί για περίπου 6 με 8 ώρες .
+Εκτός αυτού η βιταμίνη C βαθμιαίας αποδέσμευσης της Lamberts® περιέχει και μία σημαντική ποσότητα βιοφλαβονοειδών τα οποία συμβάλλουν στην απορρόφησή της από τον οργανισμό. Τα βιοφλαβονοειδή που περιέχονται στο συγκεκριμένο σκεύασμα περιλαμβάνουν ρουτίνη, κερσετίνη, σιτρίνη και εσπεριδίνη.
+Οι ταμπλέτες Βιταμίνης C Time Release κυκλοφορούν σε 3 διαφορετικές περιεκτικότητες, των 500 mg , 1000 mg και 1500mg, για την κάλυψη διαφορετικών αναγκών και την δυνατότητα εξατομίκευσης της αγωγής.
+Το παρόν σκεύασμα παρέχει 1000mg Βιταμίνης C σε ταμπλέτα βαθμιαίας αποδέσμευσης και όπως όλα τα σκευάσματα της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Βιταμίνη C
+1000mg
+Σκόνη καρπών Αγριοτριανταφυλλιάς
+(ως τιτλοδοτημένο εκχύλισμα (4:1))
+50mg
+Σύμπλεγμα Φλαβονοειδών Κίτρου
+50mg
+Συστατικά: Βιταμίνη C (Ασκορβικό Οξύ), Υδροξυπρόπυλο Μεθυλοκυτταρίνη, Φωσφορικό Διασβέστιο, Παράγοντες αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Μαγνήσιο &amp; Στεατικό Οξύ), Σύμπλεγμα Φλαβονοειδών Κίτρου, Επικάλυψη ταμπλέτας (Υδροξυπρόπυλο Μεθυλοκυτταρίνη, Στιλβωτικοί Παράγοντες: Πολυδεξτρόζη &amp; Ανθρακικό Ασβέστιο, Χρωστικές: Οξείδιο του Σιδήρου), Γλυκερόλη, Εκχύλισμα Καρπών Αγριοτριανταφυλλιάς (Rosa canina L.).</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα, ανά 6 ώρες, με μέγιστη δόση 2 ταμπλετών ημερησίως ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Πρόσληψη άνω των 1000mg Βιταμίνης C ημερησίως μπορεί να προκαλέσει ήπιες γαστρεντερικές διαταραχές.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30,60&amp;180tabs</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 14346/28.02.2007 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη C</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
@@ -4719,7 +7219,51 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη C των 1000mg, ελεγχόμενης αποδέσμευσης</t>
+          <t xml:space="preserve">Ο ιδανικός τρόπος πρόσληψης της βιταμίνης C είναι σε μικρές ποσότητες συνεχόμενα κατά τη διάρκεια όλου του εικοσιτετραώρου. Ωστόσο, όπως είναι προφανές, κάτι τέτοιο είναι φύσει αδύνατον. Για την επίλυση του προβλήματος αυτού η Lamberts® δημιούργησε τις ταμπλέτες Βιταμίνης C Time Release (βαθμιαίας αποδέσμευσης).
+Οι ταμπλέτες παράγονται με μία εξειδικευμένη διαδικασία, η οποία ενσωματώνει τα θρεπτικά στοιχεία σε μικροσφαιρίδια, επιτρέποντάς την σταδιακή απελευθέρωση τους κατόπιν της κατάποσης. Με τον τρόπο αυτό επιτυγχάνεται η σταδιακή και συνεχόμενη απορρόφηση της βιταμίνης C η οποία διαρκεί για περίπου 6 με 8 ώρες .
+Εκτός αυτού η βιταμίνη C βαθμιαίας αποδέσμευσης της Lamberts® περιέχει και μία σημαντική ποσότητα βιοφλαβονοειδών τα οποία συμβάλλουν στην απορρόφησή της από τον οργανισμό. Τα βιοφλαβονοειδή που περιέχονται στο συγκεκριμένο σκεύασμα περιλαμβάνουν ρουτίνη, κερσετίνη, σιτρίνη και εσπεριδίνη.
+Οι ταμπλέτες Βιταμίνης C Time Release κυκλοφορούν σε 3 διαφορετικές περιεκτικότητες, των 500 mg , 1000 mg και 1500mg, για την κάλυψη διαφορετικών αναγκών και την δυνατότητα εξατομίκευσης της αγωγής.
+Το παρόν σκεύασμα παρέχει 1000mg Βιταμίνης C σε ταμπλέτα βαθμιαίας αποδέσμευσης και όπως όλα τα σκευάσματα της Lamberts® παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Βιταμίνη C
+1000mg
+Σκόνη καρπών Αγριοτριανταφυλλιάς
+(ως τιτλοδοτημένο εκχύλισμα (4:1))
+50mg
+Σύμπλεγμα Φλαβονοειδών Κίτρου
+50mg
+Συστατικά: Βιταμίνη C (Ασκορβικό Οξύ), Υδροξυπρόπυλο Μεθυλοκυτταρίνη, Φωσφορικό Διασβέστιο, Παράγοντες αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Μαγνήσιο &amp; Στεατικό Οξύ), Σύμπλεγμα Φλαβονοειδών Κίτρου, Επικάλυψη ταμπλέτας (Υδροξυπρόπυλο Μεθυλοκυτταρίνη, Στιλβωτικοί Παράγοντες: Πολυδεξτρόζη &amp; Ανθρακικό Ασβέστιο, Χρωστικές: Οξείδιο του Σιδήρου), Γλυκερόλη, Εκχύλισμα Καρπών Αγριοτριανταφυλλιάς (Rosa canina L.).</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα, ανά 6 ώρες, με μέγιστη δόση 2 ταμπλετών ημερησίως ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Πρόσληψη άνω των 1000mg Βιταμίνης C ημερησίως μπορεί να προκαλέσει ήπιες γαστρεντερικές διαταραχές.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30,60&amp;180tabs</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 14346/28.02.2007 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη C</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
@@ -4772,7 +7316,45 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής ισχύος αναβράζοντα δισκία Βιταμίνης C</t>
+          <t xml:space="preserve">Τα αναβράζοντα δισκία βιταμίνης C των 1000mg της Lamberts® αποτελούν ένα εύκολο τρόπο λήψης βιταμίνης C, ιδιαίτερα από άτομα που δυσκολεύονται να καταπιούν μεγάλες ταμπλέτες, όπως οι έφηβοι και οι ηλικιωμένοι.
+Το συγκεκριμένο σκεύασμα έχει ευχάριστη γεύση πορτοκάλι και δεν περιέχει ζάχαρη.
+Όπως όλα τα σκευάσματα της Lamberts, παρασκευάζεται σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
+Αριθ. Πρωτ. Γνωστοποίησης ΕΟΦ: 93183/05.12.2013</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά δισκίο
+Βιταμίνη C
+1000mg
+Συστατικά: Κιτρικό Οξύ, Βιταμίνη C (Ασκορβικό Οξύ), Ρυθμιστές Οξύτητας (Διττανθρακικό Νάτριο &amp; Ανθρακικό Νάτριο), Υγραντικό (Σορβιτόλη), Ινουλίνη, Άμυλο, Φωσφορικό Τριασβέστιο, Ενισχυτικό Γεύσης, Γλυκαντικός Παράγοντας (Σουκραλόζη), Μαλτοδεξτρίνη, Χρωστικές (Κόκκινο Παντζάρι και Ριβοφλαβίνη).</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 δισκίο ημερησίως (διαλυμένο σε ένα ποτήρι νερό) με το γεύμα ή σύμφωνα με τη σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Πρόσληψη άνω των 1000mg Βιταμίνης C ημερησίως μπορεί να προκαλέσει ήπιες γαστρεντερικές διαταραχές.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20 δισκία</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη C</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
@@ -4825,7 +7407,47 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 2000iu</t>
+          <t xml:space="preserve">Την τελευταία εικοσαετία, η βιταμίνη D έχει επανέλθει δυναμικά στο προσκήνιο του επιστημονικού ενδιαφέροντος καθώς απεδείχθη ότι επηρεάζει την λειτουργία του οργανισμού από την εμβρυική ζωή, έως την τρίτη ηλικία. Πιο συγκεκριμένα, αποτελεί μια στεροειδική προ-ορμόνη, η οποία συμβάλλει στην φυσιολογική απορρόφηση και χρησιμοποίηση του ασβεστίου και του φωσφόρου, στην διατήρηση των φυσιολογικών επιπέδων ασβεστίου στο αίμα, στη στην διατήρηση της φυσιολογικής κατάστασης των οστών, των μυών και των δοντιών, στη κυτταρική διαίρεση και στην φυσιολογική λειτουργία του ανοσοποιητικού συστήματος *.
+Η βιταμίνη D του οργανισμού αποτελεί το άθροισμα της βιταμίνης D που συντίθεται στο δέρμα και της βιταμίνης D που λαμβάνεται από την τροφή. Εντούτοις και παρά το γεγονός ότι το σημαντικότερο ποσοστό της βιταμίνης συντίθεται ενδογενώς, ένα μεγάλο μέρος του πληθυσμού εμφανίζει ανεπάρκεια βιταμίνης D.
+Η Lamberts® διαθέτει μια ολοκληρωμένη γκάμα σκευασμάτων βιταμίνης D, προκειμένου να καλύπτει όσο το δυνατόν πιο εξατομικευμένα τις ανάγκες του οργανισμού. Σε όλα τα σκευάσματα βιταμίνης D της Lamberts® χρησιμοποιείται χοληκαλσιφερόλη (βιταμίνη D3), η οποία αποτελεί την ενεργό μορφή της βιταμίνης.
+Η χοληκαλσιφερόλη της Lamberts® είναι κλινικά ελεγμένη με εξαιρετική απορρόφηση και βιοδιαθεσιμότητα (1) .
+Το παρόν σκεύασμα παρέχει 2000iu βιταμίνης D3 (χοληκαλσιφερόλη) ανά ταμπλέτα και όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+(1) Makariou S, Lymperopoulos E, Challa A, Elisaf M. Association of vitamin d levels with risk factors and drugs for cardiovascular disease in adolescents and adults.</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη D (D3) 2000iu
+50μg
+Συστατικά: Έλαιο Ηλιόσπορου, Περίβλημα Κάψουλας (Πηκτωματοποιητές: Τροποποιημένο Άμυλο &amp; Καραγενάννη), Υγροποιητής: Γλυκερόλη), Βιταμίνη D3 (Χοληκαλσιφερόλη).</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30,60&amp;120 caps</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 73424/15.07.2020 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη D3</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
@@ -4883,7 +7505,47 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 400iu</t>
+          <t xml:space="preserve">Την τελευταία εικοσαετία, η βιταμίνη D έχει επανέλθει δυναμικά στο προσκήνιο του επιστημονικού ενδιαφέροντος καθώς απεδείχθη ότι επηρεάζει την λειτουργία του οργανισμού από την εμβρυική ζωή, έως την τρίτη ηλικία. Πιο συγκεκριμένα, αποτελεί μια στεροειδική προ-ορμόνη, η οποία συμβάλλει στην φυσιολογική απορρόφηση και χρησιμοποίηση του ασβεστίου και του φωσφόρου, στην διατήρηση των φυσιολογικών επιπέδων ασβεστίου στο αίμα, στη στην διατήρηση της φυσιολογικής κατάστασης των οστών, των μυών και των δοντιών, στη κυτταρική διαίρεση και στην φυσιολογική λειτουργία του ανοσοποιητικού συστήματος *.
+Η βιταμίνη D του οργανισμού αποτελεί το άθροισμα της βιταμίνης D που συντίθεται στο δέρμα και της βιταμίνης D που λαμβάνεται από την τροφή. Εντούτοις και παρά το γεγονός ότι το σημαντικότερο ποσοστό της βιταμίνης συντίθεται ενδογενώς, ένα μεγάλο μέρος του πληθυσμού εμφανίζει ανεπάρκεια βιταμίνης D.
+Η Lamberts® διαθέτει μια ολοκληρωμένη γκάμα σκευασμάτων βιταμίνης D, προκειμένου να καλύπτει όσο το δυνατόν πιο εξατομικευμένα τις ανάγκες του οργανισμού. Σε όλα τα σκευάσματα βιταμίνης D της Lamberts® χρησιμοποιείται χοληκαλσιφερόλη (βιταμίνη D3), η οποία αποτελεί την ενεργό μορφή της βιταμίνης.
+Η χοληκαλσιφερόλη της Lamberts® είναι κλινικά ελεγμένη με εξαιρετική απορρόφηση και βιοδιαθεσιμότητα (1) .
+Το παρόν σκεύασμα παρέχει 400iu βιταμίνης D3 (χοληκαλσιφερόλη) ανά ταμπλέτα και όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+(1) Makariou S, Lymperopoulos E, Challa A, Elisaf M. Association of vitamin d levels with risk factors and drugs for cardiovascular disease in adolescents and adults.</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Βιταμίνη D (ως Βιταμίνη D3)
+400iu (10μg)
+Συστατικά: Διογκωτικοί Παράγοντες (Φωσφορικό Διασβέστιο &amp; Κυτταρίνη), Βιταμίνη D3 (Χοληκαλσιφερόλη), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο).</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">120tabs</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 93179/05.12.2013 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη D3</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
@@ -4936,7 +7598,47 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Συνδυασμός υψηλής ισχύος Βιταμινών Κ2 &amp; D3 (2000iu)</t>
+          <t xml:space="preserve">Νεότερα επιστημονικά δεδομένα καταδεικνύουν την συνεργιστική δράση της βιταμίνης Κ (ιδιαιτέρως της βιταμίνης Κ2) και της βιταμίνης D στην υγεία του καρδιαγγειακού και του μυοσκελετικού συστήματος* και συνιστούν στους Επαγγελματίες της Υγείας παρακολούθηση τη λήψης και των δύο αυτών βιταμινών.
+Το σκεύασμα D3 και K2 της Lamberts® αποδίδει 2000 μονάδες (50μg) φυσικής και κλινικά ελεγμένης βιταμίνης D (ως χοληκαλσιφερόλη) καθώς και την εντυπωσιακή ποσότητα των 90μg (καθαρής και απαλλαγμένης από τα cis-ισομερή της) βιταμίνη Κ2, στη φυσική της μορφή (ως μενακινόνη/ΜΚ-7).
+H Κ2 της Lamberts® παρασκευάζεται από ρεβίθια μέσω μιας ειδικής διαδικασίας ζύμωσης. Το γεγονός αυτό διασφαλίζει ότι το σκεύασμά μας δεν περιέχει ως διατροφικά αλλεργιογόνα σόγια και υποπροϊόντα γάλακτος.
+Το Vitamin D3 2000iu &amp; K2 90 µg όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη D (D3)
+50μg (2000iu)
+Βιταμίνη K (Κ2)
+90μg
+Συστατικά: Ηλιέλαιο, Περίβλημα Κάψουλας (Γλυκερόλη, Τροποποιημένο Άμυλο, Πηκτωματοποιητής: Καραγεννάνη, Χρωστικές: Οξείδιο του Σιδήρου), Βιταμίνη Κ2 (Μενακινόνη-7 (ΜΚ-7)), Βιταμίνη D3 Χοληκαλσιφερόλη).</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες. Να μην λαμβάνεται από άτομα που βρίσκονται υπό αγωγή με κουμαρινικά αντιπηκτικά, εκτός εάν υπάρχει αντίθετη ιατρική σύσταση.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90caps</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 108838/14.10.2022 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη Κ2 &amp; συνδυασμοί με D3</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
@@ -4989,7 +7691,47 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 1000iu</t>
+          <t xml:space="preserve">Την τελευταία εικοσαετία, η βιταμίνη D έχει επανέλθει δυναμικά στο προσκήνιο του επιστημονικού ενδιαφέροντος καθώς απεδείχθη ότι επηρεάζει την λειτουργία του οργανισμού από την εμβρυική ζωή, έως την τρίτη ηλικία. Πιο συγκεκριμένα, αποτελεί μια στεροειδική προ-ορμόνη, η οποία συμβάλλει στην φυσιολογική απορρόφηση και χρησιμοποίηση του ασβεστίου και του φωσφόρου, στην διατήρηση των φυσιολογικών επιπέδων ασβεστίου στο αίμα, στη στην διατήρηση της φυσιολογικής κατάστασης των οστών, των μυών και των δοντιών, στη κυτταρική διαίρεση και στην φυσιολογική λειτουργία του ανοσοποιητικού συστήματος *.
+Η βιταμίνη D του οργανισμού αποτελεί το άθροισμα της βιταμίνης D που συντίθεται στο δέρμα και της βιταμίνης D που λαμβάνεται από την τροφή. Εντούτοις και παρά το γεγονός ότι το σημαντικότερο ποσοστό της βιταμίνης συντίθεται ενδογενώς, ένα μεγάλο μέρος του πληθυσμού εμφανίζει ανεπάρκεια βιταμίνης D.
+Η Lamberts® διαθέτει μια ολοκληρωμένη γκάμα σκευασμάτων βιταμίνης D, προκειμένου να καλύπτει όσο το δυνατόν πιο εξατομικευμένα τις ανάγκες του οργανισμού. Σε όλα τα σκευάσματα βιταμίνης D της Lamberts® χρησιμοποιείται χοληκαλσιφερόλη (βιταμίνη D3), η οποία αποτελεί την ενεργό μορφή της βιταμίνης.
+Η χοληκαλσιφερόλη της Lamberts® είναι κλινικά ελεγμένη με εξαιρετική απορρόφηση και βιοδιαθεσιμότητα (1) .
+Το παρόν σκεύασμα παρέχει 1000iu βιταμίνης D3 (χοληκαλσιφερόλη) ανά ταμπλέτα και όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+(1) Makariou S, Lymperopoulos E, Challa A, Elisaf M. Association of vitamin d levels with risk factors and drugs for cardiovascular disease in adolescents and adults.</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη D (ως Βιταμίνη D3)
+1000iu (25μg)
+Συστατικά: Ηλιέλαιο, Περίβλημα Κάψουλας (Βόειος Ζελατίνη, Γλυκερόλη), Βιταμίνη D3 (Xοληκαλσιφερόλη &amp;, Αντιοξειδωτικό: dl-a-Tοκοφερόλη).</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30&amp;120caps</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 18102/04.03.2013 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη D3</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
@@ -5009,7 +7751,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/vitamin-d3-1000iu-gummies-5055148410599.png</t>
+          <t xml:space="preserve">lamberts/vitamin-d-1000iu-5055148410599.png</t>
         </is>
       </c>
       <c r="Q97" t="inlineStr">
@@ -5047,7 +7789,47 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 1000iu</t>
+          <t xml:space="preserve">Την τελευταία εικοσαετία, η βιταμίνη D έχει επανέλθει δυναμικά στο προσκήνιο του επιστημονικού ενδιαφέροντος καθώς απεδείχθη ότι επηρεάζει την λειτουργία του οργανισμού από την εμβρυική ζωή, έως την τρίτη ηλικία. Πιο συγκεκριμένα, αποτελεί μια στεροειδική προ-ορμόνη, η οποία συμβάλλει στην φυσιολογική απορρόφηση και χρησιμοποίηση του ασβεστίου και του φωσφόρου, στην διατήρηση των φυσιολογικών επιπέδων ασβεστίου στο αίμα, στη στην διατήρηση της φυσιολογικής κατάστασης των οστών, των μυών και των δοντιών, στη κυτταρική διαίρεση και στην φυσιολογική λειτουργία του ανοσοποιητικού συστήματος *.
+Η βιταμίνη D του οργανισμού αποτελεί το άθροισμα της βιταμίνης D που συντίθεται στο δέρμα και της βιταμίνης D που λαμβάνεται από την τροφή. Εντούτοις και παρά το γεγονός ότι το σημαντικότερο ποσοστό της βιταμίνης συντίθεται ενδογενώς, ένα μεγάλο μέρος του πληθυσμού εμφανίζει ανεπάρκεια βιταμίνης D.
+Η Lamberts® διαθέτει μια ολοκληρωμένη γκάμα σκευασμάτων βιταμίνης D, προκειμένου να καλύπτει όσο το δυνατόν πιο εξατομικευμένα τις ανάγκες του οργανισμού. Σε όλα τα σκευάσματα βιταμίνης D της Lamberts® χρησιμοποιείται χοληκαλσιφερόλη (βιταμίνη D3), η οποία αποτελεί την ενεργό μορφή της βιταμίνης.
+Η χοληκαλσιφερόλη της Lamberts® είναι κλινικά ελεγμένη με εξαιρετική απορρόφηση και βιοδιαθεσιμότητα (1) .
+Το παρόν σκεύασμα παρέχει 1000iu βιταμίνης D3 (χοληκαλσιφερόλη) ανά ταμπλέτα και όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+(1) Makariou S, Lymperopoulos E, Challa A, Elisaf M. Association of vitamin d levels with risk factors and drugs for cardiovascular disease in adolescents and adults.</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη D (ως Βιταμίνη D3)
+1000iu (25μg)
+Συστατικά: Ηλιέλαιο, Περίβλημα Κάψουλας (Βόειος Ζελατίνη, Γλυκερόλη), Βιταμίνη D3 (Xοληκαλσιφερόλη &amp;, Αντιοξειδωτικό: dl-a-Tοκοφερόλη).</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30&amp;120caps</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 18102/04.03.2013 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη D3</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -5062,7 +7844,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/vitamin-d3-1000iu-gummies-5055148411480.png</t>
+          <t xml:space="preserve">lamberts/vitamin-d-1000iu-5055148411480.png</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr">
@@ -5100,7 +7882,47 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Συνδυασμός υψηλής ισχύος Βιταμινών Κ2 &amp; D3 (2000iu)</t>
+          <t xml:space="preserve">Νεότερα επιστημονικά δεδομένα καταδεικνύουν την συνεργιστική δράση της βιταμίνης Κ (ιδιαιτέρως της βιταμίνης Κ2) και της βιταμίνης D στην υγεία του καρδιαγγειακού και του μυοσκελετικού συστήματος* και συνιστούν στους Επαγγελματίες της Υγείας παρακολούθηση τη λήψης και των δύο αυτών βιταμινών.
+Το σκεύασμα D3 και K2 της Lamberts® αποδίδει 2000 μονάδες (50μg) φυσικής και κλινικά ελεγμένης βιταμίνης D (ως χοληκαλσιφερόλη) καθώς και την εντυπωσιακή ποσότητα των 90μg (καθαρής και απαλλαγμένης από τα cis-ισομερή της) βιταμίνη Κ2, στη φυσική της μορφή (ως μενακινόνη/ΜΚ-7).
+H Κ2 της Lamberts® παρασκευάζεται από ρεβίθια μέσω μιας ειδικής διαδικασίας ζύμωσης. Το γεγονός αυτό διασφαλίζει ότι το σκεύασμά μας δεν περιέχει ως διατροφικά αλλεργιογόνα σόγια και υποπροϊόντα γάλακτος.
+Το Vitamin D3 2000iu &amp; K2 90 µg όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη D (D3)
+50μg (2000iu)
+Βιταμίνη K (Κ2)
+90μg
+Συστατικά: Ηλιέλαιο, Περίβλημα Κάψουλας (Γλυκερόλη, Τροποποιημένο Άμυλο, Πηκτωματοποιητής: Καραγεννάνη, Χρωστικές: Οξείδιο του Σιδήρου), Βιταμίνη Κ2 (Μενακινόνη-7 (ΜΚ-7)), Βιταμίνη D3 Χοληκαλσιφερόλη).</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες. Να μην λαμβάνεται από άτομα που βρίσκονται υπό αγωγή με κουμαρινικά αντιπηκτικά, εκτός εάν υπάρχει αντίθετη ιατρική σύσταση.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90caps</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 108838/14.10.2022 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη Κ2 &amp; συνδυασμοί με D3</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">
@@ -5153,7 +7975,47 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 2000iu</t>
+          <t xml:space="preserve">Την τελευταία εικοσαετία, η βιταμίνη D έχει επανέλθει δυναμικά στο προσκήνιο του επιστημονικού ενδιαφέροντος καθώς απεδείχθη ότι επηρεάζει την λειτουργία του οργανισμού από την εμβρυική ζωή, έως την τρίτη ηλικία. Πιο συγκεκριμένα, αποτελεί μια στεροειδική προ-ορμόνη, η οποία συμβάλλει στην φυσιολογική απορρόφηση και χρησιμοποίηση του ασβεστίου και του φωσφόρου, στην διατήρηση των φυσιολογικών επιπέδων ασβεστίου στο αίμα, στη στην διατήρηση της φυσιολογικής κατάστασης των οστών, των μυών και των δοντιών, στη κυτταρική διαίρεση και στην φυσιολογική λειτουργία του ανοσοποιητικού συστήματος *.
+Η βιταμίνη D του οργανισμού αποτελεί το άθροισμα της βιταμίνης D που συντίθεται στο δέρμα και της βιταμίνης D που λαμβάνεται από την τροφή. Εντούτοις και παρά το γεγονός ότι το σημαντικότερο ποσοστό της βιταμίνης συντίθεται ενδογενώς, ένα μεγάλο μέρος του πληθυσμού εμφανίζει ανεπάρκεια βιταμίνης D.
+Η Lamberts® διαθέτει μια ολοκληρωμένη γκάμα σκευασμάτων βιταμίνης D, προκειμένου να καλύπτει όσο το δυνατόν πιο εξατομικευμένα τις ανάγκες του οργανισμού. Σε όλα τα σκευάσματα βιταμίνης D της Lamberts® χρησιμοποιείται χοληκαλσιφερόλη (βιταμίνη D3), η οποία αποτελεί την ενεργό μορφή της βιταμίνης.
+Η χοληκαλσιφερόλη της Lamberts® είναι κλινικά ελεγμένη με εξαιρετική απορρόφηση και βιοδιαθεσιμότητα (1) .
+Το παρόν σκεύασμα παρέχει 2000iu βιταμίνης D3 (χοληκαλσιφερόλη) ανά ταμπλέτα και όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+(1) Makariou S, Lymperopoulos E, Challa A, Elisaf M. Association of vitamin d levels with risk factors and drugs for cardiovascular disease in adolescents and adults.</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη D (D3) 2000iu
+50μg
+Συστατικά: Έλαιο Ηλιόσπορου, Περίβλημα Κάψουλας (Πηκτωματοποιητές: Τροποποιημένο Άμυλο &amp; Καραγενάννη), Υγροποιητής: Γλυκερόλη), Βιταμίνη D3 (Χοληκαλσιφερόλη).</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30,60&amp;120 caps</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 73424/15.07.2020 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη D3</t>
         </is>
       </c>
       <c r="M100" t="inlineStr">
@@ -5168,7 +8030,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/vitamin-d3-2000iu-k2-90-g-5055148413248.png</t>
+          <t xml:space="preserve">lamberts/vitamin-d-2000iu-5055148413248.png</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
@@ -5206,7 +8068,47 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 2000iu</t>
+          <t xml:space="preserve">Την τελευταία εικοσαετία, η βιταμίνη D έχει επανέλθει δυναμικά στο προσκήνιο του επιστημονικού ενδιαφέροντος καθώς απεδείχθη ότι επηρεάζει την λειτουργία του οργανισμού από την εμβρυική ζωή, έως την τρίτη ηλικία. Πιο συγκεκριμένα, αποτελεί μια στεροειδική προ-ορμόνη, η οποία συμβάλλει στην φυσιολογική απορρόφηση και χρησιμοποίηση του ασβεστίου και του φωσφόρου, στην διατήρηση των φυσιολογικών επιπέδων ασβεστίου στο αίμα, στη στην διατήρηση της φυσιολογικής κατάστασης των οστών, των μυών και των δοντιών, στη κυτταρική διαίρεση και στην φυσιολογική λειτουργία του ανοσοποιητικού συστήματος *.
+Η βιταμίνη D του οργανισμού αποτελεί το άθροισμα της βιταμίνης D που συντίθεται στο δέρμα και της βιταμίνης D που λαμβάνεται από την τροφή. Εντούτοις και παρά το γεγονός ότι το σημαντικότερο ποσοστό της βιταμίνης συντίθεται ενδογενώς, ένα μεγάλο μέρος του πληθυσμού εμφανίζει ανεπάρκεια βιταμίνης D.
+Η Lamberts® διαθέτει μια ολοκληρωμένη γκάμα σκευασμάτων βιταμίνης D, προκειμένου να καλύπτει όσο το δυνατόν πιο εξατομικευμένα τις ανάγκες του οργανισμού. Σε όλα τα σκευάσματα βιταμίνης D της Lamberts® χρησιμοποιείται χοληκαλσιφερόλη (βιταμίνη D3), η οποία αποτελεί την ενεργό μορφή της βιταμίνης.
+Η χοληκαλσιφερόλη της Lamberts® είναι κλινικά ελεγμένη με εξαιρετική απορρόφηση και βιοδιαθεσιμότητα (1) .
+Το παρόν σκεύασμα παρέχει 2000iu βιταμίνης D3 (χοληκαλσιφερόλη) ανά ταμπλέτα και όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+(1) Makariou S, Lymperopoulos E, Challa A, Elisaf M. Association of vitamin d levels with risk factors and drugs for cardiovascular disease in adolescents and adults.</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη D (D3) 2000iu
+50μg
+Συστατικά: Έλαιο Ηλιόσπορου, Περίβλημα Κάψουλας (Πηκτωματοποιητές: Τροποποιημένο Άμυλο &amp; Καραγενάννη), Υγροποιητής: Γλυκερόλη), Βιταμίνη D3 (Χοληκαλσιφερόλη).</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30,60&amp;120 caps</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 73424/15.07.2020 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη D3</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
@@ -5221,7 +8123,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/vitamin-d3-2000iu-k2-90-g-5055148413224.png</t>
+          <t xml:space="preserve">lamberts/vitamin-d-2000iu-5055148413224.png</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
@@ -5259,7 +8161,48 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 4000iu</t>
+          <t xml:space="preserve">Την τελευταία εικοσαετία, η βιταμίνη D έχει επανέλθει δυναμικά στο προσκήνιο του επιστημονικού ενδιαφέροντος καθώς απεδείχθη ότι επηρεάζει την λειτουργία του οργανισμού από την εμβρυική ζωή, έως την τρίτη ηλικία. Πιο συγκεκριμένα, αποτελεί μια στεροειδική προ-ορμόνη, η οποία συμβάλλει στην φυσιολογική απορρόφηση και χρησιμοποίηση του ασβεστίου και του φωσφόρου, στην διατήρηση των φυσιολογικών επιπέδων ασβεστίου στο αίμα, στη στην διατήρηση της φυσιολογικής κατάστασης των οστών, των μυών και των δοντιών, στη κυτταρική διαίρεση και στην φυσιολογική λειτουργία του ανοσοποιητικού συστήματος *.
+Η βιταμίνη D του οργανισμού αποτελεί το άθροισμα της βιταμίνης D που συντίθεται στο δέρμα και της βιταμίνης D που λαμβάνεται από την τροφή. Εντούτοις και παρά το γεγονός ότι το σημαντικότερο ποσοστό της βιταμίνης συντίθεται ενδογενώς, ένα μεγάλο μέρος του πληθυσμού εμφανίζει ανεπάρκεια βιταμίνης D.
+Η Lamberts® διαθέτει μια ολοκληρωμένη γκάμα σκευασμάτων βιταμίνης D, προκειμένου να καλύπτει όσο το δυνατόν πιο εξατομικευμένα τις ανάγκες του οργανισμού. Σε όλα τα σκευάσματα βιταμίνης D της Lamberts® χρησιμοποιείται χοληκαλσιφερόλη (βιταμίνη D3), η οποία αποτελεί την ενεργό μορφή της βιταμίνης.
+Η χοληκαλσιφερόλη της Lamberts® είναι κλινικά ελεγμένη με εξαιρετική απορρόφηση και βιοδιαθεσιμότητα (1) .
+Το παρόν σκεύασμα παρέχει 4000iu βιταμίνης D3 (χοληκαλσιφερόλη) ανά ταμπλέτα και όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+Η δόση των 4000iu συνιστάται να λαμβάνεται μετά από σύσταση Επαγγελματία υγείας.
+(1) Makariou S, Lymperopoulos E, Challa A, Elisaf M. Association of vitamin d levels with risk factors and drugs for cardiovascular disease in adolescents and adults.</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη D (ως Βιταμίνη D3)
+4000iu (100μg)
+Συστατικά: Έλαιο Ηλιόσπορου, Περίβλημα Κάψουλας (Τροποποιημένο Άμυλο, Γλυκερόλη, Πηκτωματοποιητής: Καραγενάννη), Βιταμίνη D3 (Χοληκαλσιφερόλη).</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30&amp;120caps</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 8569/16.01.2014 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη D3</t>
         </is>
       </c>
       <c r="M102" t="inlineStr">
@@ -5312,7 +8255,48 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνη D3 (Χοληκαλσιφερόλη) των 4000iu</t>
+          <t xml:space="preserve">Την τελευταία εικοσαετία, η βιταμίνη D έχει επανέλθει δυναμικά στο προσκήνιο του επιστημονικού ενδιαφέροντος καθώς απεδείχθη ότι επηρεάζει την λειτουργία του οργανισμού από την εμβρυική ζωή, έως την τρίτη ηλικία. Πιο συγκεκριμένα, αποτελεί μια στεροειδική προ-ορμόνη, η οποία συμβάλλει στην φυσιολογική απορρόφηση και χρησιμοποίηση του ασβεστίου και του φωσφόρου, στην διατήρηση των φυσιολογικών επιπέδων ασβεστίου στο αίμα, στη στην διατήρηση της φυσιολογικής κατάστασης των οστών, των μυών και των δοντιών, στη κυτταρική διαίρεση και στην φυσιολογική λειτουργία του ανοσοποιητικού συστήματος *.
+Η βιταμίνη D του οργανισμού αποτελεί το άθροισμα της βιταμίνης D που συντίθεται στο δέρμα και της βιταμίνης D που λαμβάνεται από την τροφή. Εντούτοις και παρά το γεγονός ότι το σημαντικότερο ποσοστό της βιταμίνης συντίθεται ενδογενώς, ένα μεγάλο μέρος του πληθυσμού εμφανίζει ανεπάρκεια βιταμίνης D.
+Η Lamberts® διαθέτει μια ολοκληρωμένη γκάμα σκευασμάτων βιταμίνης D, προκειμένου να καλύπτει όσο το δυνατόν πιο εξατομικευμένα τις ανάγκες του οργανισμού. Σε όλα τα σκευάσματα βιταμίνης D της Lamberts® χρησιμοποιείται χοληκαλσιφερόλη (βιταμίνη D3), η οποία αποτελεί την ενεργό μορφή της βιταμίνης.
+Η χοληκαλσιφερόλη της Lamberts® είναι κλινικά ελεγμένη με εξαιρετική απορρόφηση και βιοδιαθεσιμότητα (1) .
+Το παρόν σκεύασμα παρέχει 4000iu βιταμίνης D3 (χοληκαλσιφερόλη) ανά ταμπλέτα και όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+Η δόση των 4000iu συνιστάται να λαμβάνεται μετά από σύσταση Επαγγελματία υγείας.
+(1) Makariou S, Lymperopoulos E, Challa A, Elisaf M. Association of vitamin d levels with risk factors and drugs for cardiovascular disease in adolescents and adults.</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Βιταμίνη D (ως Βιταμίνη D3)
+4000iu (100μg)
+Συστατικά: Έλαιο Ηλιόσπορου, Περίβλημα Κάψουλας (Τροποποιημένο Άμυλο, Γλυκερόλη, Πηκτωματοποιητής: Καραγενάννη), Βιταμίνη D3 (Χοληκαλσιφερόλη).</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 κάψουλα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30&amp;120caps</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 8569/16.01.2014 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη D3</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
@@ -5370,7 +8354,47 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Φυσική Βιταμίνη D3 σε έξτρα παρθένο ελαιόλαδο</t>
+          <t xml:space="preserve">Η βιταμίνη D3 Drops είναι ένας εύκολος και βολικός τρόπος λήψης βιταμίνης D και μια εξαιρετική επιλογή για όλη την οικογένεια.
+Κάθε σταγόνα παρέχει 5μg (200iu) βιταμίνης D (ως βιταμίνης D3-χοληκαλσιφερόλης), και κάθε φιάλη περιέχει 600 σταγόνες. Ως εκ τούτου αποτελεί μια εξαιρετική επιλογή για άτομα στα οποία απαιτείται μακροχρόνια χορήγηση. Επιπροσθέτως αποτελεί μια αποτελεσματική εναλλακτική για άτομα που δεν μπορούν ή δεν επιθυμούν να καταπιούν κάψουλες.
+Η βιταμίνη D3 βρίσκεται διαλυμένη σε έξτρα παρθένο ελαιόλαδο, είναι άοσμη και άγευστη. Επιπλέον, έχει προστεθεί ένα μίγμα φυσικών τοκοφερολών (βιταμίνη Ε) για την προστασία της χοληκαλσιφερόλης από την οξείδωση.
+Τέλος το προϊόν δεν περιέχει κανένα έκδοχο και κανένα συντηρητικό, γεγονός ιδιαίτερα σημαντικό για περιπτώσεις χορήγησης σε μικρές ηλικίες.
+Όπως όλα τα σκευάσματα της Lamberts® , το Vitamin D3 Drops παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Ανά σταγόνα
+Βιταμίνη D (ως Βιταμίνη D3)
+200iu
+Συστατικά: Βιταμίνη D3 (Χολικαλσιφερόλη), Έξτρα Παρθένο Ελαιόλαδο, Μίγμα Φυσικών Τοκοφερολών.</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1-5 σταγόνες ημερησίως μετά το γεύμα. Ο αριθμός των προσλαμβανόμενων σταγόνων μπορεί να τροποποιηθεί κατόπιν συστάσεως του Ιατρού.
+ΑΝΑΚΙΝΕΙΣΤΕ ΚΑΛΑ ΠΡΙΝ ΑΠΟ ΤΗΝ ΧΡΗΣΗ. Αφαιρέστε το κάλυμμα και περιστρέψτε πλήρως το φιαλίδιο πάνω από ένα κουταλάκι. Σιγουρευτείτε ότι το φιαλίδιο είναι ανεστραμμένο και σε κάθετη θέση, ώστε να διασφαλίσετε την ακριβή δοσολογία. Να μην γίνεται υπέρβαση της συνιστώμενης ημερήσιας πρόσληψης.</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Καμία γνωστή για την προτεινόμενη δοσολογία.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20ml</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 67258/24.05.2019 | Κατηγορία lamberts.gr: Βιταμίνες › Βιταμίνη D3</t>
         </is>
       </c>
       <c r="M104" t="inlineStr">
@@ -5461,7 +8485,46 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Υψηλής ισχύος τιτλοδοτημένο εκχύλισμα Λυγαριάς</t>
+          <t xml:space="preserve">Η λυγαριά (Vitex agnus-castus) αποτελεί βότανο που ενδημεί στις μεσογειακές χώρες, με τις πρώτες αναφορές χρήσης του βοτάνου να ανευρίσκονται στην Αρχαία Ελλάδα.
+Οι φυτοχημικά δραστικές ουσίες ανευρίσκονται στα μούρα της λυγαριάς και περιλαμβάνουν ένα μεγάλο εύρος φυτοχημικά δραστικών ουσιών, συμπεριλαμβανομένων των φλαβονοειδών και των ιριδοειδών αλκαλοειδών.
+Οι ουσίες αυτές βοηθούν στη διατήρηση της ευεξίας κατά τη διάρκεια της εμμήνου ρήσεως, συμβάλλουν στη ορμονική ισορροπία κατά τη διάρκεια της κλιμακτηρίου και συμβάλλουν στην ανακούφιση των συμπτωμάτων της εμμηνόπαυσης*.
+To Vitex Agnus Castus της Lamberts® αποτελεί ένα υψηλής ισχύος τιτλοδοτημένο εκχύλισμα αποξηραμένων καρπών λυγαριάς, το οποίο παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP). Μπορεί να χρησιμοποιηθεί μαζί με άλλα συμπληρώματα διατροφής όπως η βιταμίνη Β6, η οποία συμβάλλει στη ρύθμιση της ορμονικής δραστηριότητας* και το έλαιο νυχτολούλουδου (Evening primrose oil), το οποίο συμβάλλει στη διατήρηση της ορμονικής ισορροπίας*.</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Λυγαριά (Vitex Agnus Castus)
+(ως 200 mg τιτλοδοτημένου εκχυλίσματος (5:1))
+1000mg
+Συστατικά: Διογκωτικοί Παράγοντες (Ανθρακικό Ασβέστιο, Κυτταρίνη), Εκχύλισμα Λυγαριάς (Vitex Agnus Castus), Επικάλυψη ταμπλέτας (Υδρόξυπροπυλο Μεθυλοκυτταρίνη, Σπιρουλίνα, Μήλο, Συμπυκνωμένο Κάρθαμο, Λεμόνι, Υδρόξυπροπυλο Κυτταρίνη), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο.</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1 ταμπλέτα ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60tabs</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 75027/16.11.2007 | Κατηγορία lamberts.gr: Βότανα › Βότανα για τη Γυναίκα</t>
         </is>
       </c>
       <c r="M106" t="inlineStr">

</xml_diff>

<commit_message>
Lamberts: approve renamed products as manual matches
Products the supplier still lists under their old names now map to their
renamed lamberts.gr pages: Glucosamine & Chondroitin → Glucosamine &
Phytodroitin, Ibisene → Artichoke 7425mg, Neuro-Logical PEA → Neuro-Logical
Plus, Magnesium 375 → Magnesium Citrate, Min Iron 14mg → Bio-Iron Complex,
Acidophilus Extra 10 (Milk Free) → Biome Balance Everyday, Aswagandha
Complex → Ashwagandha Advance, Osteoguard → Osteoguard Advance, MagAsorb
300mg 20tabs → MagAsorb Effervescent, Omega 3 Cats & Dog → High Potency
Omega 3s for Cats and Dogs. Multi Guard ADR has no page (null).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014FFaAMeHCcSLrUaq49VqHm
</commit_message>
<xml_diff>
--- a/lamberts-catalog.xlsx
+++ b/lamberts-catalog.xlsx
@@ -546,7 +546,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Για έλεγχο</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Για έλεγχο</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2605,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Glucosamine &amp; Chondroitin Complex 60tabs</t>
+          <t xml:space="preserve">Lamberts Glucosamine &amp; Phytodroitin™ Complex</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Συνδυασμός Θειικής Γλυκοζαμίνης &amp; Χονδροϊτίνης φυτικής προελεύσεως</t>
         </is>
       </c>
       <c r="C33">
@@ -2616,12 +2621,63 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Συμπλήρωμα διατροφής Lamberts — LAMBERTS Glucosamine &amp; Chondroitin Complex 60tabs</t>
+          <t xml:space="preserve">Το Glucosamine &amp; Phytodroitin™ Complex της Lamberts® αποτελεί σύμπλεγμα θειικής γλυκοζαμίνης και χονδροϊτίνης φυτικής προελεύσεως (GlucosaGreen® και φυτοδροϊτίνης , αντίστοιχα).
+Η GlucosaGreen® αποτελεί θειική γλυκοζαμίνη 100% φυτικής προελεύσεως που παρασκευάζεται από μη γενετικά τροποποιημένο καλαμπόκι μέσω μιας εξειδικευμένης και πρωτοποριακής διαδικασίας ζύμωσης. Η διαδικασία αυτή διασφαλίζει την παραγωγή θειικής γλυκοζαμίνης που είναι πανομοιότυπη και βιοισοδύναμη με τη θειική γλυκοζαμίνη των οστρακοειδών.
+Επιπροσθέτως:
+1.Δεν περιέχει κανένα διατροφικό αλλεργιογόνο και ως εκ τούτου είναι κατάλληλη για χρήση από άτομα με ιστορικό υπερευαισθησίας στα οστρακοειδή.
+2.Ο έλεγχος των πρώτων υλών και η ιχνηλασιμότητα στην όλη διαδικασία διασφαλίζει την απουσία περιβαλλοντικών ρύπων στο τελικό προϊόν και την δυνατότητα ασφαλούς μακροχρόνιας χορήγησης.
+3.Η όλη διαδικασία παραγωγής είναι φιλική ως προς το περιβάλλον καθώς απαιτεί μικρότερή κατανάλωση νερού και άλλων πρώτων υλών και συνοδεύεται από συντριπτικά μικρότερη παραγωγή υγρών και στερεών αποβλήτων.
+Η φυτοδροϊτίνη αποτελεί χονδροϊτίνη 100% φυτικής προελεύσεως με ταυτόσημη χημική δομή και βιοισοδυναμία με τη θειική χονδροϊτίνη που παρασκευάζεται από ζωικές πηγές. Η πηγή προελεύσεως της φυτοδροϊτίνης είναι τα βρώσιμα θαλάσσια φύκια, κυστοειδές φύκι (Fucus Vesicullosus) και μαρούλι της θάλασσας (Ulva lactuca).
+Η συνιστώμενη ημερήσια δόση των 3 ταμπλετών του Glucosamine &amp; Phytodroitin™ Complex της Lamberts® παρέχει 1400mg θειικής γλυκοζαμίνης , μια συγκέντρωση που έχει χρησιμοποιηθεί στην πλειονότητα των κλινικών μελετών και 300mg χονδροϊτίνης.
+Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά 3 ταμπλέτες
+GlucosaGreen®
+Θειϊκή Γλυκοζαμίνη 2KCl
+619mg
+Η οποία περιέχει Θειϊκή Γλυκοζαμίνη
+467mg
+Η οποία αποδίδει Βάση Γλυκοζαμίνης
+366mg
+Φυτοδροϊτίνη™
+(Ισοδύναμο Χονδροϊτίνης 100mg)
+110mg
+Συστατικά: GlucosaGreen® (Θειϊκή Γλυκοζαμίνη 2KCl), Τροποποιημένο Άμυλο, Φυτοδροϊτίνη™ (Fucus Vesiculosus, Ulva Lactura, Υαλουρονικό Νάτριο), Κυτταρίνη, Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Επικάλυψη Ταμπλέτας (Υδροξυπροπυλο Mεθυλοκυτταρίνη &amp; Γλυκερόλη).</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε από 1 έως 3 ταμπλέτες ημερησίως μετά το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60&amp;120tabs</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 2413/10.01.2023 | Κατηγορία lamberts.gr: Συμπληρώματα για Αρθρώσεις</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Διάφορα</t>
+          <t xml:space="preserve">Υγεία Οστών &amp; Αρθρώσεων</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2634,9 +2690,24 @@
           <t xml:space="preserve">5055148412333, 5054148408886, 5055148408886, 5054148412333, 5055150000000</t>
         </is>
       </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://lamberts.gr/wp-content/uploads/2025/01/8516-120-1.png</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://lamberts.gr/product/glucosamine-phytodroitin-complex/</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lamberts.gr</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Χωρίς σελίδα</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>
@@ -3273,7 +3344,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Artichoke High Strength 7425mg, 180tabs</t>
+          <t xml:space="preserve">Lamberts Artichoke 7425mg</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Υψηλής ισχύος τιτλοδοτημένο εκχύλισμα Αγκινάρας</t>
         </is>
       </c>
       <c r="C43">
@@ -3284,7 +3360,47 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Artichoke High Strength 7425mg, 180tabs - Συμπλήρωμα Διατροφής με Αγκινάρα για τη Διατήρηση της Υγείας του Ήπατος &amp; τη Σωστή Λειτουργία της Πέψης</t>
+          <t xml:space="preserve">Αν και η πρώτη ιστορικά καταγεγραμμένη αναφορά για την χρήση της αγκινάρας (Cynara scolymus) ως βοτάνου αφορούσε στην αντιμετώπιση της δυσπεψίας, σύγχρονες έρευνες ωστόσο, συνδέουν την αγκινάρα με τον μεταβολισμό των λιπιδίων, καθώς φαίνεται ότι υποστηρίζει τη διατήρηση των φυσιολογικών επιπέδων χοληστερόλης του αίματος*.
+Η φυτοχημικά δραστική ουσία που ευθύνεται για τις βιολογικές δράσεις της αγκινάρας , εντοπίζεται στα φύλλα του βοτάνου και ονομάζεται συναρίνη (cynarin). Η συγκέντρωση της συναρίνης χρησιμοποιείται ως δείκτης τιτλοδότησης και ισχύος του εκχυλίσματος των φύλλων της αγκινάρας.
+Το Artichoke της Lamberts® αποτελεί ένα υψηλής ισχύος τιτλοδοτημένο εκχύλισμα φύλλων αγκινάρας (Cynara scolymus) , το οποίο παρέχει εγγυημένα 16mg συναρίνης ανά ταμπλέτα. Όπως όλα τα σκευάσματα της Lamberts®, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ταμπλέτα
+Αγκινάρα ως 330 mg τιτλοδοτημένου εκχυλίσματος (22,5:1)
+7425mg
+Το οποίο αποδίδει:
+Cynarin
+16mg
+Συστατικά: Τιτλοδοτημένο Εκχύλισμα Αγκινάρας (Cynara scolymus), Διογκωτικοί Παράγοντες (Φωσφορικό Διασβέστιο &amp; Κυτταρίνη), Επικάλυψη Ταμπλέτας (Στιλβωτικοί Παράγοντες: Υδρόξυπροπυλο Μεθυλοκυτταρίνη, Ανθρακικό Ασβέστιο, Υδρόξυπροπυλο Κυτταρίνη, Στεατικό Οξύ &amp; Κυτταρίνη, Χρωστικές: Σπιρουλίνα, Μήλο, Κάρθαμο &amp; Λεμόνι), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου &amp; Στεατικό Μαγνήσιο).</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1-2 ταμπλέτες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Εναλλακτικά μπορείτε να λάβετε 2 ταμπλέτες μαζί, πριν από την κατανάλωση ενός λιπαρού γεύματος. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες και από παιδιά.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">180tabs</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 19615/01.03.2021 | Κατηγορία lamberts.gr: Βότανα › Βότανα Μεταβολισμού</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3309,17 +3425,17 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.pharm24.gr/lambertsartichoke-high-strength-7425mg-180tabs-p-53272.html</t>
+          <t xml:space="preserve">https://lamberts.gr/product/artichoke-7425mg/</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharm24.gr</t>
+          <t xml:space="preserve">lamberts.gr</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Χωρίς σελίδα</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>
@@ -3633,14 +3749,19 @@
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Για έλεγχο</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Magnesium 375 100% Nrv 180tabs</t>
+          <t xml:space="preserve">Lamberts Magnesium Citrate</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ζελεδάκια κιτρικού Μαγνησίου, υψηλής απορρόφησης</t>
         </is>
       </c>
       <c r="C49">
@@ -3651,12 +3772,61 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Magnesium 375 100% NRV 180tabs - Συμπλήρωμα Διατροφής Μαγνησίου για την Καλή Λειτουργία του Νευρικού &amp; Μυοσκελετικού Συστήματος</t>
+          <t xml:space="preserve">Με φυσική γεύση Φράουλα και Κεράσι
+Τα ζελεδάκια Magnesium Citrate της Lamberts® παρέχουν την εντυπωσιακή ποσότητα των 150mg στοιχειακού μαγνησίου ανά ζελεδάκι. Το άλας που χρησιμοποιείται στο παρόν σκεύασμα είναι το κιτρικό άλας μαγνησίου (Magnesium Citrate). Το κιτρικό άλας μαγνησίου διαθέτει αυξημένη διαλυτότητα και ως εκ τούτου χαρακτηρίζεται από αυξημένη απορρόφηση και βιοδιαθεσιμότητα.
+Όπως σε όλα τα σκευάσματα της σειράς gummies της Lamberts®, τα ζελεδάκια Magnesium Citrate:
+• Δεν περιέχουν ζάχαρη ή / και τεχνητά γλυκαντικά
+• Δεν περιέχουν ζελατίνη
+• Δεν περιέχουν τεχνητές γεύσεις και τεχνητές χρωστικές
+Ως γλυκαντική ουσία και ως υποκατάστατο ζελατίνης χρησιμοποιούνται φρούκτο-ολιγοσακχαρίτες (FOS) από ίνες ρίζας Κιχωρίου. Οι φρούκτο-ολιγοσακχαρίτες (FOS), αποτελούν μια φυσική μορφή ευδιάλυτων υδατανθράκων, που συναντώνται σε πολλά λαχανικά, όπως τα αντίδια και τα κρεμμύδια. Όταν λαμβάνονται από του στόματος απορροφώνται μόνο εν μέρει ,καθώς το μεγαλύτερο ποσοστό τους χρησιμοποιείται σαν θρεπτικό υπόστρωμα για την ανάπτυξη της φυσιολογικής βακτηριακής χλωρίδας του εντέρου (κυρίως τα γένη Bifidobacteria και Lactobacillus).
+Τα ζελεδάκια Magnesium Citrate της Lamberts® παρασκευάζονται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+Αριθ. Πρωτ. Γνωστοποίησης ΕΟΦ: 20175/19.02.2025</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ζελεδάκι
+Μαγνήσιο
+150mg
+Φρουκτο-ολιγοσακχαρίτες (FOS)
+956mg
+Συστατικά: Ίνες Ρίζας Κιχωρίου (Φρουκτο-ολιγοσακχαρίτες (FOS)), Κιτρικό Μαγνήσιο, Νερό, Ρυθμιστές Οξύτητας (Κιτρικό Οξύ &amp; Κιτρικό Νάτριο), Συμπύκνωμα Μαύρου Καρότου, Φυσικό Άρωμα Φράουλας &amp; Κερασιού, Στιλβωτικός Παράγοντας (Κηρός Καρναούμπα).</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ενήλικες μασήστε 1 έως 2 ζελεδάκια ημερησίως ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις:
+Κατανάλωση Μαγνησίου που υπερβαίνει τα 250mg, μπορεί να προκαλέσει
+ήπιες γαστρεντερικέ
+ς διαταραχές. Η μείωση της δόσης ή ο διαμερισμός της μέσα στην
+ημέρα, μπορεί να βοηθήσει.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40 gummies</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατηγορία lamberts.gr: Μέταλλα › Μαγνήσιο</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Διάφορα</t>
+          <t xml:space="preserve">Υγεία Οστών &amp; Αρθρώσεων</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3671,24 +3841,29 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.pharm24.gr/lamberts-magnesium-375-100-nrv-180tabs-p-40297.html</t>
+          <t xml:space="preserve">https://lamberts.gr/product/magnesium-citrate/</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharm24.gr</t>
+          <t xml:space="preserve">lamberts.gr</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Χωρίς σελίδα</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Magnesium 375 100% Nrv 60tabs</t>
+          <t xml:space="preserve">Lamberts Magnesium Citrate</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ζελεδάκια κιτρικού Μαγνησίου, υψηλής απορρόφησης</t>
         </is>
       </c>
       <c r="C50">
@@ -3699,12 +3874,61 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Magnesium 375 100% NRV 60tabs - Συμπλήρωμα Διατροφής Μαγνησίου για την Καλή Λειτουργία του Νευρικού &amp; Μυοσκελετικού Συστήματος</t>
+          <t xml:space="preserve">Με φυσική γεύση Φράουλα και Κεράσι
+Τα ζελεδάκια Magnesium Citrate της Lamberts® παρέχουν την εντυπωσιακή ποσότητα των 150mg στοιχειακού μαγνησίου ανά ζελεδάκι. Το άλας που χρησιμοποιείται στο παρόν σκεύασμα είναι το κιτρικό άλας μαγνησίου (Magnesium Citrate). Το κιτρικό άλας μαγνησίου διαθέτει αυξημένη διαλυτότητα και ως εκ τούτου χαρακτηρίζεται από αυξημένη απορρόφηση και βιοδιαθεσιμότητα.
+Όπως σε όλα τα σκευάσματα της σειράς gummies της Lamberts®, τα ζελεδάκια Magnesium Citrate:
+• Δεν περιέχουν ζάχαρη ή / και τεχνητά γλυκαντικά
+• Δεν περιέχουν ζελατίνη
+• Δεν περιέχουν τεχνητές γεύσεις και τεχνητές χρωστικές
+Ως γλυκαντική ουσία και ως υποκατάστατο ζελατίνης χρησιμοποιούνται φρούκτο-ολιγοσακχαρίτες (FOS) από ίνες ρίζας Κιχωρίου. Οι φρούκτο-ολιγοσακχαρίτες (FOS), αποτελούν μια φυσική μορφή ευδιάλυτων υδατανθράκων, που συναντώνται σε πολλά λαχανικά, όπως τα αντίδια και τα κρεμμύδια. Όταν λαμβάνονται από του στόματος απορροφώνται μόνο εν μέρει ,καθώς το μεγαλύτερο ποσοστό τους χρησιμοποιείται σαν θρεπτικό υπόστρωμα για την ανάπτυξη της φυσιολογικής βακτηριακής χλωρίδας του εντέρου (κυρίως τα γένη Bifidobacteria και Lactobacillus).
+Τα ζελεδάκια Magnesium Citrate της Lamberts® παρασκευάζονται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+Αριθ. Πρωτ. Γνωστοποίησης ΕΟΦ: 20175/19.02.2025</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά ζελεδάκι
+Μαγνήσιο
+150mg
+Φρουκτο-ολιγοσακχαρίτες (FOS)
+956mg
+Συστατικά: Ίνες Ρίζας Κιχωρίου (Φρουκτο-ολιγοσακχαρίτες (FOS)), Κιτρικό Μαγνήσιο, Νερό, Ρυθμιστές Οξύτητας (Κιτρικό Οξύ &amp; Κιτρικό Νάτριο), Συμπύκνωμα Μαύρου Καρότου, Φυσικό Άρωμα Φράουλας &amp; Κερασιού, Στιλβωτικός Παράγοντας (Κηρός Καρναούμπα).</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ενήλικες μασήστε 1 έως 2 ζελεδάκια ημερησίως ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις:
+Κατανάλωση Μαγνησίου που υπερβαίνει τα 250mg, μπορεί να προκαλέσει
+ήπιες γαστρεντερικέ
+ς διαταραχές. Η μείωση της δόσης ή ο διαμερισμός της μέσα στην
+ημέρα, μπορεί να βοηθήσει.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40 gummies</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατηγορία lamberts.gr: Μέταλλα › Μαγνήσιο</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Διάφορα</t>
+          <t xml:space="preserve">Υγεία Οστών &amp; Αρθρώσεων</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3719,17 +3943,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.pharm24.gr/lamberts-magnesium-375-100-nrv-60tabs-p-40861.html</t>
+          <t xml:space="preserve">https://lamberts.gr/product/magnesium-citrate/</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharm24.gr</t>
+          <t xml:space="preserve">lamberts.gr</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Χωρίς σελίδα</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>
@@ -3898,7 +4122,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Iron 14mg, 100tabs</t>
+          <t xml:space="preserve">Lamberts Bio-Iron Complex</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Σύμπλεγμα Δισγλικινικού Σιδήρου, Λυσίνης και Βιταμίνης Β12</t>
         </is>
       </c>
       <c r="C53">
@@ -3909,12 +4138,58 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Iron 14mg, 100tabs - Συμπλήρωμα Διατροφής Σιδήρου σε Κιτρική Μορφή Κατάλληλο για Άτομα με Γαστρεντερικές Διαταραχές Άμεσης Απορρόφησης</t>
+          <t xml:space="preserve">Το Vegan Iron Complex, αποτελεί μια ειδικά σχεδιασμένη φόρμουλα σιδήρου και βιταμίνης Β12 για χορτοφάγους και αποκλειστικά χορτοφάγους (vegans), καθώς σε αυτές τις πληθυσμιακές ομάδες η ανεπάρκεια σιδήρου και βιταμίνης Β12 είναι αρκετά συχνή λόγω των διατροφικών περιορισμών.
+Συγκεκριμένα, η ανεπάρκεια της βιταμίνης Β12 οφείλεται στο ότι ανευρίσκεται σχεδόν αποκλειστικά σε ζωικές πρωτεΐνες, ενώ η ανεπάρκεια σιδήρου οφείλεται στο ότι ο σίδηρος των τροφών φυτικής προσελεύσεως είναι μη αιμικός και απορροφάται σε μικρότερο βαθμό από τον αιμικό σίδηρο των τροφών ζωικής προσελεύσεως.
+Εκτός από υψηλά επίπεδα στοιχειακού σιδήρου και βιταμίνης Β12 το Vegan Iron Complex παρέχει πολύ υψηλά επίπεδα λυσίνης. Η λυσίνη αποτελεί αμινοξύ που βρίσκεται κυρίως στο κρέας και αυξάνει την απορρόφηση του σιδήρου (δρα ως επιταχυντής της απορρόφησης).
+O σίδηρος που χρησιμοποιείται στο Vegan Iron Complex είναι σε μορφή δισγλυκινικού σιδήρου, η οποία (μαζί με τον κιτρικό σίδηρο) είναι πολύ καλά ανεκτή από το γαστρεντερικό σύστημα.
+Όπως όλα τα σκευάσματα της Lamberts® , το Vegan Iron Complex παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά 2 ταμπλέτες
+Βιταμίνη Β12
+250μg
+Σίδηρος
+20mg
+Υδροχλωρική L-Λυσίνη
+1250mg
+η οποία αποδίδει:
+L-Λυσίνη
+1000mg
+Συστατικά: Υδροχλωρική L-Λυσίνη, Διογκωτικοί Παράγοντες (Φωσφορικό Διασβέστιο &amp; Κυτταρίνη), Σίδηρος (Δισγλυκινικός Σίδηρος) Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ &amp; Στεατικό Μαγνήσιο), Στιλβωτικοί Παράγοντες (Υδρόξυπροπυλο Μεθυλοκυτταρίνη, Γλυκερόλη), Βιταμίνη Β12 (Μεθυλοκοβαλαμίνη).</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 2 ταμπλέτες ημερησίως ή σύμφωνα με τις οδηγίες του γιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη. Για την κατάποση των ταμπλετών χρησιμοποιείστε νερό ή χυμό φρούτων. Να αποφεύγεται η λήψη των ταμπλετών με γάλα ή πρωτεϊνικά ροφήματα. Για καλύτερη απορρόφηση να καταπίνετε ολόκληρες τις ταμπλέτες, μισή έως μια ώρα προ φαγητού ή με άδειο στομάχι.</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Το προϊόν αυτό περιέχει σίδηρο, και η υπέρβαση της δοσολογίας μπορεί να είναι επιζήμια, ιδιαίτερα σε μικρά παιδιά. Να φυλάσσεται σε μέρος και θέση την οποία δεν βλέπουν και δεν προσεγγίζουν παιδιά. Πρόσληψη σιδήρου άνω των 20mg μπορεί να προκαλέσει ήπιες γαστρεντερικές διαταραχές σε ορισμένα άτομα. Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">120tabs</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 71774/17.06.2024 | Κατηγορία lamberts.gr: Μέταλλα › Σίδηρος</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Διάφορα</t>
+          <t xml:space="preserve">Μεταλλικά Στοιχεία</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3929,17 +4204,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.pharm24.gr/lamberts-iron-14mg-100tabs-p-14096.html</t>
+          <t xml:space="preserve">https://lamberts.gr/product/bio-iron-complex/</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t xml:space="preserve">pharm24.gr</t>
+          <t xml:space="preserve">lamberts.gr</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Χωρίς σελίδα</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>
@@ -4148,7 +4423,7 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Για έλεγχο</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>
@@ -4339,12 +4614,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts MultiGuard OsteoAdvance 50+</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Πλήρης κάλυψη γυναικών γυναικών &gt; 50 ετών</t>
+          <t xml:space="preserve">Lamberts Multi Guard Adr 120Tabs</t>
         </is>
       </c>
       <c r="C59">
@@ -4355,109 +4625,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Η Multi-Guard® Osteo Advance 50+ αποτελεί την πιο ολοκληρωμένη και υψηλής περιεκτικότητας πολυβιταμινούχο φόρμουλα που κυκλοφορεί στο Ηνωμένο Βασίλειο για γυναίκες άνω των 50 ετών.
-Ο σχεδιασμός της συγκεκριμένης φόρμουλας έχει ως κεντρικό άξονα την ομοιοστασία του οστικού μεταβολισμού. Για τον λόγο αυτό έχουν προστεθεί επαρκή επίπεδα βιταμίνης D που συμβάλλει στη φυσιολογική απορρόφηση / χρησιμοποίηση του ασβεστίου και υψηλά επίπεδα βιταμίνης Κ2 (ως μενακινόνη /ΜΚ7), ασβεστίου (500mg) και μαγνησίου (250mg) καθώς αυτά τα μικροθρεπτικά συστατικά συμβάλλουν στη διατήρηση της φυσιολογικής κατάστασης των οστών*.
-Οι υψηλές δόσεις ασβεστίου και μαγνησίου, οδήγησαν στην συνιστώμενη ημερήσια δόση των 3 ταμπλετών, ωστόσο καθιστούν περιττή την λήψη ξεχωριστών σκευασμάτων ασβεστίου και μαγνησίου και ως εκ τούτου διασφαλίζουν την ευκολότερη συμμόρφωση στις οδηγίες του Επαγγελματία της Υγείας. Επιπροσθέτως, η αναλογία ασβεστίου/μαγνησίου του Osteoguard® Advance είναι 2:1, γεγονός που ενισχύει περαιτέρω την απορρόφηση του ασβεστίου από τον εντερικό βλεννογόνο.
-Εκτός της βιταμίνης D και των υψηλών δόσεων ασβεστίου και μαγνησίου, η Multi-Guard® Osteo Advance 50+ παρέχει άλλα 23 μικροθρεπτικά συστατικά αποτελώντας μια ολοκληρωμένη επιλογή για γυναίκες άνω των 50 ετών. Μεταξύ αυτών παρέχει τις αντιοξειδωτικές βιταμίνες A,C,E, το σύνολο των βιταμινών Β και άριστα επίπεδα όλων των ιχνοστοιχείων.
-Τέλος, το Multi-Guard® Osteo Advance 50+ περιέχει λουτεΐνη και υψηλές ποσότητες φυσικών αντιοξειδωτικών. Η λουτεΐνη αποτελεί καροτενοειδές που βρίσκεται στα πράσινα λαχανικά και διαδραματίζει σημαντικό ρόλο στην υγεία του οφθαλμού. Σε κάθε ταμπλέτα Multi-Guard® Osteo Advance 50+ περιέχονται 2mg λουτεΐνης φυσικής προσελεύσεως.
-Τα φυσικά αντιοξειδωτικά που περιλαμβάνονται στο Multi-Guard® Osteo Advance 50+ προέρχονται από τιτλοδοτημένα εκχυλίσματα κουρκουμά (Curcuma longa) , δενδρολίβανου (Rosmarinus officinalis L.) και σπόρων κόκκινου σταφυλιού (Vitis vinifera). Και τα τρία βότανα συνοδεύονται από σημαντικό όγκο αναφορών στη σύγχρονη βιβλιογραφία σχετικά με τις βιολογικές τους δράσεις.
-To Multi-Guard® Osteo Advance 50+, όπως όλα τα σκευάσματα της Lamberts®, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Διατροφικές Πληροφορίες
-Ανά 3 ταμπλέτες
-Βιταμίνη A
-800µg
-Βιταμίνη D (D3)
-10μg
-Βιταμίνη Ε
-24mg α-TE
-Βιταμίνη Κ (Κ2)
-75μg
-Βιταμίνη C
-120mg
-Θειαμίνη (Β1)
-5mg
-Ριβοφλαβίνη (Β2)
-4mg
-Νιασίνη (Β3)
-16mg
-Βιταμίνη Β6
-10mg
-Φολικό Οξύ
-200μg
-Βιταμίνη Β12
-100µg
-Βιοτίνη
-150μg
-Παντοθενικό Οξύ (Β5)
-12mg
-Ασβέστιο
-500mg
-Μαγνήσιο
-250mg
-Σίδηρος
-7mg
-Ψευδάργυρος
-15mg
-Χαλκός
-1mg
-Μαγγάνιο
-0,45mg
-Σελήνιο
-110µg
-Χρώμιο
-200μg
-Ιώδιο
-150μg
-Διτρυγική Χολίνη
-5mg
-Ινοσιτόλη
-5mg
-PABA
-5mg
-Λουτεΐνη
-2mg
-Τιτλοδοτημένο εκχύλισμα κουρκουμά
-50mg
-Τιτλοδοτημένο εκχύλισμα δενδρολίβανου
-13mg
-Τιτλοδοτημένο εκχύλισμα σπόρων κόκκινου σταφυλιού
-50mg
-Συστατικά: Ανθρακικό Ασβέστιο, Ανθρακικό και Κιτρικό Μαγνήσιο, Κυτταρίνη, Ασκορβικό Οξύ, Επικάλυψη Ταμπλέτας (Υδρόξυπροπυλο Μεθυλοκυτταρίνη, Πολυδεξτρόζη, Ανθρακικό Ασβέστιο, Χρωστικές: Οξείδιο του Σιδήρου), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ και Στεατικό Μαγνήσιο), Dl-α Τοκοφερόλη, Εκχύλισμα Κουρκουμά (Curcuma longa), Εκχύλισμα Σπόρου Κόκκινου Σταφυλιού (Vitis vinifera), Κιτρικός Ψευδάργυρος, Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη), Μενακινόνη-7 (MΚ-7), Φουμαρικός Σίδηρος, Νικοτιναμίδιο, Παντοθενικό Ασβέστιο, Εκχύλισμα Δενδρολίβανου (Rosmarinus officinalis), Υδροχλωρική Πυριδοξίνη, Κυανοκοβαλαμίνη, Σύμπλεγμα Λουτεΐνης (Λουτεΐνη (Tagetes erecta) &amp; Αντιοξειδωτικά: Εκχύλισμα Δενδρολίβανου (Rosmarinus officinalis)), Οξεική Βιταμίνη Α, Γλυκονικός Χαλκός, Μονονιτρική Θειαμίνη, Χοληκαλσιφερόλη, Παρα Αμινο Βενζοϊκό Οξύ, Διτρυγική Χολίνη, Ινοσιτόλη, Ριβοφλαβίνη, Γλυκονικό Μαγγάνιο, Πικολινικό Χρώμιο, L-Σεληνομεθειονίνη &amp; Νατριούχος Σελενίτης, Φολικό οξύ, Ιωδιούχο Κάλιο, Βιοτίνη.</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Λαμβάνετε 3 ταμπλέτες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Προφυλάξεις: Μπορεί να προκληθεί κίτρινος χρωματισμός των ούρων. Αυτό είναι αβλαβές και υποδεικνύει ότι το σώμα αποβάλλει την περίσσια ποσότητα της βιταμίνης Β2 (riboflavin). Το προϊόν αυτό περιέχει σίδηρο, και η υπέρβαση της δοσολογίας μπορεί να είναι επιζήμια, ιδιαίτερα σε μικρά παιδιά. Φυλάξτε το σε σημείο ασφαλές από τα παιδιά. Δεν συνιστάται για εγκύους ή θηλάζουσες γυναίκες ή γυναίκες με πιθανότητα μελλοντικής εγκυμοσύνης, εκτός εάν υπάρχει σαφής σύσταση από θεράποντα γυναικολόγο. Να μην λαμβάνεται από άτομα που βρίσκονται υπό αγωγή με κουμαρινικά αντιπηκτικά, εκτός εάν υπάρχει αντίθετη ιατρική σύσταση. Δεν συνίσταται για άτομα κάτω των 18 ετών.
-Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">120tabs</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 89115/16.12.2015 | Κατηγορία lamberts.gr: Πολυβιταμίνες › Για τη γυναίκα</t>
+          <t xml:space="preserve">Συμπλήρωμα διατροφής Lamberts — LAMBERTS MULTI GUARD ADR 120TABS</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνες</t>
+          <t xml:space="preserve">Διάφορα</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -4475,31 +4648,16 @@
           <t xml:space="preserve">lamberts/multi-guard-hair-skin-nails-5055148412111.png</t>
         </is>
       </c>
-      <c r="Q59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://lamberts.gr/product/multiguard-osteoadvance-50/</t>
-        </is>
-      </c>
-      <c r="R59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">lamberts.gr</t>
-        </is>
-      </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Για έλεγχο</t>
+          <t xml:space="preserve">Χωρίς σελίδα</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts MultiGuard OsteoAdvance 50+</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Πλήρης κάλυψη γυναικών γυναικών &gt; 50 ετών</t>
+          <t xml:space="preserve">Lamberts Multi Guard Adr 60Tabs</t>
         </is>
       </c>
       <c r="C60">
@@ -4510,109 +4668,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Η Multi-Guard® Osteo Advance 50+ αποτελεί την πιο ολοκληρωμένη και υψηλής περιεκτικότητας πολυβιταμινούχο φόρμουλα που κυκλοφορεί στο Ηνωμένο Βασίλειο για γυναίκες άνω των 50 ετών.
-Ο σχεδιασμός της συγκεκριμένης φόρμουλας έχει ως κεντρικό άξονα την ομοιοστασία του οστικού μεταβολισμού. Για τον λόγο αυτό έχουν προστεθεί επαρκή επίπεδα βιταμίνης D που συμβάλλει στη φυσιολογική απορρόφηση / χρησιμοποίηση του ασβεστίου και υψηλά επίπεδα βιταμίνης Κ2 (ως μενακινόνη /ΜΚ7), ασβεστίου (500mg) και μαγνησίου (250mg) καθώς αυτά τα μικροθρεπτικά συστατικά συμβάλλουν στη διατήρηση της φυσιολογικής κατάστασης των οστών*.
-Οι υψηλές δόσεις ασβεστίου και μαγνησίου, οδήγησαν στην συνιστώμενη ημερήσια δόση των 3 ταμπλετών, ωστόσο καθιστούν περιττή την λήψη ξεχωριστών σκευασμάτων ασβεστίου και μαγνησίου και ως εκ τούτου διασφαλίζουν την ευκολότερη συμμόρφωση στις οδηγίες του Επαγγελματία της Υγείας. Επιπροσθέτως, η αναλογία ασβεστίου/μαγνησίου του Osteoguard® Advance είναι 2:1, γεγονός που ενισχύει περαιτέρω την απορρόφηση του ασβεστίου από τον εντερικό βλεννογόνο.
-Εκτός της βιταμίνης D και των υψηλών δόσεων ασβεστίου και μαγνησίου, η Multi-Guard® Osteo Advance 50+ παρέχει άλλα 23 μικροθρεπτικά συστατικά αποτελώντας μια ολοκληρωμένη επιλογή για γυναίκες άνω των 50 ετών. Μεταξύ αυτών παρέχει τις αντιοξειδωτικές βιταμίνες A,C,E, το σύνολο των βιταμινών Β και άριστα επίπεδα όλων των ιχνοστοιχείων.
-Τέλος, το Multi-Guard® Osteo Advance 50+ περιέχει λουτεΐνη και υψηλές ποσότητες φυσικών αντιοξειδωτικών. Η λουτεΐνη αποτελεί καροτενοειδές που βρίσκεται στα πράσινα λαχανικά και διαδραματίζει σημαντικό ρόλο στην υγεία του οφθαλμού. Σε κάθε ταμπλέτα Multi-Guard® Osteo Advance 50+ περιέχονται 2mg λουτεΐνης φυσικής προσελεύσεως.
-Τα φυσικά αντιοξειδωτικά που περιλαμβάνονται στο Multi-Guard® Osteo Advance 50+ προέρχονται από τιτλοδοτημένα εκχυλίσματα κουρκουμά (Curcuma longa) , δενδρολίβανου (Rosmarinus officinalis L.) και σπόρων κόκκινου σταφυλιού (Vitis vinifera). Και τα τρία βότανα συνοδεύονται από σημαντικό όγκο αναφορών στη σύγχρονη βιβλιογραφία σχετικά με τις βιολογικές τους δράσεις.
-To Multi-Guard® Osteo Advance 50+, όπως όλα τα σκευάσματα της Lamberts®, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Διατροφικές Πληροφορίες
-Ανά 3 ταμπλέτες
-Βιταμίνη A
-800µg
-Βιταμίνη D (D3)
-10μg
-Βιταμίνη Ε
-24mg α-TE
-Βιταμίνη Κ (Κ2)
-75μg
-Βιταμίνη C
-120mg
-Θειαμίνη (Β1)
-5mg
-Ριβοφλαβίνη (Β2)
-4mg
-Νιασίνη (Β3)
-16mg
-Βιταμίνη Β6
-10mg
-Φολικό Οξύ
-200μg
-Βιταμίνη Β12
-100µg
-Βιοτίνη
-150μg
-Παντοθενικό Οξύ (Β5)
-12mg
-Ασβέστιο
-500mg
-Μαγνήσιο
-250mg
-Σίδηρος
-7mg
-Ψευδάργυρος
-15mg
-Χαλκός
-1mg
-Μαγγάνιο
-0,45mg
-Σελήνιο
-110µg
-Χρώμιο
-200μg
-Ιώδιο
-150μg
-Διτρυγική Χολίνη
-5mg
-Ινοσιτόλη
-5mg
-PABA
-5mg
-Λουτεΐνη
-2mg
-Τιτλοδοτημένο εκχύλισμα κουρκουμά
-50mg
-Τιτλοδοτημένο εκχύλισμα δενδρολίβανου
-13mg
-Τιτλοδοτημένο εκχύλισμα σπόρων κόκκινου σταφυλιού
-50mg
-Συστατικά: Ανθρακικό Ασβέστιο, Ανθρακικό και Κιτρικό Μαγνήσιο, Κυτταρίνη, Ασκορβικό Οξύ, Επικάλυψη Ταμπλέτας (Υδρόξυπροπυλο Μεθυλοκυτταρίνη, Πολυδεξτρόζη, Ανθρακικό Ασβέστιο, Χρωστικές: Οξείδιο του Σιδήρου), Παράγοντες Αντισυσσωμάτωσης (Διοξείδιο του Πυριτίου, Στεατικό Οξύ και Στεατικό Μαγνήσιο), Dl-α Τοκοφερόλη, Εκχύλισμα Κουρκουμά (Curcuma longa), Εκχύλισμα Σπόρου Κόκκινου Σταφυλιού (Vitis vinifera), Κιτρικός Ψευδάργυρος, Υγροποιητής (Διασταυρούμενη Νατριούχος Σελλουλόζη), Μενακινόνη-7 (MΚ-7), Φουμαρικός Σίδηρος, Νικοτιναμίδιο, Παντοθενικό Ασβέστιο, Εκχύλισμα Δενδρολίβανου (Rosmarinus officinalis), Υδροχλωρική Πυριδοξίνη, Κυανοκοβαλαμίνη, Σύμπλεγμα Λουτεΐνης (Λουτεΐνη (Tagetes erecta) &amp; Αντιοξειδωτικά: Εκχύλισμα Δενδρολίβανου (Rosmarinus officinalis)), Οξεική Βιταμίνη Α, Γλυκονικός Χαλκός, Μονονιτρική Θειαμίνη, Χοληκαλσιφερόλη, Παρα Αμινο Βενζοϊκό Οξύ, Διτρυγική Χολίνη, Ινοσιτόλη, Ριβοφλαβίνη, Γλυκονικό Μαγγάνιο, Πικολινικό Χρώμιο, L-Σεληνομεθειονίνη &amp; Νατριούχος Σελενίτης, Φολικό οξύ, Ιωδιούχο Κάλιο, Βιοτίνη.</t>
-        </is>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Λαμβάνετε 3 ταμπλέτες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Προφυλάξεις: Μπορεί να προκληθεί κίτρινος χρωματισμός των ούρων. Αυτό είναι αβλαβές και υποδεικνύει ότι το σώμα αποβάλλει την περίσσια ποσότητα της βιταμίνης Β2 (riboflavin). Το προϊόν αυτό περιέχει σίδηρο, και η υπέρβαση της δοσολογίας μπορεί να είναι επιζήμια, ιδιαίτερα σε μικρά παιδιά. Φυλάξτε το σε σημείο ασφαλές από τα παιδιά. Δεν συνιστάται για εγκύους ή θηλάζουσες γυναίκες ή γυναίκες με πιθανότητα μελλοντικής εγκυμοσύνης, εκτός εάν υπάρχει σαφής σύσταση από θεράποντα γυναικολόγο. Να μην λαμβάνεται από άτομα που βρίσκονται υπό αγωγή με κουμαρινικά αντιπηκτικά, εκτός εάν υπάρχει αντίθετη ιατρική σύσταση. Δεν συνίσταται για άτομα κάτω των 18 ετών.
-Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">120tabs</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 89115/16.12.2015 | Κατηγορία lamberts.gr: Πολυβιταμίνες › Για τη γυναίκα</t>
+          <t xml:space="preserve">Συμπλήρωμα διατροφής Lamberts — LAMBERTS MULTI GUARD ADR 60TABS</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Βιταμίνες</t>
+          <t xml:space="preserve">Διάφορα</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -4625,19 +4686,9 @@
           <t xml:space="preserve">lamberts/multi-guard-hair-skin-nails-5055148412708.png</t>
         </is>
       </c>
-      <c r="Q60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://lamberts.gr/product/multiguard-osteoadvance-50/</t>
-        </is>
-      </c>
-      <c r="R60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">lamberts.gr</t>
-        </is>
-      </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Για έλεγχο</t>
+          <t xml:space="preserve">Χωρίς σελίδα</t>
         </is>
       </c>
     </row>
@@ -4972,7 +5023,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Neuro-Logical Pea (B1, B6 &amp; B12) 60Caps</t>
+          <t xml:space="preserve">Lamberts Neuro-Logical Plus</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Παλμιτοϋλαιθανολαμίδιο υψηλής ισχύος με Β1, Β6 &amp; Β12</t>
         </is>
       </c>
       <c r="C65">
@@ -4983,7 +5039,52 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Συμπλήρωμα διατροφής Lamberts — LAMBERTS NEURO-LOGICAL PEA (B1, B6 &amp; B12) 60CAPS</t>
+          <t xml:space="preserve">Το Neuro-Logical PLUS της Lamberts® αποτελεί μια ειδικά σχεδιασμένη φόρμουλα κλινικής διατροφής, η οποία παρέχει 400mg παλμιτοϋλαιθανολαμιδίου ανά κάψουλα, σε συνδυασμό με βιταμίνες Β1,Β6 και Β12, οι οποίες συμβάλλουν στη φυσιολογική λειτουργία του νευρικού συστήματος και στη φυσιολογική ψυχολογική λειτουργία*.
+Το παλμιτοϋλαιθανολαμίδιο (PEA) αποτελεί ένα ενδογενές λιπίδιο, δηλαδή ένα λιπίδιο που παράγεται φυσιολογικά στον οργανισμό. Η παραγωγή του γίνεται από το σύνολο των κυττάρων του οργανισμού και αυξάνεται σημαντικά σε περιπτώσεις κυτταρικής βλάβης, φλεγμονής και πόνου.
+Η συμμετοχή του παλμιτοϋλαιθανολαμιδίου στη ρύθμιση της κυτταρικής ομοιοστασίας, το έθεσε στο επίκεντρο σημαντικής και αξιόλογης έρευνας την τελευταία 15ετία. Μάλιστα, καθώς διαθέτει δράση παρόμοια των ενδοκανναβινοειδών, αρκετές μελέτες περιγράφουν το παλμιτοϋλαιθανολαμίδιο ως μια «ασφαλή εναλλακτική» της κανναβιδιόλης (CBD).
+Το παλμιτοϋλαιθανολαμίδιο που χρησιμοποιείται στην παρασκευή των Neuro-Logical PLUS αποτελεί μια πατενταρισμένη, υψηλής ποιότητας, μικρο-ιονισμένη μορφή (OptiPEA®). Η μικρο-ιονισμένη μορφή διασφαλίζει πολύ υψηλή απορρόφηση και είναι πανομοιότυπη με αυτή που έχει χρησιμοποιηθεί στις δημοσιευμένες κλινικές μελέτες.
+Το Neuro-Logical PLUS , όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζονται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Διατροφικές πληροφορίες
+Aνά κάψουλα
+Παλμιτοϋλαιθανολαμίδη (PEA)
+400mg
+Θειαμίνη (Βιταμίνη Β1)
+4,4mg
+Βιταμίνη Β6
+2,8mg
+Βιταμίνη Β12
+50μg
+Συστατικά: OptiPEA® (Παλμιτοϋλαιθανολαμίδη), Περίβλημα Κάψουλας Υδροξυπρόπυλο Μεθυλοκυτταρίνη), Διογκωτικός Παράγοντας (Κυτταρίνη), Παράγοντες Αντισυσσωμάτωσης (Στεατικό Μαγνήσιο), Υδροχλωρική Θειαμίνη, Βιταμίνη Β6 (Υδροχλωρική Πυριδοξίνη), Βιταμίνη Β12 (Κυανοκοβαλαμίνη).</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Λαμβάνετε 1- 2 κάψουλες ημερησίως με το γεύμα ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Προφυλάξεις: Να μην λαμβάνεται από έγκυες ή θηλάζουσες γυναίκες.
+Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60caps</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Αρ. Γνωστ. ΕΟΦ: 90010/30.08.2023 | Κατηγορία lamberts.gr: Ειδικά Διατροφικά Συμπληρώματα › Παλμιτοϋλαιθανολαμίδιο</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -5001,21 +5102,31 @@
           <t xml:space="preserve">lamberts/neuro-logical-plus-5055148413644.png</t>
         </is>
       </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://lamberts.gr/product/neuro-logical-plus/</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lamberts.gr</t>
+        </is>
+      </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Χωρίς σελίδα</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lamberts Vegan Omega 3 Oil</t>
+          <t xml:space="preserve">Lamberts High Potency Omega 3s for Cats and Dogs</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Έλαιο EPA &amp; DHA από άλγη ελεγχόμενης καλλιέργειας</t>
+          <t xml:space="preserve">Βοηθάει στη διατήρηση υγιούς τριχώματος</t>
         </is>
       </c>
       <c r="C66">
@@ -5026,56 +5137,55 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Το Vegan Omega 3 Oil αποτελεί συμπλήρωμα διατροφής σε μορφή ελαίου από την άλγη Schizochytrium sp. .Το Vegan Omega 3 Oil παρέχει 100mg EPA και 500mg DHA ανά 5ml ελαίου, μια ποσότητα που συμβάλλει στην φυσιολογική λειτουργία της καρδιάς και στη διατήρηση της φυσιολογικής λειτουργίας του εγκεφάλου και της φυσιολογικής όρασης*.
-Η καλλιέργεια της άλγης που χρησιμοποιούμε για την παρασκευή της συγκεκριμένης σειράς, γίνεται σε ελεγχόμενο περιβάλλον, διασφαλίζοντας την απουσία περιβαλλοντικών επιμολύνσεων στο παραγόμενο έλαιο.
-Το έλαιο του Vegan Omega 3 Oil:
-περιέχει τα Ω3 λιπαρά οξέα στην τριγλυκεριδική μορφή τους
-προστατεύεται από την οξείδωση με την προσθήκη φυσικών αντιοξειδωτικών (τοκοφερόλες και εκχύλισμα δενδρολίβανου)
-περιέχει μηδενικούς περιβαλλοντικούς ρύπους, καθώς η καλλιέργεια της άλγης για την παραγωγή του ελαίου γίνεται σε ελεγχόμενο περιβάλλον.
-Το παρόν συμπλήρωμα στοχεύει στην κάλυψη συγκεκριμένων πληθυσμιακών ομάδων όπως οι χορτοφάγοι (Vegetarians) και οι αποκλειστικά χορτοφάγοι (Vegans), οι οποίες διατρέχουν αυξημένο κίνδυνο διατροφικής έλλειψης Ω3 λιπαρών οξέων, λόγω διατροφικών περιορισμών.
-Εκτός των χορτοφάγων και των αποκλειστικά χορτοφάγων , το παρόν συμπλήρωμα μπορεί να χρησιμοποιηθεί και από άτομα με αλλεργία στο ψάρι, τα οποία διατρέχουν αυξημένο κίνδυνο διατροφικής ανεπάρκειας του EPA και του DHA.
-Όπως όλα τα σκευάσματα της Lamberts® , παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της Φαρμακευτικής GMP (Pharmaceutical GMP).
-Αρ. Πρ. Γνωστ. ΕΟΦ: 133292/12.11.2024</t>
+          <t xml:space="preserve">Το συγκεκριμένο σκεύασμα Ωμέγα 3 λιπαρών οξέων διασφαλίζει ότι το κατοικίδιό σας λαμβάνει την αναγκαία ποσότητα EPA και DHA. Τα δύο αυτά απαραίτητα λιπαρά οξέα λείπουν συχνά από τις τροφές για τα κατοικίδια ζώα, εξαιτίας τόσο του κόστους παρασκευής τους, όσο και της δυσκολίας προσθήκης τους στην ξηρά τροφή (τείνουν να ταγγίζουν όταν εκτίθενται στον αέρα).
+Το High Potency Omega 3s for Cats and Dogs της Lamberts®, αποτελεί ένα υψηλής Ισχύος σκεύασμα Ω3 λιπαρών Οξέων για σκύλους, το οποίο διασφαλίζει την επαρκή πρόσληψη των EPA &amp; DHA Λιπαρών Οξέων.
+Οι κάψουλες μπορούν να προστεθούν στο φαγητό του κατοικίδιου, ενώ μπορεί να συγχορηγηθεί με το σκεύασμα μασώμενης γλυκοζαμίνης για την διατήρηση της υγείας των αρθρώσεων.
+Το High Potency Omega 3s for Cats and Dogs της Lamberts®, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+Οι κάψουλες μπορούν να προστεθούν στο φαγητό του κατοικίδιου, ενώ μπορεί να συγχορηγηθεί με το σκεύασμα μασώμενης γλυκοζαμίνης για την διατήρηση της υγείας των αρθρώσεων.
+Το High Potency Omega 3s for Cats and Dogs της Lamberts®, παρασκευάζεται εντός του Ηνωμένου Βασιλείου σύμφωνα με τα αυστηρά πρότυπα της φαρμακευτικής GMP (Pharmaceutical GMP).
+Τα συμπληρώματα διατροφής για κατοικίδια ζώα υπάγονται στην αρμοδιότητα της Διεύθυνσης Αγροτικής Οικονομίας και Κτηνιατρικής και του Υπουργείου Αγροτικής Ανάπτυξης και Τροφίμων</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Κατάλληλο για χορτοφάγους · Vegan · Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
+          <t xml:space="preserve">Χωρίς γλουτένη · Χωρίς γαλακτοκομικά</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
           <t xml:space="preserve">Διατροφικές πληροφορίες
-Aνά 5ml
-Έλαιο Θαλάσσιας Άλγης
-4885mg
-το οποίο παρέχει:
-EPA
-100mg
-DHA
-500mg
-Συστατικά: Έλαιο Θαλάσσιας Άλγης (έλαιο πλούσιο σε DHA &amp; EPA από την μικροάλγη Schizochytrium sp.), Γεύση Λεμονιού, Αντιοξειδωτικά (Μίγμα Φυσικών Τοκοφερολών &amp; Εκχύλισμα Δενδρολίβανου).</t>
+Aνά κάψουλα
+Ιχθυέλαιο το οποίο περιέχει:
+Eicosapenaenoic Acid (EPA)
+99mg
+Docosahexaenoic Acid (DHA)
+66mg
+Σύνθεση: Ιχθυέλαιο, Περίβλημα Κάψουλας (Ζελατίνη, Γλυκερίνη).</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Το προϊόν συνιστάται μόνο για ενήλικες. Λαμβάνετε 5ml (1 κουταλάκι του γλυκού) ημερησίως ή σύμφωνα με την σύσταση του ιατρού ή του φαρμακοποιού σας. Μην υπερβαίνετε την προτεινόμενη ημερήσια πρόσληψη.</t>
+          <t xml:space="preserve">ΗΜΕΡΗΣΙΑ ΔΟΣΗ ΓΙΑ ΣΚΥΛΟΥΣ ΚΑΙ ΓΑΤΕΣ
+Γάτες 1 κάψουλα
+Μικρού Μεγέθους Σκύλοι (0-10 κιλά) 1 κάψουλα
+Μεσαίου Μεγέθους Σκύλοι (10-25 κιλά) 2 κάψουλες
+Μεγάλοι Σκύλοι 2 κάψουλες</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Προφυλάξεις: Έγκυες ή θηλάζουσες γυναίκες συνιστάται να λαμβάνουν 1 κάψουλα ημερησίως. Να μην λαμβάνεται από άτομα κάτω των 18 ετών.
-Αλλεργίες: ΤΟ ΣΥΓΚΕΚΡΙΜΕΝΟ ΣΚΕΥΑΣΜΑ ΔΕΝ ΠΕΡΙΕΧΕΙ: γλουτένη, αλλεργιογόνα σίτου, κριθάρι, σόγια, αυγά, γάλα (και παράγωγα γάλακτος), λακτόζη, ξηρούς καρπούς, ψάρι, οστρακοειδή και θειώδη.</t>
+          <t xml:space="preserve">Προφυλάξεις: Μόνο για χρήση σε ζώα. Αυτό το προϊόν προορίζεται αποκλειστικά για διακεκομμένη ή συμπληρωματική σίτιση. Πάντα να συμβουλεύεστε τον κτηνίατρό σας πριν κάνετε αλλαγές στη διατροφή του κατοικιδίου σας.
+Αλλεργίες: Περιέχει ψάρι. Το συστατικό Μαγιά περιέχει γλουτένη.</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t xml:space="preserve">150ml υγρό</t>
+          <t xml:space="preserve">120 caps</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Κατηγορία lamberts.gr: Ω - Λιπαρά Οξέα › Ω-3 Λιπαρά οξέα φυτικής προελεύσεως</t>
+          <t xml:space="preserve">Κατηγορία lamberts.gr: Σειρά Pet</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -5095,7 +5205,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/product/vegan-omega-3-oil/</t>
+          <t xml:space="preserve">https://lamberts.gr/product/high-potency-omega-3s-for-cats-and-dogs/</t>
         </is>
       </c>
       <c r="R66" t="inlineStr">
@@ -5105,7 +5215,7 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Για έλεγχο</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5541,7 @@
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Για έλεγχο</t>
+          <t xml:space="preserve">Χειροκίνητο</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lamberts: images for manual matches
</commit_message>
<xml_diff>
--- a/lamberts-catalog.xlsx
+++ b/lamberts-catalog.xlsx
@@ -2692,7 +2692,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://lamberts.gr/wp-content/uploads/2025/01/8516-120-1.png</t>
+          <t xml:space="preserve">lamberts/glucosamine-phytodroitin-complex-5055148414139.png</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -3420,7 +3420,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/artichoke-high-strength-7425mg-180tabs-pharm24-gr-5055148413743.jpg</t>
+          <t xml:space="preserve">lamberts/artichoke-7425mg-5055148413743.png</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/magnesium-375-100-nrv-180tabs-pharm24-gr-5055148411428.jpg</t>
+          <t xml:space="preserve">lamberts/magnesium-citrate-5055148411428.png</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/magnesium-375-100-nrv-60tabs-pharm24-gr-5055148412876.jpg</t>
+          <t xml:space="preserve">lamberts/magnesium-citrate-5055148412876.png</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t xml:space="preserve">lamberts/iron-14mg-100tabs-pharm24-gr-5055148401931.jpg</t>
+          <t xml:space="preserve">lamberts/bio-iron-complex-5055148401931.png</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">

</xml_diff>